<commit_message>
Speed up reports and add EXPREZ Can freshness row
</commit_message>
<xml_diff>
--- a/templates/template_general.xlsx
+++ b/templates/template_general.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Bot\KB_Market_Survey_Telegram_V33_14_KHMER_SUMMARY_RENDER_FIXED\backend\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Bot\Market_Survey\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81E86045-28BA-43AA-BC3E-09ECCAC3319A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9430C19B-5D2F-4DDF-AA65-AFDC11DAFEFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="94">
   <si>
     <t>Market Improvement Report</t>
   </si>
@@ -365,7 +365,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -419,11 +419,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -446,7 +459,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
@@ -455,32 +468,41 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -759,7 +781,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AA49"/>
+  <dimension ref="A1:AA50"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -785,7 +807,7 @@
       <c r="D1" s="7"/>
     </row>
     <row r="2" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="15" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="9"/>
@@ -816,7 +838,7 @@
       <c r="AA2" s="9"/>
     </row>
     <row r="3" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="16" t="s">
         <v>1</v>
       </c>
       <c r="B3" s="9"/>
@@ -847,18 +869,18 @@
       <c r="AA3" s="9"/>
     </row>
     <row r="4" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A4" s="17" t="s">
+      <c r="A4" s="13" t="s">
         <v>2</v>
       </c>
       <c r="B4" s="12"/>
-      <c r="C4" s="17" t="s">
+      <c r="C4" s="13" t="s">
         <v>3</v>
       </c>
       <c r="D4" s="11"/>
       <c r="E4" s="11"/>
       <c r="F4" s="11"/>
       <c r="G4" s="12"/>
-      <c r="H4" s="17" t="s">
+      <c r="H4" s="13" t="s">
         <v>4</v>
       </c>
       <c r="I4" s="11"/>
@@ -875,7 +897,7 @@
       <c r="T4" s="11"/>
       <c r="U4" s="11"/>
       <c r="V4" s="12"/>
-      <c r="W4" s="17" t="s">
+      <c r="W4" s="13" t="s">
         <v>5</v>
       </c>
       <c r="X4" s="11"/>
@@ -884,7 +906,7 @@
       <c r="AA4" s="12"/>
     </row>
     <row r="5" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="14" t="s">
+      <c r="A5" s="22" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="11"/>
@@ -921,42 +943,42 @@
       <c r="B6" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="18" t="s">
+      <c r="C6" s="20" t="s">
         <v>9</v>
       </c>
       <c r="D6" s="11"/>
       <c r="E6" s="11"/>
       <c r="F6" s="11"/>
       <c r="G6" s="12"/>
-      <c r="H6" s="15" t="s">
+      <c r="H6" s="14" t="s">
         <v>10</v>
       </c>
       <c r="I6" s="11"/>
       <c r="J6" s="11"/>
       <c r="K6" s="12"/>
-      <c r="L6" s="15" t="s">
+      <c r="L6" s="14" t="s">
         <v>11</v>
       </c>
       <c r="M6" s="11"/>
       <c r="N6" s="11"/>
       <c r="O6" s="12"/>
-      <c r="P6" s="15" t="s">
+      <c r="P6" s="14" t="s">
         <v>12</v>
       </c>
       <c r="Q6" s="11"/>
       <c r="R6" s="11"/>
       <c r="S6" s="12"/>
-      <c r="T6" s="15" t="s">
+      <c r="T6" s="14" t="s">
         <v>13</v>
       </c>
       <c r="U6" s="11"/>
       <c r="V6" s="12"/>
-      <c r="W6" s="18" t="s">
+      <c r="W6" s="20" t="s">
         <v>14</v>
       </c>
       <c r="X6" s="11"/>
       <c r="Y6" s="12"/>
-      <c r="Z6" s="18" t="s">
+      <c r="Z6" s="20" t="s">
         <v>15</v>
       </c>
       <c r="AA6" s="12"/>
@@ -1324,7 +1346,7 @@
       <c r="Z17" s="10"/>
       <c r="AA17" s="12"/>
     </row>
-    <row r="18" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:27" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A18" s="3">
         <v>12</v>
       </c>
@@ -1357,78 +1379,78 @@
       <c r="Z18" s="10"/>
       <c r="AA18" s="12"/>
     </row>
-    <row r="19" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:27" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A19" s="3">
         <v>13</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="C19" s="10"/>
-      <c r="D19" s="11"/>
-      <c r="E19" s="11"/>
-      <c r="F19" s="11"/>
-      <c r="G19" s="12"/>
-      <c r="H19" s="10"/>
-      <c r="I19" s="11"/>
-      <c r="J19" s="11"/>
-      <c r="K19" s="12"/>
-      <c r="L19" s="10"/>
-      <c r="M19" s="11"/>
-      <c r="N19" s="11"/>
-      <c r="O19" s="12"/>
-      <c r="P19" s="10"/>
-      <c r="Q19" s="11"/>
-      <c r="R19" s="11"/>
-      <c r="S19" s="12"/>
-      <c r="T19" s="10"/>
-      <c r="U19" s="11"/>
-      <c r="V19" s="12"/>
-      <c r="W19" s="10"/>
-      <c r="X19" s="11"/>
-      <c r="Y19" s="12"/>
-      <c r="Z19" s="10"/>
-      <c r="AA19" s="12"/>
-    </row>
-    <row r="20" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="C19" s="23"/>
+      <c r="D19" s="24"/>
+      <c r="E19" s="24"/>
+      <c r="F19" s="24"/>
+      <c r="G19" s="25"/>
+      <c r="H19" s="23"/>
+      <c r="I19" s="24"/>
+      <c r="J19" s="24"/>
+      <c r="K19" s="25"/>
+      <c r="L19" s="23"/>
+      <c r="M19" s="24"/>
+      <c r="N19" s="24"/>
+      <c r="O19" s="25"/>
+      <c r="P19" s="23"/>
+      <c r="Q19" s="24"/>
+      <c r="R19" s="24"/>
+      <c r="S19" s="25"/>
+      <c r="T19" s="23"/>
+      <c r="U19" s="24"/>
+      <c r="V19" s="25"/>
+      <c r="W19" s="23"/>
+      <c r="X19" s="24"/>
+      <c r="Y19" s="25"/>
+      <c r="Z19" s="23"/>
+      <c r="AA19" s="25"/>
+    </row>
+    <row r="20" spans="1:27" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A20" s="3">
         <v>14</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C20" s="10"/>
-      <c r="D20" s="11"/>
-      <c r="E20" s="11"/>
-      <c r="F20" s="11"/>
-      <c r="G20" s="12"/>
-      <c r="H20" s="10"/>
-      <c r="I20" s="11"/>
-      <c r="J20" s="11"/>
-      <c r="K20" s="12"/>
-      <c r="L20" s="10"/>
-      <c r="M20" s="11"/>
-      <c r="N20" s="11"/>
-      <c r="O20" s="12"/>
-      <c r="P20" s="10"/>
-      <c r="Q20" s="11"/>
-      <c r="R20" s="11"/>
-      <c r="S20" s="12"/>
-      <c r="T20" s="10"/>
-      <c r="U20" s="11"/>
-      <c r="V20" s="12"/>
-      <c r="W20" s="10"/>
-      <c r="X20" s="11"/>
-      <c r="Y20" s="12"/>
-      <c r="Z20" s="10"/>
-      <c r="AA20" s="12"/>
-    </row>
-    <row r="21" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+        <v>52</v>
+      </c>
+      <c r="C20" s="23"/>
+      <c r="D20" s="24"/>
+      <c r="E20" s="24"/>
+      <c r="F20" s="24"/>
+      <c r="G20" s="25"/>
+      <c r="H20" s="23"/>
+      <c r="I20" s="24"/>
+      <c r="J20" s="24"/>
+      <c r="K20" s="25"/>
+      <c r="L20" s="23"/>
+      <c r="M20" s="24"/>
+      <c r="N20" s="24"/>
+      <c r="O20" s="25"/>
+      <c r="P20" s="23"/>
+      <c r="Q20" s="24"/>
+      <c r="R20" s="24"/>
+      <c r="S20" s="25"/>
+      <c r="T20" s="23"/>
+      <c r="U20" s="24"/>
+      <c r="V20" s="25"/>
+      <c r="W20" s="23"/>
+      <c r="X20" s="24"/>
+      <c r="Y20" s="25"/>
+      <c r="Z20" s="23"/>
+      <c r="AA20" s="25"/>
+    </row>
+    <row r="21" spans="1:27" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A21" s="3">
         <v>15</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C21" s="10"/>
       <c r="D21" s="11"/>
@@ -1461,7 +1483,7 @@
         <v>16</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C22" s="10"/>
       <c r="D22" s="11"/>
@@ -1494,7 +1516,7 @@
         <v>17</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C23" s="10"/>
       <c r="D23" s="11"/>
@@ -1527,7 +1549,7 @@
         <v>18</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C24" s="10"/>
       <c r="D24" s="11"/>
@@ -1556,164 +1578,158 @@
       <c r="AA24" s="12"/>
     </row>
     <row r="25" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="13" t="s">
+      <c r="A25" s="3">
+        <v>19</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C25" s="10"/>
+      <c r="D25" s="11"/>
+      <c r="E25" s="11"/>
+      <c r="F25" s="11"/>
+      <c r="G25" s="12"/>
+      <c r="H25" s="10"/>
+      <c r="I25" s="11"/>
+      <c r="J25" s="11"/>
+      <c r="K25" s="12"/>
+      <c r="L25" s="10"/>
+      <c r="M25" s="11"/>
+      <c r="N25" s="11"/>
+      <c r="O25" s="12"/>
+      <c r="P25" s="10"/>
+      <c r="Q25" s="11"/>
+      <c r="R25" s="11"/>
+      <c r="S25" s="12"/>
+      <c r="T25" s="10"/>
+      <c r="U25" s="11"/>
+      <c r="V25" s="12"/>
+      <c r="W25" s="10"/>
+      <c r="X25" s="11"/>
+      <c r="Y25" s="12"/>
+      <c r="Z25" s="10"/>
+      <c r="AA25" s="12"/>
+    </row>
+    <row r="26" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="16" t="s">
         <v>27</v>
       </c>
-      <c r="B25" s="9"/>
-      <c r="C25" s="9"/>
-      <c r="D25" s="9"/>
-      <c r="E25" s="9"/>
-      <c r="F25" s="9"/>
-      <c r="G25" s="9"/>
-      <c r="H25" s="9"/>
-      <c r="I25" s="9"/>
-      <c r="J25" s="9"/>
-      <c r="K25" s="9"/>
-      <c r="L25" s="9"/>
-      <c r="M25" s="9"/>
-      <c r="N25" s="9"/>
-      <c r="O25" s="9"/>
-      <c r="P25" s="9"/>
-      <c r="Q25" s="9"/>
-      <c r="R25" s="9"/>
-      <c r="S25" s="9"/>
-      <c r="T25" s="9"/>
-      <c r="U25" s="9"/>
-      <c r="V25" s="9"/>
-      <c r="W25" s="9"/>
-      <c r="X25" s="9"/>
-      <c r="Y25" s="9"/>
-      <c r="Z25" s="9"/>
-      <c r="AA25" s="9"/>
-    </row>
-    <row r="26" spans="1:27" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A26" s="4" t="s">
+      <c r="B26" s="9"/>
+      <c r="C26" s="9"/>
+      <c r="D26" s="9"/>
+      <c r="E26" s="9"/>
+      <c r="F26" s="9"/>
+      <c r="G26" s="9"/>
+      <c r="H26" s="9"/>
+      <c r="I26" s="9"/>
+      <c r="J26" s="9"/>
+      <c r="K26" s="9"/>
+      <c r="L26" s="9"/>
+      <c r="M26" s="9"/>
+      <c r="N26" s="9"/>
+      <c r="O26" s="9"/>
+      <c r="P26" s="9"/>
+      <c r="Q26" s="9"/>
+      <c r="R26" s="9"/>
+      <c r="S26" s="9"/>
+      <c r="T26" s="9"/>
+      <c r="U26" s="9"/>
+      <c r="V26" s="9"/>
+      <c r="W26" s="9"/>
+      <c r="X26" s="9"/>
+      <c r="Y26" s="9"/>
+      <c r="Z26" s="9"/>
+      <c r="AA26" s="9"/>
+    </row>
+    <row r="27" spans="1:27" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A27" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B26" s="4" t="s">
+      <c r="B27" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C26" s="4" t="s">
+      <c r="C27" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D26" s="4" t="s">
+      <c r="D27" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="E26" s="4" t="s">
+      <c r="E27" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="F26" s="4" t="s">
+      <c r="F27" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="G26" s="4" t="s">
+      <c r="G27" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="H26" s="4" t="s">
+      <c r="H27" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="I26" s="4" t="s">
+      <c r="I27" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="J26" s="4" t="s">
+      <c r="J27" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="K26" s="4" t="s">
+      <c r="K27" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="L26" s="4" t="s">
+      <c r="L27" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="M26" s="4" t="s">
+      <c r="M27" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="N26" s="4" t="s">
+      <c r="N27" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="O26" s="4" t="s">
+      <c r="O27" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="P26" s="4" t="s">
+      <c r="P27" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="Q26" s="4" t="s">
+      <c r="Q27" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="R26" s="4" t="s">
+      <c r="R27" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="S26" s="4" t="s">
+      <c r="S27" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="T26" s="4" t="s">
+      <c r="T27" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="U26" s="4" t="s">
+      <c r="U27" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="V26" s="4" t="s">
+      <c r="V27" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="W26" s="4" t="s">
+      <c r="W27" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="X26" s="4" t="s">
+      <c r="X27" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="Y26" s="4" t="s">
+      <c r="Y27" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="Z26" s="4" t="s">
+      <c r="Z27" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="AA26" s="4" t="s">
+      <c r="AA27" s="4" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="27" spans="1:27" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A27" s="3">
-        <v>1</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="C27" s="3"/>
-      <c r="D27" s="3"/>
-      <c r="E27" s="3"/>
-      <c r="F27" s="3"/>
-      <c r="G27" s="3"/>
-      <c r="H27" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="I27" s="3"/>
-      <c r="J27" s="3"/>
-      <c r="K27" s="3"/>
-      <c r="L27" s="3"/>
-      <c r="M27" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="N27" s="3"/>
-      <c r="O27" s="3"/>
-      <c r="P27" s="3"/>
-      <c r="Q27" s="3"/>
-      <c r="R27" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="S27" s="3"/>
-      <c r="T27" s="3"/>
-      <c r="U27" s="3"/>
-      <c r="V27" s="3"/>
-      <c r="W27" s="1"/>
-      <c r="X27" s="3"/>
-      <c r="Y27" s="3"/>
-      <c r="Z27" s="3"/>
-      <c r="AA27" s="3"/>
     </row>
     <row r="28" spans="1:27" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A28" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="C28" s="3"/>
       <c r="D28" s="3"/>
@@ -1721,21 +1737,21 @@
       <c r="F28" s="3"/>
       <c r="G28" s="3"/>
       <c r="H28" s="1" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="I28" s="3"/>
       <c r="J28" s="3"/>
       <c r="K28" s="3"/>
       <c r="L28" s="3"/>
       <c r="M28" s="1" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="N28" s="3"/>
       <c r="O28" s="3"/>
       <c r="P28" s="3"/>
       <c r="Q28" s="3"/>
       <c r="R28" s="1" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="S28" s="3"/>
       <c r="T28" s="3"/>
@@ -1747,12 +1763,12 @@
       <c r="Z28" s="3"/>
       <c r="AA28" s="3"/>
     </row>
-    <row r="29" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:27" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A29" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C29" s="3"/>
       <c r="D29" s="3"/>
@@ -1760,29 +1776,27 @@
       <c r="F29" s="3"/>
       <c r="G29" s="3"/>
       <c r="H29" s="1" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="I29" s="3"/>
       <c r="J29" s="3"/>
       <c r="K29" s="3"/>
       <c r="L29" s="3"/>
       <c r="M29" s="1" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="N29" s="3"/>
       <c r="O29" s="3"/>
       <c r="P29" s="3"/>
       <c r="Q29" s="3"/>
       <c r="R29" s="1" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="S29" s="3"/>
       <c r="T29" s="3"/>
       <c r="U29" s="3"/>
       <c r="V29" s="3"/>
-      <c r="W29" s="1" t="s">
-        <v>91</v>
-      </c>
+      <c r="W29" s="1"/>
       <c r="X29" s="3"/>
       <c r="Y29" s="3"/>
       <c r="Z29" s="3"/>
@@ -1790,34 +1804,40 @@
     </row>
     <row r="30" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="3">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C30" s="3"/>
       <c r="D30" s="3"/>
       <c r="E30" s="3"/>
       <c r="F30" s="3"/>
       <c r="G30" s="3"/>
-      <c r="H30" s="1"/>
+      <c r="H30" s="1" t="s">
+        <v>88</v>
+      </c>
       <c r="I30" s="3"/>
       <c r="J30" s="3"/>
       <c r="K30" s="3"/>
       <c r="L30" s="3"/>
       <c r="M30" s="1" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="N30" s="3"/>
       <c r="O30" s="3"/>
       <c r="P30" s="3"/>
       <c r="Q30" s="3"/>
-      <c r="R30" s="1"/>
+      <c r="R30" s="1" t="s">
+        <v>90</v>
+      </c>
       <c r="S30" s="3"/>
       <c r="T30" s="3"/>
       <c r="U30" s="3"/>
       <c r="V30" s="3"/>
-      <c r="W30" s="1"/>
+      <c r="W30" s="1" t="s">
+        <v>91</v>
+      </c>
       <c r="X30" s="3"/>
       <c r="Y30" s="3"/>
       <c r="Z30" s="3"/>
@@ -1825,24 +1845,24 @@
     </row>
     <row r="31" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="3">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>34</v>
+        <v>79</v>
       </c>
       <c r="C31" s="3"/>
       <c r="D31" s="3"/>
       <c r="E31" s="3"/>
       <c r="F31" s="3"/>
       <c r="G31" s="3"/>
-      <c r="H31" s="1" t="s">
-        <v>35</v>
-      </c>
+      <c r="H31" s="1"/>
       <c r="I31" s="3"/>
       <c r="J31" s="3"/>
       <c r="K31" s="3"/>
       <c r="L31" s="3"/>
-      <c r="M31" s="1"/>
+      <c r="M31" s="1" t="s">
+        <v>92</v>
+      </c>
       <c r="N31" s="3"/>
       <c r="O31" s="3"/>
       <c r="P31" s="3"/>
@@ -1860,10 +1880,10 @@
     </row>
     <row r="32" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="3">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="C32" s="3"/>
       <c r="D32" s="3"/>
@@ -1871,7 +1891,7 @@
       <c r="F32" s="3"/>
       <c r="G32" s="3"/>
       <c r="H32" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="I32" s="3"/>
       <c r="J32" s="3"/>
@@ -1882,9 +1902,7 @@
       <c r="O32" s="3"/>
       <c r="P32" s="3"/>
       <c r="Q32" s="3"/>
-      <c r="R32" s="1" t="s">
-        <v>37</v>
-      </c>
+      <c r="R32" s="1"/>
       <c r="S32" s="3"/>
       <c r="T32" s="3"/>
       <c r="U32" s="3"/>
@@ -1897,10 +1915,10 @@
     </row>
     <row r="33" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="3">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="C33" s="3"/>
       <c r="D33" s="3"/>
@@ -1908,21 +1926,19 @@
       <c r="F33" s="3"/>
       <c r="G33" s="3"/>
       <c r="H33" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="I33" s="3"/>
       <c r="J33" s="3"/>
       <c r="K33" s="3"/>
       <c r="L33" s="3"/>
-      <c r="M33" s="1" t="s">
-        <v>93</v>
-      </c>
+      <c r="M33" s="1"/>
       <c r="N33" s="3"/>
       <c r="O33" s="3"/>
       <c r="P33" s="3"/>
       <c r="Q33" s="3"/>
       <c r="R33" s="1" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="S33" s="3"/>
       <c r="T33" s="3"/>
@@ -1936,10 +1952,10 @@
     </row>
     <row r="34" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="3">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>80</v>
+        <v>22</v>
       </c>
       <c r="C34" s="3"/>
       <c r="D34" s="3"/>
@@ -1947,21 +1963,21 @@
       <c r="F34" s="3"/>
       <c r="G34" s="3"/>
       <c r="H34" s="1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="I34" s="3"/>
       <c r="J34" s="3"/>
       <c r="K34" s="3"/>
       <c r="L34" s="3"/>
       <c r="M34" s="1" t="s">
-        <v>39</v>
+        <v>93</v>
       </c>
       <c r="N34" s="3"/>
       <c r="O34" s="3"/>
       <c r="P34" s="3"/>
       <c r="Q34" s="3"/>
       <c r="R34" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="S34" s="3"/>
       <c r="T34" s="3"/>
@@ -1975,10 +1991,10 @@
     </row>
     <row r="35" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="3">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>18</v>
+        <v>80</v>
       </c>
       <c r="C35" s="3"/>
       <c r="D35" s="3"/>
@@ -1986,19 +2002,21 @@
       <c r="F35" s="3"/>
       <c r="G35" s="3"/>
       <c r="H35" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="I35" s="3"/>
       <c r="J35" s="3"/>
       <c r="K35" s="3"/>
       <c r="L35" s="3"/>
-      <c r="M35" s="1"/>
+      <c r="M35" s="1" t="s">
+        <v>39</v>
+      </c>
       <c r="N35" s="3"/>
       <c r="O35" s="3"/>
       <c r="P35" s="3"/>
       <c r="Q35" s="3"/>
       <c r="R35" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="S35" s="3"/>
       <c r="T35" s="3"/>
@@ -2012,10 +2030,10 @@
     </row>
     <row r="36" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="3">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C36" s="3"/>
       <c r="D36" s="3"/>
@@ -2023,7 +2041,7 @@
       <c r="F36" s="3"/>
       <c r="G36" s="3"/>
       <c r="H36" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I36" s="3"/>
       <c r="J36" s="3"/>
@@ -2034,7 +2052,9 @@
       <c r="O36" s="3"/>
       <c r="P36" s="3"/>
       <c r="Q36" s="3"/>
-      <c r="R36" s="1"/>
+      <c r="R36" s="1" t="s">
+        <v>44</v>
+      </c>
       <c r="S36" s="3"/>
       <c r="T36" s="3"/>
       <c r="U36" s="3"/>
@@ -2045,12 +2065,12 @@
       <c r="Z36" s="3"/>
       <c r="AA36" s="3"/>
     </row>
-    <row r="37" spans="1:27" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="3">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>46</v>
+        <v>19</v>
       </c>
       <c r="C37" s="3"/>
       <c r="D37" s="3"/>
@@ -2058,7 +2078,7 @@
       <c r="F37" s="3"/>
       <c r="G37" s="3"/>
       <c r="H37" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="I37" s="3"/>
       <c r="J37" s="3"/>
@@ -2069,9 +2089,7 @@
       <c r="O37" s="3"/>
       <c r="P37" s="3"/>
       <c r="Q37" s="3"/>
-      <c r="R37" s="1" t="s">
-        <v>49</v>
-      </c>
+      <c r="R37" s="1"/>
       <c r="S37" s="3"/>
       <c r="T37" s="3"/>
       <c r="U37" s="3"/>
@@ -2084,10 +2102,10 @@
     </row>
     <row r="38" spans="1:27" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A38" s="3">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="C38" s="3"/>
       <c r="D38" s="3"/>
@@ -2095,20 +2113,20 @@
       <c r="F38" s="3"/>
       <c r="G38" s="3"/>
       <c r="H38" s="1" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="I38" s="3"/>
       <c r="J38" s="3"/>
       <c r="K38" s="3"/>
       <c r="L38" s="3"/>
-      <c r="M38" s="1" t="s">
-        <v>48</v>
-      </c>
+      <c r="M38" s="1"/>
       <c r="N38" s="3"/>
       <c r="O38" s="3"/>
       <c r="P38" s="3"/>
       <c r="Q38" s="3"/>
-      <c r="R38" s="1"/>
+      <c r="R38" s="1" t="s">
+        <v>49</v>
+      </c>
       <c r="S38" s="3"/>
       <c r="T38" s="3"/>
       <c r="U38" s="3"/>
@@ -2121,10 +2139,10 @@
     </row>
     <row r="39" spans="1:27" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A39" s="3">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="C39" s="3"/>
       <c r="D39" s="3"/>
@@ -2132,22 +2150,20 @@
       <c r="F39" s="3"/>
       <c r="G39" s="3"/>
       <c r="H39" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="I39" s="3"/>
       <c r="J39" s="3"/>
       <c r="K39" s="3"/>
       <c r="L39" s="3"/>
       <c r="M39" s="1" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="N39" s="3"/>
       <c r="O39" s="3"/>
       <c r="P39" s="3"/>
       <c r="Q39" s="3"/>
-      <c r="R39" s="1" t="s">
-        <v>54</v>
-      </c>
+      <c r="R39" s="1"/>
       <c r="S39" s="3"/>
       <c r="T39" s="3"/>
       <c r="U39" s="3"/>
@@ -2160,10 +2176,10 @@
     </row>
     <row r="40" spans="1:27" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A40" s="3">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>55</v>
+        <v>81</v>
       </c>
       <c r="C40" s="3"/>
       <c r="D40" s="3"/>
@@ -2171,21 +2187,21 @@
       <c r="F40" s="3"/>
       <c r="G40" s="3"/>
       <c r="H40" s="1" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="I40" s="3"/>
       <c r="J40" s="3"/>
       <c r="K40" s="3"/>
       <c r="L40" s="3"/>
       <c r="M40" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="N40" s="3"/>
       <c r="O40" s="3"/>
       <c r="P40" s="3"/>
       <c r="Q40" s="3"/>
       <c r="R40" s="1" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="S40" s="3"/>
       <c r="T40" s="3"/>
@@ -2199,10 +2215,10 @@
     </row>
     <row r="41" spans="1:27" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A41" s="3">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="C41" s="3"/>
       <c r="D41" s="3"/>
@@ -2210,29 +2226,27 @@
       <c r="F41" s="3"/>
       <c r="G41" s="3"/>
       <c r="H41" s="1" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="I41" s="3"/>
       <c r="J41" s="3"/>
       <c r="K41" s="3"/>
       <c r="L41" s="3"/>
       <c r="M41" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="N41" s="3"/>
       <c r="O41" s="3"/>
       <c r="P41" s="3"/>
       <c r="Q41" s="3"/>
       <c r="R41" s="1" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="S41" s="3"/>
       <c r="T41" s="3"/>
       <c r="U41" s="3"/>
       <c r="V41" s="3"/>
-      <c r="W41" s="1" t="s">
-        <v>62</v>
-      </c>
+      <c r="W41" s="1"/>
       <c r="X41" s="3"/>
       <c r="Y41" s="3"/>
       <c r="Z41" s="3"/>
@@ -2240,10 +2254,10 @@
     </row>
     <row r="42" spans="1:27" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A42" s="3">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C42" s="3"/>
       <c r="D42" s="3"/>
@@ -2251,28 +2265,28 @@
       <c r="F42" s="3"/>
       <c r="G42" s="3"/>
       <c r="H42" s="1" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="I42" s="3"/>
       <c r="J42" s="3"/>
       <c r="K42" s="3"/>
       <c r="L42" s="3"/>
       <c r="M42" s="1" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="N42" s="3"/>
       <c r="O42" s="3"/>
       <c r="P42" s="3"/>
       <c r="Q42" s="3"/>
       <c r="R42" s="1" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="S42" s="3"/>
       <c r="T42" s="3"/>
       <c r="U42" s="3"/>
       <c r="V42" s="3"/>
       <c r="W42" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="X42" s="3"/>
       <c r="Y42" s="3"/>
@@ -2280,66 +2294,72 @@
       <c r="AA42" s="3"/>
     </row>
     <row r="43" spans="1:27" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A43" s="13" t="s">
+      <c r="A43" s="3">
+        <v>16</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C43" s="3"/>
+      <c r="D43" s="3"/>
+      <c r="E43" s="3"/>
+      <c r="F43" s="3"/>
+      <c r="G43" s="3"/>
+      <c r="H43" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="I43" s="3"/>
+      <c r="J43" s="3"/>
+      <c r="K43" s="3"/>
+      <c r="L43" s="3"/>
+      <c r="M43" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="N43" s="3"/>
+      <c r="O43" s="3"/>
+      <c r="P43" s="3"/>
+      <c r="Q43" s="3"/>
+      <c r="R43" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="S43" s="3"/>
+      <c r="T43" s="3"/>
+      <c r="U43" s="3"/>
+      <c r="V43" s="3"/>
+      <c r="W43" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="X43" s="3"/>
+      <c r="Y43" s="3"/>
+      <c r="Z43" s="3"/>
+      <c r="AA43" s="3"/>
+    </row>
+    <row r="44" spans="1:27" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A44" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="B43" s="9"/>
-      <c r="C43" s="9"/>
-      <c r="D43" s="9"/>
-    </row>
-    <row r="44" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="4" t="s">
+      <c r="B44" s="9"/>
+      <c r="C44" s="9"/>
+      <c r="D44" s="9"/>
+    </row>
+    <row r="45" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A45" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B44" s="20" t="s">
+      <c r="B45" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="C44" s="12"/>
-      <c r="D44" s="16" t="s">
+      <c r="C45" s="12"/>
+      <c r="D45" s="21" t="s">
         <v>67</v>
       </c>
-      <c r="E44" s="12"/>
-      <c r="F44" s="21" t="s">
+      <c r="E45" s="12"/>
+      <c r="F45" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="G44" s="12"/>
-      <c r="I44" s="19" t="s">
+      <c r="G45" s="12"/>
+      <c r="I45" s="8" t="s">
         <v>69</v>
-      </c>
-      <c r="J44" s="9"/>
-      <c r="K44" s="9"/>
-      <c r="L44" s="9"/>
-      <c r="M44" s="9"/>
-      <c r="N44" s="9"/>
-      <c r="O44" s="9"/>
-      <c r="P44" s="9"/>
-      <c r="Q44" s="9"/>
-      <c r="S44" s="19" t="s">
-        <v>70</v>
-      </c>
-      <c r="T44" s="9"/>
-      <c r="U44" s="9"/>
-      <c r="V44" s="9"/>
-      <c r="W44" s="9"/>
-      <c r="X44" s="9"/>
-      <c r="Y44" s="9"/>
-      <c r="Z44" s="9"/>
-      <c r="AA44" s="9"/>
-    </row>
-    <row r="45" spans="1:27" ht="60" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A45" s="3">
-        <v>1</v>
-      </c>
-      <c r="B45" s="14" t="s">
-        <v>71</v>
-      </c>
-      <c r="C45" s="12"/>
-      <c r="D45" s="10"/>
-      <c r="E45" s="12"/>
-      <c r="F45" s="10"/>
-      <c r="G45" s="12"/>
-      <c r="I45" s="13">
-        <v>1</v>
       </c>
       <c r="J45" s="9"/>
       <c r="K45" s="9"/>
@@ -2349,8 +2369,8 @@
       <c r="O45" s="9"/>
       <c r="P45" s="9"/>
       <c r="Q45" s="9"/>
-      <c r="S45" s="13">
-        <v>1</v>
+      <c r="S45" s="8" t="s">
+        <v>70</v>
       </c>
       <c r="T45" s="9"/>
       <c r="U45" s="9"/>
@@ -2361,20 +2381,20 @@
       <c r="Z45" s="9"/>
       <c r="AA45" s="9"/>
     </row>
-    <row r="46" spans="1:27" ht="62.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:27" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" s="3">
-        <v>2</v>
-      </c>
-      <c r="B46" s="14" t="s">
-        <v>72</v>
+        <v>1</v>
+      </c>
+      <c r="B46" s="22" t="s">
+        <v>71</v>
       </c>
       <c r="C46" s="12"/>
       <c r="D46" s="10"/>
       <c r="E46" s="12"/>
       <c r="F46" s="10"/>
       <c r="G46" s="12"/>
-      <c r="I46" s="13" t="s">
-        <v>73</v>
+      <c r="I46" s="16">
+        <v>1</v>
       </c>
       <c r="J46" s="9"/>
       <c r="K46" s="9"/>
@@ -2384,8 +2404,8 @@
       <c r="O46" s="9"/>
       <c r="P46" s="9"/>
       <c r="Q46" s="9"/>
-      <c r="S46" s="13">
-        <v>2</v>
+      <c r="S46" s="16">
+        <v>1</v>
       </c>
       <c r="T46" s="9"/>
       <c r="U46" s="9"/>
@@ -2396,16 +2416,20 @@
       <c r="Z46" s="9"/>
       <c r="AA46" s="9"/>
     </row>
-    <row r="47" spans="1:27" ht="72.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A47" s="5"/>
-      <c r="B47" s="8"/>
-      <c r="C47" s="9"/>
-      <c r="D47" s="8"/>
-      <c r="E47" s="9"/>
-      <c r="F47" s="8"/>
-      <c r="G47" s="9"/>
-      <c r="I47" s="13" t="s">
-        <v>74</v>
+    <row r="47" spans="1:27" ht="62.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A47" s="3">
+        <v>2</v>
+      </c>
+      <c r="B47" s="22" t="s">
+        <v>72</v>
+      </c>
+      <c r="C47" s="12"/>
+      <c r="D47" s="10"/>
+      <c r="E47" s="12"/>
+      <c r="F47" s="10"/>
+      <c r="G47" s="12"/>
+      <c r="I47" s="16" t="s">
+        <v>73</v>
       </c>
       <c r="J47" s="9"/>
       <c r="K47" s="9"/>
@@ -2415,8 +2439,8 @@
       <c r="O47" s="9"/>
       <c r="P47" s="9"/>
       <c r="Q47" s="9"/>
-      <c r="S47" s="13">
-        <v>3</v>
+      <c r="S47" s="16">
+        <v>2</v>
       </c>
       <c r="T47" s="9"/>
       <c r="U47" s="9"/>
@@ -2427,16 +2451,16 @@
       <c r="Z47" s="9"/>
       <c r="AA47" s="9"/>
     </row>
-    <row r="48" spans="1:27" ht="95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:27" ht="72.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A48" s="5"/>
-      <c r="B48" s="8"/>
+      <c r="B48" s="17"/>
       <c r="C48" s="9"/>
-      <c r="D48" s="8"/>
+      <c r="D48" s="17"/>
       <c r="E48" s="9"/>
-      <c r="F48" s="8"/>
+      <c r="F48" s="17"/>
       <c r="G48" s="9"/>
-      <c r="I48" s="13" t="s">
-        <v>75</v>
+      <c r="I48" s="16" t="s">
+        <v>74</v>
       </c>
       <c r="J48" s="9"/>
       <c r="K48" s="9"/>
@@ -2446,8 +2470,8 @@
       <c r="O48" s="9"/>
       <c r="P48" s="9"/>
       <c r="Q48" s="9"/>
-      <c r="S48" s="13" t="s">
-        <v>75</v>
+      <c r="S48" s="16">
+        <v>3</v>
       </c>
       <c r="T48" s="9"/>
       <c r="U48" s="9"/>
@@ -2458,108 +2482,92 @@
       <c r="Z48" s="9"/>
       <c r="AA48" s="9"/>
     </row>
-    <row r="49" ht="25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="49" spans="1:27" ht="95" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A49" s="5"/>
+      <c r="B49" s="17"/>
+      <c r="C49" s="9"/>
+      <c r="D49" s="17"/>
+      <c r="E49" s="9"/>
+      <c r="F49" s="17"/>
+      <c r="G49" s="9"/>
+      <c r="I49" s="16" t="s">
+        <v>75</v>
+      </c>
+      <c r="J49" s="9"/>
+      <c r="K49" s="9"/>
+      <c r="L49" s="9"/>
+      <c r="M49" s="9"/>
+      <c r="N49" s="9"/>
+      <c r="O49" s="9"/>
+      <c r="P49" s="9"/>
+      <c r="Q49" s="9"/>
+      <c r="S49" s="16" t="s">
+        <v>75</v>
+      </c>
+      <c r="T49" s="9"/>
+      <c r="U49" s="9"/>
+      <c r="V49" s="9"/>
+      <c r="W49" s="9"/>
+      <c r="X49" s="9"/>
+      <c r="Y49" s="9"/>
+      <c r="Z49" s="9"/>
+      <c r="AA49" s="9"/>
+    </row>
+    <row r="50" spans="1:27" ht="25" customHeight="1" x14ac:dyDescent="0.35"/>
   </sheetData>
-  <mergeCells count="167">
-    <mergeCell ref="I44:Q44"/>
-    <mergeCell ref="L18:O18"/>
-    <mergeCell ref="P11:S11"/>
-    <mergeCell ref="H11:K11"/>
-    <mergeCell ref="Z13:AA13"/>
-    <mergeCell ref="C13:G13"/>
-    <mergeCell ref="T20:V20"/>
-    <mergeCell ref="P10:S10"/>
-    <mergeCell ref="W4:AA4"/>
-    <mergeCell ref="L6:O6"/>
-    <mergeCell ref="Z8:AA8"/>
-    <mergeCell ref="L8:O8"/>
-    <mergeCell ref="T8:V8"/>
-    <mergeCell ref="C10:G10"/>
-    <mergeCell ref="Z19:AA19"/>
-    <mergeCell ref="Z9:AA9"/>
-    <mergeCell ref="W15:Y15"/>
-    <mergeCell ref="Z18:AA18"/>
-    <mergeCell ref="W24:Y24"/>
-    <mergeCell ref="C12:G12"/>
-    <mergeCell ref="T19:V19"/>
-    <mergeCell ref="W14:Y14"/>
-    <mergeCell ref="L19:O19"/>
-    <mergeCell ref="A2:AA2"/>
-    <mergeCell ref="T23:V23"/>
-    <mergeCell ref="W19:Y19"/>
+  <mergeCells count="160">
+    <mergeCell ref="B49:C49"/>
+    <mergeCell ref="P13:S13"/>
+    <mergeCell ref="D49:E49"/>
+    <mergeCell ref="L12:O12"/>
+    <mergeCell ref="T12:V12"/>
+    <mergeCell ref="A3:AA3"/>
+    <mergeCell ref="P15:S15"/>
+    <mergeCell ref="H22:K22"/>
+    <mergeCell ref="S48:AA48"/>
+    <mergeCell ref="W18:Y18"/>
+    <mergeCell ref="A5:AA5"/>
+    <mergeCell ref="W12:Y12"/>
+    <mergeCell ref="L14:O14"/>
+    <mergeCell ref="D46:E46"/>
+    <mergeCell ref="W21:Y21"/>
+    <mergeCell ref="H6:K6"/>
+    <mergeCell ref="S47:AA47"/>
+    <mergeCell ref="P23:S23"/>
+    <mergeCell ref="H23:K23"/>
+    <mergeCell ref="P9:S9"/>
+    <mergeCell ref="C9:G9"/>
+    <mergeCell ref="L16:O16"/>
+    <mergeCell ref="T16:V16"/>
+    <mergeCell ref="C18:G18"/>
+    <mergeCell ref="S46:AA46"/>
+    <mergeCell ref="W16:Y16"/>
+    <mergeCell ref="P18:S18"/>
+    <mergeCell ref="B48:C48"/>
+    <mergeCell ref="H17:K17"/>
+    <mergeCell ref="L11:O11"/>
+    <mergeCell ref="C14:G14"/>
+    <mergeCell ref="H24:K24"/>
     <mergeCell ref="P21:S21"/>
-    <mergeCell ref="I46:Q46"/>
-    <mergeCell ref="W9:Y9"/>
-    <mergeCell ref="T6:V6"/>
-    <mergeCell ref="L20:O20"/>
-    <mergeCell ref="Z22:AA22"/>
-    <mergeCell ref="C22:G22"/>
-    <mergeCell ref="H10:K10"/>
-    <mergeCell ref="P23:S23"/>
-    <mergeCell ref="L13:O13"/>
-    <mergeCell ref="Z24:AA24"/>
-    <mergeCell ref="A43:D43"/>
-    <mergeCell ref="P6:S6"/>
-    <mergeCell ref="C24:G24"/>
-    <mergeCell ref="Z14:AA14"/>
-    <mergeCell ref="F45:G45"/>
-    <mergeCell ref="T21:V21"/>
-    <mergeCell ref="C8:G8"/>
-    <mergeCell ref="L15:O15"/>
-    <mergeCell ref="T15:V15"/>
-    <mergeCell ref="C23:G23"/>
-    <mergeCell ref="I48:Q48"/>
-    <mergeCell ref="S48:AA48"/>
-    <mergeCell ref="Z16:AA16"/>
-    <mergeCell ref="H4:V4"/>
-    <mergeCell ref="C19:G19"/>
-    <mergeCell ref="W21:Y21"/>
-    <mergeCell ref="H14:K14"/>
-    <mergeCell ref="L22:O22"/>
-    <mergeCell ref="W23:Y23"/>
-    <mergeCell ref="H16:K16"/>
-    <mergeCell ref="I45:Q45"/>
-    <mergeCell ref="H24:K24"/>
-    <mergeCell ref="H19:K19"/>
-    <mergeCell ref="W13:Y13"/>
+    <mergeCell ref="C16:G16"/>
+    <mergeCell ref="L25:O25"/>
+    <mergeCell ref="D45:E45"/>
+    <mergeCell ref="P25:S25"/>
+    <mergeCell ref="Z11:AA11"/>
+    <mergeCell ref="A26:AA26"/>
+    <mergeCell ref="Z21:AA21"/>
     <mergeCell ref="C21:G21"/>
-    <mergeCell ref="W22:Y22"/>
-    <mergeCell ref="H9:K9"/>
-    <mergeCell ref="T9:V9"/>
-    <mergeCell ref="W10:Y10"/>
+    <mergeCell ref="P17:S17"/>
+    <mergeCell ref="D47:E47"/>
     <mergeCell ref="F47:G47"/>
-    <mergeCell ref="T18:V18"/>
-    <mergeCell ref="F44:G44"/>
-    <mergeCell ref="L17:O17"/>
-    <mergeCell ref="Z23:AA23"/>
-    <mergeCell ref="F48:G48"/>
-    <mergeCell ref="Z15:AA15"/>
-    <mergeCell ref="P12:S12"/>
-    <mergeCell ref="W11:Y11"/>
-    <mergeCell ref="H18:K18"/>
-    <mergeCell ref="H12:K12"/>
-    <mergeCell ref="I47:Q47"/>
-    <mergeCell ref="S44:AA44"/>
-    <mergeCell ref="L21:O21"/>
-    <mergeCell ref="H20:K20"/>
-    <mergeCell ref="L23:O23"/>
-    <mergeCell ref="P14:S14"/>
-    <mergeCell ref="H13:K13"/>
-    <mergeCell ref="T13:V13"/>
-    <mergeCell ref="T22:V22"/>
-    <mergeCell ref="P16:S16"/>
-    <mergeCell ref="H15:K15"/>
-    <mergeCell ref="Z17:AA17"/>
-    <mergeCell ref="C11:G11"/>
-    <mergeCell ref="C17:G17"/>
-    <mergeCell ref="T24:V24"/>
-    <mergeCell ref="B44:C44"/>
-    <mergeCell ref="T14:V14"/>
-    <mergeCell ref="T17:V17"/>
+    <mergeCell ref="T11:V11"/>
+    <mergeCell ref="D48:E48"/>
+    <mergeCell ref="B46:C46"/>
+    <mergeCell ref="B47:C47"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="L9:O9"/>
     <mergeCell ref="W6:Y6"/>
-    <mergeCell ref="Z21:AA21"/>
+    <mergeCell ref="Z22:AA22"/>
     <mergeCell ref="Z6:AA6"/>
     <mergeCell ref="C6:G6"/>
     <mergeCell ref="L10:O10"/>
@@ -2567,7 +2575,6 @@
     <mergeCell ref="P8:S8"/>
     <mergeCell ref="H8:K8"/>
     <mergeCell ref="Z10:AA10"/>
-    <mergeCell ref="P19:S19"/>
     <mergeCell ref="Z12:AA12"/>
     <mergeCell ref="C15:G15"/>
     <mergeCell ref="W8:Y8"/>
@@ -2580,54 +2587,95 @@
     <mergeCell ref="W7:Y7"/>
     <mergeCell ref="Z7:AA7"/>
     <mergeCell ref="C4:G4"/>
+    <mergeCell ref="F49:G49"/>
+    <mergeCell ref="Z15:AA15"/>
+    <mergeCell ref="P12:S12"/>
+    <mergeCell ref="W11:Y11"/>
+    <mergeCell ref="H18:K18"/>
+    <mergeCell ref="H12:K12"/>
+    <mergeCell ref="I48:Q48"/>
     <mergeCell ref="S45:AA45"/>
-    <mergeCell ref="W16:Y16"/>
-    <mergeCell ref="P18:S18"/>
-    <mergeCell ref="B47:C47"/>
-    <mergeCell ref="H17:K17"/>
-    <mergeCell ref="L11:O11"/>
-    <mergeCell ref="C14:G14"/>
-    <mergeCell ref="H23:K23"/>
-    <mergeCell ref="P20:S20"/>
-    <mergeCell ref="C16:G16"/>
+    <mergeCell ref="L22:O22"/>
+    <mergeCell ref="H21:K21"/>
     <mergeCell ref="L24:O24"/>
-    <mergeCell ref="D44:E44"/>
+    <mergeCell ref="P14:S14"/>
+    <mergeCell ref="H13:K13"/>
+    <mergeCell ref="T13:V13"/>
+    <mergeCell ref="T23:V23"/>
+    <mergeCell ref="P16:S16"/>
+    <mergeCell ref="H15:K15"/>
+    <mergeCell ref="Z17:AA17"/>
+    <mergeCell ref="C11:G11"/>
+    <mergeCell ref="C17:G17"/>
+    <mergeCell ref="T25:V25"/>
+    <mergeCell ref="B45:C45"/>
+    <mergeCell ref="T14:V14"/>
+    <mergeCell ref="T17:V17"/>
+    <mergeCell ref="I49:Q49"/>
+    <mergeCell ref="S49:AA49"/>
+    <mergeCell ref="Z16:AA16"/>
+    <mergeCell ref="H4:V4"/>
+    <mergeCell ref="W22:Y22"/>
+    <mergeCell ref="H14:K14"/>
+    <mergeCell ref="L23:O23"/>
+    <mergeCell ref="W24:Y24"/>
+    <mergeCell ref="H16:K16"/>
+    <mergeCell ref="I46:Q46"/>
+    <mergeCell ref="H25:K25"/>
+    <mergeCell ref="W13:Y13"/>
+    <mergeCell ref="C22:G22"/>
+    <mergeCell ref="W23:Y23"/>
+    <mergeCell ref="H9:K9"/>
+    <mergeCell ref="T9:V9"/>
+    <mergeCell ref="W10:Y10"/>
+    <mergeCell ref="F48:G48"/>
+    <mergeCell ref="T18:V18"/>
+    <mergeCell ref="F45:G45"/>
+    <mergeCell ref="L17:O17"/>
+    <mergeCell ref="Z24:AA24"/>
+    <mergeCell ref="A2:AA2"/>
+    <mergeCell ref="T24:V24"/>
+    <mergeCell ref="P22:S22"/>
+    <mergeCell ref="I47:Q47"/>
+    <mergeCell ref="W9:Y9"/>
+    <mergeCell ref="T6:V6"/>
+    <mergeCell ref="L21:O21"/>
+    <mergeCell ref="Z23:AA23"/>
+    <mergeCell ref="C23:G23"/>
+    <mergeCell ref="H10:K10"/>
     <mergeCell ref="P24:S24"/>
-    <mergeCell ref="Z11:AA11"/>
-    <mergeCell ref="A25:AA25"/>
-    <mergeCell ref="Z20:AA20"/>
-    <mergeCell ref="C20:G20"/>
-    <mergeCell ref="P17:S17"/>
-    <mergeCell ref="D46:E46"/>
+    <mergeCell ref="L13:O13"/>
+    <mergeCell ref="Z25:AA25"/>
+    <mergeCell ref="A44:D44"/>
+    <mergeCell ref="P6:S6"/>
+    <mergeCell ref="C25:G25"/>
+    <mergeCell ref="Z14:AA14"/>
     <mergeCell ref="F46:G46"/>
-    <mergeCell ref="T11:V11"/>
-    <mergeCell ref="D47:E47"/>
-    <mergeCell ref="B45:C45"/>
-    <mergeCell ref="B46:C46"/>
-    <mergeCell ref="B48:C48"/>
-    <mergeCell ref="P13:S13"/>
-    <mergeCell ref="D48:E48"/>
-    <mergeCell ref="L12:O12"/>
-    <mergeCell ref="T12:V12"/>
-    <mergeCell ref="A3:AA3"/>
-    <mergeCell ref="P15:S15"/>
-    <mergeCell ref="H21:K21"/>
-    <mergeCell ref="S47:AA47"/>
-    <mergeCell ref="W18:Y18"/>
-    <mergeCell ref="A5:AA5"/>
-    <mergeCell ref="W12:Y12"/>
-    <mergeCell ref="L14:O14"/>
-    <mergeCell ref="D45:E45"/>
-    <mergeCell ref="W20:Y20"/>
-    <mergeCell ref="H6:K6"/>
-    <mergeCell ref="S46:AA46"/>
-    <mergeCell ref="P22:S22"/>
-    <mergeCell ref="H22:K22"/>
-    <mergeCell ref="P9:S9"/>
-    <mergeCell ref="C9:G9"/>
-    <mergeCell ref="L16:O16"/>
-    <mergeCell ref="T16:V16"/>
-    <mergeCell ref="C18:G18"/>
+    <mergeCell ref="T22:V22"/>
+    <mergeCell ref="C8:G8"/>
+    <mergeCell ref="L15:O15"/>
+    <mergeCell ref="T15:V15"/>
+    <mergeCell ref="C24:G24"/>
+    <mergeCell ref="I45:Q45"/>
+    <mergeCell ref="L18:O18"/>
+    <mergeCell ref="P11:S11"/>
+    <mergeCell ref="H11:K11"/>
+    <mergeCell ref="Z13:AA13"/>
+    <mergeCell ref="C13:G13"/>
+    <mergeCell ref="T21:V21"/>
+    <mergeCell ref="P10:S10"/>
+    <mergeCell ref="W4:AA4"/>
+    <mergeCell ref="L6:O6"/>
+    <mergeCell ref="Z8:AA8"/>
+    <mergeCell ref="L8:O8"/>
+    <mergeCell ref="T8:V8"/>
+    <mergeCell ref="C10:G10"/>
+    <mergeCell ref="Z9:AA9"/>
+    <mergeCell ref="W15:Y15"/>
+    <mergeCell ref="Z18:AA18"/>
+    <mergeCell ref="W25:Y25"/>
+    <mergeCell ref="C12:G12"/>
+    <mergeCell ref="W14:Y14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Fix flexible final summary reporting and status export
</commit_message>
<xml_diff>
--- a/templates/template_general.xlsx
+++ b/templates/template_general.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Bot\Market_Survey\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9032AA15-8290-4939-9B1E-5C14B57541F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1B045FC-0648-4A64-95F5-ECCA58BAA02B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,12 +18,24 @@
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">Simaple_form!$A$1:$AA$49</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="95">
   <si>
     <t>Market Improvement Report</t>
   </si>
@@ -293,13 +305,30 @@
   </si>
   <si>
     <t>Dealer :                                                      Report Date:</t>
+  </si>
+  <si>
+    <t>No Compromise</t>
+  </si>
+  <si>
+    <t>1.Mass Products មិនត្រូវឲ្យខ្វះស្លកក្នុងផ្ទះមួយ
+(CBL/Wurkz/Exprez/Dazz/Water/Sport PET 500ml/Ize PET 500ml)</t>
+  </si>
+  <si>
+    <t>2.ផលិតផលហួសដឺឡេ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. ការបញ្ចូលរបាយការណ៍លក់មិនត្រឹមត្រូវ
+</t>
+  </si>
+  <si>
+    <t>4. របាយការណ៍លក់ជូនអតិថិជនមិនពិត (ទាំងចំនួនលក់ និងតម្លៃ)។</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -366,8 +395,20 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Noto Sans Khmer"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="20"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -387,6 +428,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF003B6F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -472,7 +519,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -507,11 +554,8 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -519,31 +563,41 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -937,11 +991,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AA50"/>
+  <dimension ref="A1:AA55"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -967,134 +1021,134 @@
       <c r="D1" s="5"/>
     </row>
     <row r="2" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="27" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="14"/>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="14"/>
-      <c r="I2" s="14"/>
-      <c r="J2" s="14"/>
-      <c r="K2" s="14"/>
-      <c r="L2" s="14"/>
-      <c r="M2" s="14"/>
-      <c r="N2" s="14"/>
-      <c r="O2" s="14"/>
-      <c r="P2" s="14"/>
-      <c r="Q2" s="14"/>
-      <c r="R2" s="14"/>
-      <c r="S2" s="14"/>
-      <c r="T2" s="14"/>
-      <c r="U2" s="14"/>
-      <c r="V2" s="14"/>
-      <c r="W2" s="14"/>
-      <c r="X2" s="14"/>
-      <c r="Y2" s="14"/>
-      <c r="Z2" s="14"/>
-      <c r="AA2" s="14"/>
+      <c r="A2" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
+      <c r="H2" s="13"/>
+      <c r="I2" s="13"/>
+      <c r="J2" s="13"/>
+      <c r="K2" s="13"/>
+      <c r="L2" s="13"/>
+      <c r="M2" s="13"/>
+      <c r="N2" s="13"/>
+      <c r="O2" s="13"/>
+      <c r="P2" s="13"/>
+      <c r="Q2" s="13"/>
+      <c r="R2" s="13"/>
+      <c r="S2" s="13"/>
+      <c r="T2" s="13"/>
+      <c r="U2" s="13"/>
+      <c r="V2" s="13"/>
+      <c r="W2" s="13"/>
+      <c r="X2" s="13"/>
+      <c r="Y2" s="13"/>
+      <c r="Z2" s="13"/>
+      <c r="AA2" s="13"/>
     </row>
     <row r="3" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="26" t="s">
         <v>89</v>
       </c>
-      <c r="B3" s="14"/>
-      <c r="C3" s="14"/>
-      <c r="D3" s="14"/>
-      <c r="E3" s="14"/>
-      <c r="F3" s="14"/>
-      <c r="G3" s="14"/>
-      <c r="H3" s="14"/>
-      <c r="I3" s="14"/>
-      <c r="J3" s="14"/>
-      <c r="K3" s="14"/>
-      <c r="L3" s="14"/>
-      <c r="M3" s="14"/>
-      <c r="N3" s="14"/>
-      <c r="O3" s="14"/>
-      <c r="P3" s="14"/>
-      <c r="Q3" s="14"/>
-      <c r="R3" s="14"/>
-      <c r="S3" s="14"/>
-      <c r="T3" s="14"/>
-      <c r="U3" s="14"/>
-      <c r="V3" s="14"/>
-      <c r="W3" s="14"/>
-      <c r="X3" s="14"/>
-      <c r="Y3" s="14"/>
-      <c r="Z3" s="14"/>
-      <c r="AA3" s="14"/>
+      <c r="B3" s="13"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
+      <c r="F3" s="13"/>
+      <c r="G3" s="13"/>
+      <c r="H3" s="13"/>
+      <c r="I3" s="13"/>
+      <c r="J3" s="13"/>
+      <c r="K3" s="13"/>
+      <c r="L3" s="13"/>
+      <c r="M3" s="13"/>
+      <c r="N3" s="13"/>
+      <c r="O3" s="13"/>
+      <c r="P3" s="13"/>
+      <c r="Q3" s="13"/>
+      <c r="R3" s="13"/>
+      <c r="S3" s="13"/>
+      <c r="T3" s="13"/>
+      <c r="U3" s="13"/>
+      <c r="V3" s="13"/>
+      <c r="W3" s="13"/>
+      <c r="X3" s="13"/>
+      <c r="Y3" s="13"/>
+      <c r="Z3" s="13"/>
+      <c r="AA3" s="13"/>
     </row>
     <row r="4" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A4" s="22" t="s">
         <v>86</v>
       </c>
-      <c r="B4" s="17"/>
+      <c r="B4" s="16"/>
       <c r="C4" s="22" t="s">
         <v>87</v>
       </c>
-      <c r="D4" s="16"/>
-      <c r="E4" s="16"/>
-      <c r="F4" s="16"/>
-      <c r="G4" s="17"/>
-      <c r="H4" s="25" t="s">
+      <c r="D4" s="15"/>
+      <c r="E4" s="15"/>
+      <c r="F4" s="15"/>
+      <c r="G4" s="16"/>
+      <c r="H4" s="19" t="s">
         <v>85</v>
       </c>
-      <c r="I4" s="16"/>
-      <c r="J4" s="16"/>
-      <c r="K4" s="16"/>
-      <c r="L4" s="16"/>
-      <c r="M4" s="16"/>
-      <c r="N4" s="16"/>
-      <c r="O4" s="16"/>
-      <c r="P4" s="16"/>
-      <c r="Q4" s="16"/>
-      <c r="R4" s="16"/>
-      <c r="S4" s="16"/>
-      <c r="T4" s="16"/>
-      <c r="U4" s="16"/>
-      <c r="V4" s="17"/>
+      <c r="I4" s="15"/>
+      <c r="J4" s="15"/>
+      <c r="K4" s="15"/>
+      <c r="L4" s="15"/>
+      <c r="M4" s="15"/>
+      <c r="N4" s="15"/>
+      <c r="O4" s="15"/>
+      <c r="P4" s="15"/>
+      <c r="Q4" s="15"/>
+      <c r="R4" s="15"/>
+      <c r="S4" s="15"/>
+      <c r="T4" s="15"/>
+      <c r="U4" s="15"/>
+      <c r="V4" s="16"/>
       <c r="W4" s="22" t="s">
         <v>88</v>
       </c>
-      <c r="X4" s="16"/>
-      <c r="Y4" s="16"/>
-      <c r="Z4" s="16"/>
-      <c r="AA4" s="17"/>
+      <c r="X4" s="15"/>
+      <c r="Y4" s="15"/>
+      <c r="Z4" s="15"/>
+      <c r="AA4" s="16"/>
     </row>
     <row r="5" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="20" t="s">
+      <c r="A5" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="16"/>
-      <c r="C5" s="16"/>
-      <c r="D5" s="16"/>
-      <c r="E5" s="16"/>
-      <c r="F5" s="16"/>
-      <c r="G5" s="16"/>
-      <c r="H5" s="16"/>
-      <c r="I5" s="16"/>
-      <c r="J5" s="16"/>
-      <c r="K5" s="16"/>
-      <c r="L5" s="16"/>
-      <c r="M5" s="16"/>
-      <c r="N5" s="16"/>
-      <c r="O5" s="16"/>
-      <c r="P5" s="16"/>
-      <c r="Q5" s="16"/>
-      <c r="R5" s="16"/>
-      <c r="S5" s="16"/>
-      <c r="T5" s="16"/>
-      <c r="U5" s="16"/>
-      <c r="V5" s="16"/>
-      <c r="W5" s="16"/>
-      <c r="X5" s="16"/>
-      <c r="Y5" s="16"/>
-      <c r="Z5" s="16"/>
-      <c r="AA5" s="17"/>
+      <c r="B5" s="15"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="15"/>
+      <c r="H5" s="15"/>
+      <c r="I5" s="15"/>
+      <c r="J5" s="15"/>
+      <c r="K5" s="15"/>
+      <c r="L5" s="15"/>
+      <c r="M5" s="15"/>
+      <c r="N5" s="15"/>
+      <c r="O5" s="15"/>
+      <c r="P5" s="15"/>
+      <c r="Q5" s="15"/>
+      <c r="R5" s="15"/>
+      <c r="S5" s="15"/>
+      <c r="T5" s="15"/>
+      <c r="U5" s="15"/>
+      <c r="V5" s="15"/>
+      <c r="W5" s="15"/>
+      <c r="X5" s="15"/>
+      <c r="Y5" s="15"/>
+      <c r="Z5" s="15"/>
+      <c r="AA5" s="16"/>
     </row>
     <row r="6" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
@@ -1103,45 +1157,45 @@
       <c r="B6" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="24" t="s">
+      <c r="C6" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="D6" s="16"/>
-      <c r="E6" s="16"/>
-      <c r="F6" s="16"/>
-      <c r="G6" s="17"/>
-      <c r="H6" s="21" t="s">
+      <c r="D6" s="15"/>
+      <c r="E6" s="15"/>
+      <c r="F6" s="15"/>
+      <c r="G6" s="16"/>
+      <c r="H6" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="I6" s="16"/>
-      <c r="J6" s="16"/>
-      <c r="K6" s="17"/>
-      <c r="L6" s="21" t="s">
+      <c r="I6" s="15"/>
+      <c r="J6" s="15"/>
+      <c r="K6" s="16"/>
+      <c r="L6" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="M6" s="16"/>
-      <c r="N6" s="16"/>
-      <c r="O6" s="17"/>
-      <c r="P6" s="21" t="s">
+      <c r="M6" s="15"/>
+      <c r="N6" s="15"/>
+      <c r="O6" s="16"/>
+      <c r="P6" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="Q6" s="16"/>
-      <c r="R6" s="16"/>
-      <c r="S6" s="17"/>
-      <c r="T6" s="21" t="s">
+      <c r="Q6" s="15"/>
+      <c r="R6" s="15"/>
+      <c r="S6" s="16"/>
+      <c r="T6" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="U6" s="16"/>
-      <c r="V6" s="17"/>
-      <c r="W6" s="23" t="s">
+      <c r="U6" s="15"/>
+      <c r="V6" s="16"/>
+      <c r="W6" s="24" t="s">
         <v>9</v>
       </c>
-      <c r="X6" s="16"/>
-      <c r="Y6" s="17"/>
-      <c r="Z6" s="23" t="s">
+      <c r="X6" s="15"/>
+      <c r="Y6" s="16"/>
+      <c r="Z6" s="24" t="s">
         <v>10</v>
       </c>
-      <c r="AA6" s="17"/>
+      <c r="AA6" s="16"/>
     </row>
     <row r="7" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="3">
@@ -1150,41 +1204,41 @@
       <c r="B7" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="15"/>
-      <c r="D7" s="16"/>
-      <c r="E7" s="16"/>
-      <c r="F7" s="16"/>
-      <c r="G7" s="17"/>
-      <c r="H7" s="15">
-        <v>0</v>
-      </c>
-      <c r="I7" s="16"/>
-      <c r="J7" s="16"/>
-      <c r="K7" s="17"/>
-      <c r="L7" s="15">
-        <v>0</v>
-      </c>
-      <c r="M7" s="16"/>
-      <c r="N7" s="16"/>
-      <c r="O7" s="17"/>
-      <c r="P7" s="15">
-        <v>0</v>
-      </c>
-      <c r="Q7" s="16"/>
-      <c r="R7" s="16"/>
-      <c r="S7" s="17"/>
-      <c r="T7" s="15">
-        <v>0</v>
-      </c>
-      <c r="U7" s="16"/>
-      <c r="V7" s="17"/>
-      <c r="W7" s="15">
-        <v>0</v>
-      </c>
-      <c r="X7" s="16"/>
-      <c r="Y7" s="17"/>
-      <c r="Z7" s="15"/>
-      <c r="AA7" s="17"/>
+      <c r="C7" s="14"/>
+      <c r="D7" s="15"/>
+      <c r="E7" s="15"/>
+      <c r="F7" s="15"/>
+      <c r="G7" s="16"/>
+      <c r="H7" s="14">
+        <v>0</v>
+      </c>
+      <c r="I7" s="15"/>
+      <c r="J7" s="15"/>
+      <c r="K7" s="16"/>
+      <c r="L7" s="14">
+        <v>0</v>
+      </c>
+      <c r="M7" s="15"/>
+      <c r="N7" s="15"/>
+      <c r="O7" s="16"/>
+      <c r="P7" s="14">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="15"/>
+      <c r="R7" s="15"/>
+      <c r="S7" s="16"/>
+      <c r="T7" s="14">
+        <v>0</v>
+      </c>
+      <c r="U7" s="15"/>
+      <c r="V7" s="16"/>
+      <c r="W7" s="14">
+        <v>0</v>
+      </c>
+      <c r="X7" s="15"/>
+      <c r="Y7" s="16"/>
+      <c r="Z7" s="14"/>
+      <c r="AA7" s="16"/>
     </row>
     <row r="8" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="3">
@@ -1193,41 +1247,41 @@
       <c r="B8" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="15"/>
-      <c r="D8" s="16"/>
-      <c r="E8" s="16"/>
-      <c r="F8" s="16"/>
-      <c r="G8" s="17"/>
-      <c r="H8" s="15">
-        <v>0</v>
-      </c>
-      <c r="I8" s="16"/>
-      <c r="J8" s="16"/>
-      <c r="K8" s="17"/>
-      <c r="L8" s="15">
-        <v>0</v>
-      </c>
-      <c r="M8" s="16"/>
-      <c r="N8" s="16"/>
-      <c r="O8" s="17"/>
-      <c r="P8" s="15">
-        <v>0</v>
-      </c>
-      <c r="Q8" s="16"/>
-      <c r="R8" s="16"/>
-      <c r="S8" s="17"/>
-      <c r="T8" s="26">
-        <v>0</v>
-      </c>
-      <c r="U8" s="16"/>
-      <c r="V8" s="17"/>
-      <c r="W8" s="15">
-        <v>0</v>
-      </c>
-      <c r="X8" s="16"/>
-      <c r="Y8" s="17"/>
-      <c r="Z8" s="15"/>
-      <c r="AA8" s="17"/>
+      <c r="C8" s="14"/>
+      <c r="D8" s="15"/>
+      <c r="E8" s="15"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="16"/>
+      <c r="H8" s="14">
+        <v>0</v>
+      </c>
+      <c r="I8" s="15"/>
+      <c r="J8" s="15"/>
+      <c r="K8" s="16"/>
+      <c r="L8" s="14">
+        <v>0</v>
+      </c>
+      <c r="M8" s="15"/>
+      <c r="N8" s="15"/>
+      <c r="O8" s="16"/>
+      <c r="P8" s="14">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="15"/>
+      <c r="R8" s="15"/>
+      <c r="S8" s="16"/>
+      <c r="T8" s="21">
+        <v>0</v>
+      </c>
+      <c r="U8" s="15"/>
+      <c r="V8" s="16"/>
+      <c r="W8" s="14">
+        <v>0</v>
+      </c>
+      <c r="X8" s="15"/>
+      <c r="Y8" s="16"/>
+      <c r="Z8" s="14"/>
+      <c r="AA8" s="16"/>
     </row>
     <row r="9" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="3">
@@ -1236,41 +1290,41 @@
       <c r="B9" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="15"/>
-      <c r="D9" s="16"/>
-      <c r="E9" s="16"/>
-      <c r="F9" s="16"/>
-      <c r="G9" s="17"/>
-      <c r="H9" s="15">
-        <v>0</v>
-      </c>
-      <c r="I9" s="16"/>
-      <c r="J9" s="16"/>
-      <c r="K9" s="17"/>
-      <c r="L9" s="15">
-        <v>0</v>
-      </c>
-      <c r="M9" s="16"/>
-      <c r="N9" s="16"/>
-      <c r="O9" s="17"/>
-      <c r="P9" s="15">
-        <v>0</v>
-      </c>
-      <c r="Q9" s="16"/>
-      <c r="R9" s="16"/>
-      <c r="S9" s="17"/>
-      <c r="T9" s="15">
-        <v>0</v>
-      </c>
-      <c r="U9" s="16"/>
-      <c r="V9" s="17"/>
-      <c r="W9" s="15">
-        <v>0</v>
-      </c>
-      <c r="X9" s="16"/>
-      <c r="Y9" s="17"/>
-      <c r="Z9" s="15"/>
-      <c r="AA9" s="17"/>
+      <c r="C9" s="14"/>
+      <c r="D9" s="15"/>
+      <c r="E9" s="15"/>
+      <c r="F9" s="15"/>
+      <c r="G9" s="16"/>
+      <c r="H9" s="14">
+        <v>0</v>
+      </c>
+      <c r="I9" s="15"/>
+      <c r="J9" s="15"/>
+      <c r="K9" s="16"/>
+      <c r="L9" s="14">
+        <v>0</v>
+      </c>
+      <c r="M9" s="15"/>
+      <c r="N9" s="15"/>
+      <c r="O9" s="16"/>
+      <c r="P9" s="14">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="15"/>
+      <c r="R9" s="15"/>
+      <c r="S9" s="16"/>
+      <c r="T9" s="14">
+        <v>0</v>
+      </c>
+      <c r="U9" s="15"/>
+      <c r="V9" s="16"/>
+      <c r="W9" s="14">
+        <v>0</v>
+      </c>
+      <c r="X9" s="15"/>
+      <c r="Y9" s="16"/>
+      <c r="Z9" s="14"/>
+      <c r="AA9" s="16"/>
     </row>
     <row r="10" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="3">
@@ -1279,41 +1333,41 @@
       <c r="B10" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="15"/>
-      <c r="D10" s="16"/>
-      <c r="E10" s="16"/>
-      <c r="F10" s="16"/>
-      <c r="G10" s="17"/>
-      <c r="H10" s="15">
-        <v>0</v>
-      </c>
-      <c r="I10" s="16"/>
-      <c r="J10" s="16"/>
-      <c r="K10" s="17"/>
-      <c r="L10" s="15">
-        <v>0</v>
-      </c>
-      <c r="M10" s="16"/>
-      <c r="N10" s="16"/>
-      <c r="O10" s="17"/>
-      <c r="P10" s="15">
-        <v>0</v>
-      </c>
-      <c r="Q10" s="16"/>
-      <c r="R10" s="16"/>
-      <c r="S10" s="17"/>
-      <c r="T10" s="15">
-        <v>0</v>
-      </c>
-      <c r="U10" s="16"/>
-      <c r="V10" s="17"/>
-      <c r="W10" s="15">
-        <v>0</v>
-      </c>
-      <c r="X10" s="16"/>
-      <c r="Y10" s="17"/>
-      <c r="Z10" s="15"/>
-      <c r="AA10" s="17"/>
+      <c r="C10" s="14"/>
+      <c r="D10" s="15"/>
+      <c r="E10" s="15"/>
+      <c r="F10" s="15"/>
+      <c r="G10" s="16"/>
+      <c r="H10" s="14">
+        <v>0</v>
+      </c>
+      <c r="I10" s="15"/>
+      <c r="J10" s="15"/>
+      <c r="K10" s="16"/>
+      <c r="L10" s="14">
+        <v>0</v>
+      </c>
+      <c r="M10" s="15"/>
+      <c r="N10" s="15"/>
+      <c r="O10" s="16"/>
+      <c r="P10" s="14">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="15"/>
+      <c r="R10" s="15"/>
+      <c r="S10" s="16"/>
+      <c r="T10" s="14">
+        <v>0</v>
+      </c>
+      <c r="U10" s="15"/>
+      <c r="V10" s="16"/>
+      <c r="W10" s="14">
+        <v>0</v>
+      </c>
+      <c r="X10" s="15"/>
+      <c r="Y10" s="16"/>
+      <c r="Z10" s="14"/>
+      <c r="AA10" s="16"/>
     </row>
     <row r="11" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="3">
@@ -1322,41 +1376,41 @@
       <c r="B11" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="15"/>
-      <c r="D11" s="16"/>
-      <c r="E11" s="16"/>
-      <c r="F11" s="16"/>
-      <c r="G11" s="17"/>
-      <c r="H11" s="15">
-        <v>0</v>
-      </c>
-      <c r="I11" s="16"/>
-      <c r="J11" s="16"/>
-      <c r="K11" s="17"/>
-      <c r="L11" s="15">
-        <v>0</v>
-      </c>
-      <c r="M11" s="16"/>
-      <c r="N11" s="16"/>
-      <c r="O11" s="17"/>
-      <c r="P11" s="15">
-        <v>0</v>
-      </c>
-      <c r="Q11" s="16"/>
-      <c r="R11" s="16"/>
-      <c r="S11" s="17"/>
-      <c r="T11" s="15">
-        <v>0</v>
-      </c>
-      <c r="U11" s="16"/>
-      <c r="V11" s="17"/>
-      <c r="W11" s="15">
-        <v>0</v>
-      </c>
-      <c r="X11" s="16"/>
-      <c r="Y11" s="17"/>
-      <c r="Z11" s="15"/>
-      <c r="AA11" s="17"/>
+      <c r="C11" s="14"/>
+      <c r="D11" s="15"/>
+      <c r="E11" s="15"/>
+      <c r="F11" s="15"/>
+      <c r="G11" s="16"/>
+      <c r="H11" s="14">
+        <v>0</v>
+      </c>
+      <c r="I11" s="15"/>
+      <c r="J11" s="15"/>
+      <c r="K11" s="16"/>
+      <c r="L11" s="14">
+        <v>0</v>
+      </c>
+      <c r="M11" s="15"/>
+      <c r="N11" s="15"/>
+      <c r="O11" s="16"/>
+      <c r="P11" s="14">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="15"/>
+      <c r="R11" s="15"/>
+      <c r="S11" s="16"/>
+      <c r="T11" s="14">
+        <v>0</v>
+      </c>
+      <c r="U11" s="15"/>
+      <c r="V11" s="16"/>
+      <c r="W11" s="14">
+        <v>0</v>
+      </c>
+      <c r="X11" s="15"/>
+      <c r="Y11" s="16"/>
+      <c r="Z11" s="14"/>
+      <c r="AA11" s="16"/>
     </row>
     <row r="12" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="3">
@@ -1365,41 +1419,41 @@
       <c r="B12" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="15"/>
-      <c r="D12" s="16"/>
-      <c r="E12" s="16"/>
-      <c r="F12" s="16"/>
-      <c r="G12" s="17"/>
-      <c r="H12" s="15">
-        <v>0</v>
-      </c>
-      <c r="I12" s="16"/>
-      <c r="J12" s="16"/>
-      <c r="K12" s="17"/>
-      <c r="L12" s="15">
-        <v>0</v>
-      </c>
-      <c r="M12" s="16"/>
-      <c r="N12" s="16"/>
-      <c r="O12" s="17"/>
-      <c r="P12" s="15">
-        <v>0</v>
-      </c>
-      <c r="Q12" s="16"/>
-      <c r="R12" s="16"/>
-      <c r="S12" s="17"/>
-      <c r="T12" s="15">
-        <v>0</v>
-      </c>
-      <c r="U12" s="16"/>
-      <c r="V12" s="17"/>
-      <c r="W12" s="15">
-        <v>0</v>
-      </c>
-      <c r="X12" s="16"/>
-      <c r="Y12" s="17"/>
-      <c r="Z12" s="15"/>
-      <c r="AA12" s="17"/>
+      <c r="C12" s="14"/>
+      <c r="D12" s="15"/>
+      <c r="E12" s="15"/>
+      <c r="F12" s="15"/>
+      <c r="G12" s="16"/>
+      <c r="H12" s="14">
+        <v>0</v>
+      </c>
+      <c r="I12" s="15"/>
+      <c r="J12" s="15"/>
+      <c r="K12" s="16"/>
+      <c r="L12" s="14">
+        <v>0</v>
+      </c>
+      <c r="M12" s="15"/>
+      <c r="N12" s="15"/>
+      <c r="O12" s="16"/>
+      <c r="P12" s="14">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="15"/>
+      <c r="R12" s="15"/>
+      <c r="S12" s="16"/>
+      <c r="T12" s="14">
+        <v>0</v>
+      </c>
+      <c r="U12" s="15"/>
+      <c r="V12" s="16"/>
+      <c r="W12" s="14">
+        <v>0</v>
+      </c>
+      <c r="X12" s="15"/>
+      <c r="Y12" s="16"/>
+      <c r="Z12" s="14"/>
+      <c r="AA12" s="16"/>
     </row>
     <row r="13" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="3">
@@ -1408,41 +1462,41 @@
       <c r="B13" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C13" s="15"/>
-      <c r="D13" s="16"/>
-      <c r="E13" s="16"/>
-      <c r="F13" s="16"/>
-      <c r="G13" s="17"/>
-      <c r="H13" s="15">
-        <v>0</v>
-      </c>
-      <c r="I13" s="16"/>
-      <c r="J13" s="16"/>
-      <c r="K13" s="17"/>
-      <c r="L13" s="15">
-        <v>0</v>
-      </c>
-      <c r="M13" s="16"/>
-      <c r="N13" s="16"/>
-      <c r="O13" s="17"/>
-      <c r="P13" s="15">
-        <v>0</v>
-      </c>
-      <c r="Q13" s="16"/>
-      <c r="R13" s="16"/>
-      <c r="S13" s="17"/>
-      <c r="T13" s="15">
-        <v>0</v>
-      </c>
-      <c r="U13" s="16"/>
-      <c r="V13" s="17"/>
-      <c r="W13" s="15">
-        <v>0</v>
-      </c>
-      <c r="X13" s="16"/>
-      <c r="Y13" s="17"/>
-      <c r="Z13" s="15"/>
-      <c r="AA13" s="17"/>
+      <c r="C13" s="14"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="15"/>
+      <c r="F13" s="15"/>
+      <c r="G13" s="16"/>
+      <c r="H13" s="14">
+        <v>0</v>
+      </c>
+      <c r="I13" s="15"/>
+      <c r="J13" s="15"/>
+      <c r="K13" s="16"/>
+      <c r="L13" s="14">
+        <v>0</v>
+      </c>
+      <c r="M13" s="15"/>
+      <c r="N13" s="15"/>
+      <c r="O13" s="16"/>
+      <c r="P13" s="14">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="15"/>
+      <c r="R13" s="15"/>
+      <c r="S13" s="16"/>
+      <c r="T13" s="14">
+        <v>0</v>
+      </c>
+      <c r="U13" s="15"/>
+      <c r="V13" s="16"/>
+      <c r="W13" s="14">
+        <v>0</v>
+      </c>
+      <c r="X13" s="15"/>
+      <c r="Y13" s="16"/>
+      <c r="Z13" s="14"/>
+      <c r="AA13" s="16"/>
     </row>
     <row r="14" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="3">
@@ -1451,41 +1505,41 @@
       <c r="B14" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="15"/>
-      <c r="D14" s="16"/>
-      <c r="E14" s="16"/>
-      <c r="F14" s="16"/>
-      <c r="G14" s="17"/>
-      <c r="H14" s="15">
-        <v>0</v>
-      </c>
-      <c r="I14" s="16"/>
-      <c r="J14" s="16"/>
-      <c r="K14" s="17"/>
-      <c r="L14" s="15">
-        <v>0</v>
-      </c>
-      <c r="M14" s="16"/>
-      <c r="N14" s="16"/>
-      <c r="O14" s="17"/>
-      <c r="P14" s="15">
-        <v>0</v>
-      </c>
-      <c r="Q14" s="16"/>
-      <c r="R14" s="16"/>
-      <c r="S14" s="17"/>
-      <c r="T14" s="15">
-        <v>0</v>
-      </c>
-      <c r="U14" s="16"/>
-      <c r="V14" s="17"/>
-      <c r="W14" s="15">
-        <v>0</v>
-      </c>
-      <c r="X14" s="16"/>
-      <c r="Y14" s="17"/>
-      <c r="Z14" s="15"/>
-      <c r="AA14" s="17"/>
+      <c r="C14" s="14"/>
+      <c r="D14" s="15"/>
+      <c r="E14" s="15"/>
+      <c r="F14" s="15"/>
+      <c r="G14" s="16"/>
+      <c r="H14" s="14">
+        <v>0</v>
+      </c>
+      <c r="I14" s="15"/>
+      <c r="J14" s="15"/>
+      <c r="K14" s="16"/>
+      <c r="L14" s="14">
+        <v>0</v>
+      </c>
+      <c r="M14" s="15"/>
+      <c r="N14" s="15"/>
+      <c r="O14" s="16"/>
+      <c r="P14" s="14">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="15"/>
+      <c r="R14" s="15"/>
+      <c r="S14" s="16"/>
+      <c r="T14" s="14">
+        <v>0</v>
+      </c>
+      <c r="U14" s="15"/>
+      <c r="V14" s="16"/>
+      <c r="W14" s="14">
+        <v>0</v>
+      </c>
+      <c r="X14" s="15"/>
+      <c r="Y14" s="16"/>
+      <c r="Z14" s="14"/>
+      <c r="AA14" s="16"/>
     </row>
     <row r="15" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="3">
@@ -1494,41 +1548,41 @@
       <c r="B15" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C15" s="15"/>
-      <c r="D15" s="16"/>
-      <c r="E15" s="16"/>
-      <c r="F15" s="16"/>
-      <c r="G15" s="17"/>
-      <c r="H15" s="15">
-        <v>0</v>
-      </c>
-      <c r="I15" s="16"/>
-      <c r="J15" s="16"/>
-      <c r="K15" s="17"/>
-      <c r="L15" s="15">
-        <v>0</v>
-      </c>
-      <c r="M15" s="16"/>
-      <c r="N15" s="16"/>
-      <c r="O15" s="17"/>
-      <c r="P15" s="15">
-        <v>0</v>
-      </c>
-      <c r="Q15" s="16"/>
-      <c r="R15" s="16"/>
-      <c r="S15" s="17"/>
-      <c r="T15" s="15">
-        <v>0</v>
-      </c>
-      <c r="U15" s="16"/>
-      <c r="V15" s="17"/>
-      <c r="W15" s="15">
-        <v>0</v>
-      </c>
-      <c r="X15" s="16"/>
-      <c r="Y15" s="17"/>
-      <c r="Z15" s="15"/>
-      <c r="AA15" s="17"/>
+      <c r="C15" s="14"/>
+      <c r="D15" s="15"/>
+      <c r="E15" s="15"/>
+      <c r="F15" s="15"/>
+      <c r="G15" s="16"/>
+      <c r="H15" s="14">
+        <v>0</v>
+      </c>
+      <c r="I15" s="15"/>
+      <c r="J15" s="15"/>
+      <c r="K15" s="16"/>
+      <c r="L15" s="14">
+        <v>0</v>
+      </c>
+      <c r="M15" s="15"/>
+      <c r="N15" s="15"/>
+      <c r="O15" s="16"/>
+      <c r="P15" s="14">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="15"/>
+      <c r="R15" s="15"/>
+      <c r="S15" s="16"/>
+      <c r="T15" s="14">
+        <v>0</v>
+      </c>
+      <c r="U15" s="15"/>
+      <c r="V15" s="16"/>
+      <c r="W15" s="14">
+        <v>0</v>
+      </c>
+      <c r="X15" s="15"/>
+      <c r="Y15" s="16"/>
+      <c r="Z15" s="14"/>
+      <c r="AA15" s="16"/>
     </row>
     <row r="16" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="3">
@@ -1537,41 +1591,41 @@
       <c r="B16" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C16" s="15"/>
-      <c r="D16" s="16"/>
-      <c r="E16" s="16"/>
-      <c r="F16" s="16"/>
-      <c r="G16" s="17"/>
-      <c r="H16" s="15">
-        <v>0</v>
-      </c>
-      <c r="I16" s="16"/>
-      <c r="J16" s="16"/>
-      <c r="K16" s="17"/>
-      <c r="L16" s="15">
-        <v>0</v>
-      </c>
-      <c r="M16" s="16"/>
-      <c r="N16" s="16"/>
-      <c r="O16" s="17"/>
-      <c r="P16" s="15">
-        <v>0</v>
-      </c>
-      <c r="Q16" s="16"/>
-      <c r="R16" s="16"/>
-      <c r="S16" s="17"/>
-      <c r="T16" s="15">
-        <v>0</v>
-      </c>
-      <c r="U16" s="16"/>
-      <c r="V16" s="17"/>
-      <c r="W16" s="15">
-        <v>0</v>
-      </c>
-      <c r="X16" s="16"/>
-      <c r="Y16" s="17"/>
-      <c r="Z16" s="15"/>
-      <c r="AA16" s="17"/>
+      <c r="C16" s="14"/>
+      <c r="D16" s="15"/>
+      <c r="E16" s="15"/>
+      <c r="F16" s="15"/>
+      <c r="G16" s="16"/>
+      <c r="H16" s="14">
+        <v>0</v>
+      </c>
+      <c r="I16" s="15"/>
+      <c r="J16" s="15"/>
+      <c r="K16" s="16"/>
+      <c r="L16" s="14">
+        <v>0</v>
+      </c>
+      <c r="M16" s="15"/>
+      <c r="N16" s="15"/>
+      <c r="O16" s="16"/>
+      <c r="P16" s="14">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="15"/>
+      <c r="R16" s="15"/>
+      <c r="S16" s="16"/>
+      <c r="T16" s="14">
+        <v>0</v>
+      </c>
+      <c r="U16" s="15"/>
+      <c r="V16" s="16"/>
+      <c r="W16" s="14">
+        <v>0</v>
+      </c>
+      <c r="X16" s="15"/>
+      <c r="Y16" s="16"/>
+      <c r="Z16" s="14"/>
+      <c r="AA16" s="16"/>
     </row>
     <row r="17" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="3">
@@ -1580,41 +1634,41 @@
       <c r="B17" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="15"/>
-      <c r="D17" s="16"/>
-      <c r="E17" s="16"/>
-      <c r="F17" s="16"/>
-      <c r="G17" s="17"/>
-      <c r="H17" s="15">
-        <v>0</v>
-      </c>
-      <c r="I17" s="16"/>
-      <c r="J17" s="16"/>
-      <c r="K17" s="17"/>
-      <c r="L17" s="15">
-        <v>0</v>
-      </c>
-      <c r="M17" s="16"/>
-      <c r="N17" s="16"/>
-      <c r="O17" s="17"/>
-      <c r="P17" s="15">
-        <v>0</v>
-      </c>
-      <c r="Q17" s="16"/>
-      <c r="R17" s="16"/>
-      <c r="S17" s="17"/>
-      <c r="T17" s="15">
-        <v>0</v>
-      </c>
-      <c r="U17" s="16"/>
-      <c r="V17" s="17"/>
-      <c r="W17" s="15">
-        <v>0</v>
-      </c>
-      <c r="X17" s="16"/>
-      <c r="Y17" s="17"/>
-      <c r="Z17" s="15"/>
-      <c r="AA17" s="17"/>
+      <c r="C17" s="14"/>
+      <c r="D17" s="15"/>
+      <c r="E17" s="15"/>
+      <c r="F17" s="15"/>
+      <c r="G17" s="16"/>
+      <c r="H17" s="14">
+        <v>0</v>
+      </c>
+      <c r="I17" s="15"/>
+      <c r="J17" s="15"/>
+      <c r="K17" s="16"/>
+      <c r="L17" s="14">
+        <v>0</v>
+      </c>
+      <c r="M17" s="15"/>
+      <c r="N17" s="15"/>
+      <c r="O17" s="16"/>
+      <c r="P17" s="14">
+        <v>0</v>
+      </c>
+      <c r="Q17" s="15"/>
+      <c r="R17" s="15"/>
+      <c r="S17" s="16"/>
+      <c r="T17" s="14">
+        <v>0</v>
+      </c>
+      <c r="U17" s="15"/>
+      <c r="V17" s="16"/>
+      <c r="W17" s="14">
+        <v>0</v>
+      </c>
+      <c r="X17" s="15"/>
+      <c r="Y17" s="16"/>
+      <c r="Z17" s="14"/>
+      <c r="AA17" s="16"/>
     </row>
     <row r="18" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="3">
@@ -1623,41 +1677,41 @@
       <c r="B18" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C18" s="15"/>
-      <c r="D18" s="16"/>
-      <c r="E18" s="16"/>
-      <c r="F18" s="16"/>
-      <c r="G18" s="17"/>
-      <c r="H18" s="15">
-        <v>0</v>
-      </c>
-      <c r="I18" s="16"/>
-      <c r="J18" s="16"/>
-      <c r="K18" s="17"/>
-      <c r="L18" s="15">
-        <v>0</v>
-      </c>
-      <c r="M18" s="16"/>
-      <c r="N18" s="16"/>
-      <c r="O18" s="17"/>
-      <c r="P18" s="15">
-        <v>0</v>
-      </c>
-      <c r="Q18" s="16"/>
-      <c r="R18" s="16"/>
-      <c r="S18" s="17"/>
-      <c r="T18" s="15">
-        <v>0</v>
-      </c>
-      <c r="U18" s="16"/>
-      <c r="V18" s="17"/>
-      <c r="W18" s="15">
-        <v>0</v>
-      </c>
-      <c r="X18" s="16"/>
-      <c r="Y18" s="17"/>
-      <c r="Z18" s="15"/>
-      <c r="AA18" s="17"/>
+      <c r="C18" s="14"/>
+      <c r="D18" s="15"/>
+      <c r="E18" s="15"/>
+      <c r="F18" s="15"/>
+      <c r="G18" s="16"/>
+      <c r="H18" s="14">
+        <v>0</v>
+      </c>
+      <c r="I18" s="15"/>
+      <c r="J18" s="15"/>
+      <c r="K18" s="16"/>
+      <c r="L18" s="14">
+        <v>0</v>
+      </c>
+      <c r="M18" s="15"/>
+      <c r="N18" s="15"/>
+      <c r="O18" s="16"/>
+      <c r="P18" s="14">
+        <v>0</v>
+      </c>
+      <c r="Q18" s="15"/>
+      <c r="R18" s="15"/>
+      <c r="S18" s="16"/>
+      <c r="T18" s="14">
+        <v>0</v>
+      </c>
+      <c r="U18" s="15"/>
+      <c r="V18" s="16"/>
+      <c r="W18" s="14">
+        <v>0</v>
+      </c>
+      <c r="X18" s="15"/>
+      <c r="Y18" s="16"/>
+      <c r="Z18" s="14"/>
+      <c r="AA18" s="16"/>
     </row>
     <row r="19" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="3">
@@ -1666,41 +1720,41 @@
       <c r="B19" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C19" s="15"/>
-      <c r="D19" s="16"/>
-      <c r="E19" s="16"/>
-      <c r="F19" s="16"/>
-      <c r="G19" s="17"/>
-      <c r="H19" s="15">
-        <v>0</v>
-      </c>
-      <c r="I19" s="16"/>
-      <c r="J19" s="16"/>
-      <c r="K19" s="17"/>
-      <c r="L19" s="15">
-        <v>0</v>
-      </c>
-      <c r="M19" s="16"/>
-      <c r="N19" s="16"/>
-      <c r="O19" s="17"/>
-      <c r="P19" s="15">
-        <v>0</v>
-      </c>
-      <c r="Q19" s="16"/>
-      <c r="R19" s="16"/>
-      <c r="S19" s="17"/>
-      <c r="T19" s="15">
-        <v>0</v>
-      </c>
-      <c r="U19" s="16"/>
-      <c r="V19" s="17"/>
-      <c r="W19" s="15">
-        <v>0</v>
-      </c>
-      <c r="X19" s="16"/>
-      <c r="Y19" s="17"/>
-      <c r="Z19" s="15"/>
-      <c r="AA19" s="17"/>
+      <c r="C19" s="14"/>
+      <c r="D19" s="15"/>
+      <c r="E19" s="15"/>
+      <c r="F19" s="15"/>
+      <c r="G19" s="16"/>
+      <c r="H19" s="14">
+        <v>0</v>
+      </c>
+      <c r="I19" s="15"/>
+      <c r="J19" s="15"/>
+      <c r="K19" s="16"/>
+      <c r="L19" s="14">
+        <v>0</v>
+      </c>
+      <c r="M19" s="15"/>
+      <c r="N19" s="15"/>
+      <c r="O19" s="16"/>
+      <c r="P19" s="14">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="15"/>
+      <c r="R19" s="15"/>
+      <c r="S19" s="16"/>
+      <c r="T19" s="14">
+        <v>0</v>
+      </c>
+      <c r="U19" s="15"/>
+      <c r="V19" s="16"/>
+      <c r="W19" s="14">
+        <v>0</v>
+      </c>
+      <c r="X19" s="15"/>
+      <c r="Y19" s="16"/>
+      <c r="Z19" s="14"/>
+      <c r="AA19" s="16"/>
     </row>
     <row r="20" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="3">
@@ -1709,41 +1763,41 @@
       <c r="B20" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C20" s="15"/>
-      <c r="D20" s="16"/>
-      <c r="E20" s="16"/>
-      <c r="F20" s="16"/>
-      <c r="G20" s="17"/>
-      <c r="H20" s="15">
-        <v>0</v>
-      </c>
-      <c r="I20" s="16"/>
-      <c r="J20" s="16"/>
-      <c r="K20" s="17"/>
-      <c r="L20" s="15">
-        <v>0</v>
-      </c>
-      <c r="M20" s="16"/>
-      <c r="N20" s="16"/>
-      <c r="O20" s="17"/>
-      <c r="P20" s="15">
-        <v>0</v>
-      </c>
-      <c r="Q20" s="16"/>
-      <c r="R20" s="16"/>
-      <c r="S20" s="17"/>
-      <c r="T20" s="15">
-        <v>0</v>
-      </c>
-      <c r="U20" s="16"/>
-      <c r="V20" s="17"/>
-      <c r="W20" s="15">
-        <v>0</v>
-      </c>
-      <c r="X20" s="16"/>
-      <c r="Y20" s="17"/>
-      <c r="Z20" s="15"/>
-      <c r="AA20" s="17"/>
+      <c r="C20" s="14"/>
+      <c r="D20" s="15"/>
+      <c r="E20" s="15"/>
+      <c r="F20" s="15"/>
+      <c r="G20" s="16"/>
+      <c r="H20" s="14">
+        <v>0</v>
+      </c>
+      <c r="I20" s="15"/>
+      <c r="J20" s="15"/>
+      <c r="K20" s="16"/>
+      <c r="L20" s="14">
+        <v>0</v>
+      </c>
+      <c r="M20" s="15"/>
+      <c r="N20" s="15"/>
+      <c r="O20" s="16"/>
+      <c r="P20" s="14">
+        <v>0</v>
+      </c>
+      <c r="Q20" s="15"/>
+      <c r="R20" s="15"/>
+      <c r="S20" s="16"/>
+      <c r="T20" s="14">
+        <v>0</v>
+      </c>
+      <c r="U20" s="15"/>
+      <c r="V20" s="16"/>
+      <c r="W20" s="14">
+        <v>0</v>
+      </c>
+      <c r="X20" s="15"/>
+      <c r="Y20" s="16"/>
+      <c r="Z20" s="14"/>
+      <c r="AA20" s="16"/>
     </row>
     <row r="21" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="3">
@@ -1752,41 +1806,41 @@
       <c r="B21" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C21" s="15"/>
-      <c r="D21" s="16"/>
-      <c r="E21" s="16"/>
-      <c r="F21" s="16"/>
-      <c r="G21" s="17"/>
-      <c r="H21" s="15">
-        <v>0</v>
-      </c>
-      <c r="I21" s="16"/>
-      <c r="J21" s="16"/>
-      <c r="K21" s="17"/>
-      <c r="L21" s="15">
-        <v>0</v>
-      </c>
-      <c r="M21" s="16"/>
-      <c r="N21" s="16"/>
-      <c r="O21" s="17"/>
-      <c r="P21" s="15">
-        <v>0</v>
-      </c>
-      <c r="Q21" s="16"/>
-      <c r="R21" s="16"/>
-      <c r="S21" s="17"/>
-      <c r="T21" s="15">
-        <v>0</v>
-      </c>
-      <c r="U21" s="16"/>
-      <c r="V21" s="17"/>
-      <c r="W21" s="15">
-        <v>0</v>
-      </c>
-      <c r="X21" s="16"/>
-      <c r="Y21" s="17"/>
-      <c r="Z21" s="15"/>
-      <c r="AA21" s="17"/>
+      <c r="C21" s="14"/>
+      <c r="D21" s="15"/>
+      <c r="E21" s="15"/>
+      <c r="F21" s="15"/>
+      <c r="G21" s="16"/>
+      <c r="H21" s="14">
+        <v>0</v>
+      </c>
+      <c r="I21" s="15"/>
+      <c r="J21" s="15"/>
+      <c r="K21" s="16"/>
+      <c r="L21" s="14">
+        <v>0</v>
+      </c>
+      <c r="M21" s="15"/>
+      <c r="N21" s="15"/>
+      <c r="O21" s="16"/>
+      <c r="P21" s="14">
+        <v>0</v>
+      </c>
+      <c r="Q21" s="15"/>
+      <c r="R21" s="15"/>
+      <c r="S21" s="16"/>
+      <c r="T21" s="14">
+        <v>0</v>
+      </c>
+      <c r="U21" s="15"/>
+      <c r="V21" s="16"/>
+      <c r="W21" s="14">
+        <v>0</v>
+      </c>
+      <c r="X21" s="15"/>
+      <c r="Y21" s="16"/>
+      <c r="Z21" s="14"/>
+      <c r="AA21" s="16"/>
     </row>
     <row r="22" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="3">
@@ -1795,41 +1849,41 @@
       <c r="B22" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C22" s="15"/>
-      <c r="D22" s="16"/>
-      <c r="E22" s="16"/>
-      <c r="F22" s="16"/>
-      <c r="G22" s="17"/>
-      <c r="H22" s="15">
-        <v>0</v>
-      </c>
-      <c r="I22" s="16"/>
-      <c r="J22" s="16"/>
-      <c r="K22" s="17"/>
-      <c r="L22" s="15">
-        <v>0</v>
-      </c>
-      <c r="M22" s="16"/>
-      <c r="N22" s="16"/>
-      <c r="O22" s="17"/>
-      <c r="P22" s="15">
-        <v>0</v>
-      </c>
-      <c r="Q22" s="16"/>
-      <c r="R22" s="16"/>
-      <c r="S22" s="17"/>
-      <c r="T22" s="15">
-        <v>0</v>
-      </c>
-      <c r="U22" s="16"/>
-      <c r="V22" s="17"/>
-      <c r="W22" s="15">
-        <v>0</v>
-      </c>
-      <c r="X22" s="16"/>
-      <c r="Y22" s="17"/>
-      <c r="Z22" s="15"/>
-      <c r="AA22" s="17"/>
+      <c r="C22" s="14"/>
+      <c r="D22" s="15"/>
+      <c r="E22" s="15"/>
+      <c r="F22" s="15"/>
+      <c r="G22" s="16"/>
+      <c r="H22" s="14">
+        <v>0</v>
+      </c>
+      <c r="I22" s="15"/>
+      <c r="J22" s="15"/>
+      <c r="K22" s="16"/>
+      <c r="L22" s="14">
+        <v>0</v>
+      </c>
+      <c r="M22" s="15"/>
+      <c r="N22" s="15"/>
+      <c r="O22" s="16"/>
+      <c r="P22" s="14">
+        <v>0</v>
+      </c>
+      <c r="Q22" s="15"/>
+      <c r="R22" s="15"/>
+      <c r="S22" s="16"/>
+      <c r="T22" s="14">
+        <v>0</v>
+      </c>
+      <c r="U22" s="15"/>
+      <c r="V22" s="16"/>
+      <c r="W22" s="14">
+        <v>0</v>
+      </c>
+      <c r="X22" s="15"/>
+      <c r="Y22" s="16"/>
+      <c r="Z22" s="14"/>
+      <c r="AA22" s="16"/>
     </row>
     <row r="23" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="3">
@@ -1838,41 +1892,41 @@
       <c r="B23" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C23" s="15"/>
-      <c r="D23" s="16"/>
-      <c r="E23" s="16"/>
-      <c r="F23" s="16"/>
-      <c r="G23" s="17"/>
-      <c r="H23" s="15">
-        <v>0</v>
-      </c>
-      <c r="I23" s="16"/>
-      <c r="J23" s="16"/>
-      <c r="K23" s="17"/>
-      <c r="L23" s="15">
-        <v>0</v>
-      </c>
-      <c r="M23" s="16"/>
-      <c r="N23" s="16"/>
-      <c r="O23" s="17"/>
-      <c r="P23" s="15">
-        <v>0</v>
-      </c>
-      <c r="Q23" s="16"/>
-      <c r="R23" s="16"/>
-      <c r="S23" s="17"/>
-      <c r="T23" s="15">
-        <v>0</v>
-      </c>
-      <c r="U23" s="16"/>
-      <c r="V23" s="17"/>
-      <c r="W23" s="15">
-        <v>0</v>
-      </c>
-      <c r="X23" s="16"/>
-      <c r="Y23" s="17"/>
-      <c r="Z23" s="15"/>
-      <c r="AA23" s="17"/>
+      <c r="C23" s="14"/>
+      <c r="D23" s="15"/>
+      <c r="E23" s="15"/>
+      <c r="F23" s="15"/>
+      <c r="G23" s="16"/>
+      <c r="H23" s="14">
+        <v>0</v>
+      </c>
+      <c r="I23" s="15"/>
+      <c r="J23" s="15"/>
+      <c r="K23" s="16"/>
+      <c r="L23" s="14">
+        <v>0</v>
+      </c>
+      <c r="M23" s="15"/>
+      <c r="N23" s="15"/>
+      <c r="O23" s="16"/>
+      <c r="P23" s="14">
+        <v>0</v>
+      </c>
+      <c r="Q23" s="15"/>
+      <c r="R23" s="15"/>
+      <c r="S23" s="16"/>
+      <c r="T23" s="14">
+        <v>0</v>
+      </c>
+      <c r="U23" s="15"/>
+      <c r="V23" s="16"/>
+      <c r="W23" s="14">
+        <v>0</v>
+      </c>
+      <c r="X23" s="15"/>
+      <c r="Y23" s="16"/>
+      <c r="Z23" s="14"/>
+      <c r="AA23" s="16"/>
     </row>
     <row r="24" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="3">
@@ -1881,41 +1935,41 @@
       <c r="B24" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C24" s="15"/>
-      <c r="D24" s="16"/>
-      <c r="E24" s="16"/>
-      <c r="F24" s="16"/>
-      <c r="G24" s="17"/>
-      <c r="H24" s="15">
-        <v>0</v>
-      </c>
-      <c r="I24" s="16"/>
-      <c r="J24" s="16"/>
-      <c r="K24" s="17"/>
-      <c r="L24" s="15">
-        <v>0</v>
-      </c>
-      <c r="M24" s="16"/>
-      <c r="N24" s="16"/>
-      <c r="O24" s="17"/>
-      <c r="P24" s="15">
-        <v>0</v>
-      </c>
-      <c r="Q24" s="16"/>
-      <c r="R24" s="16"/>
-      <c r="S24" s="17"/>
-      <c r="T24" s="15">
-        <v>0</v>
-      </c>
-      <c r="U24" s="16"/>
-      <c r="V24" s="17"/>
-      <c r="W24" s="15">
-        <v>0</v>
-      </c>
-      <c r="X24" s="16"/>
-      <c r="Y24" s="17"/>
-      <c r="Z24" s="15"/>
-      <c r="AA24" s="17"/>
+      <c r="C24" s="14"/>
+      <c r="D24" s="15"/>
+      <c r="E24" s="15"/>
+      <c r="F24" s="15"/>
+      <c r="G24" s="16"/>
+      <c r="H24" s="14">
+        <v>0</v>
+      </c>
+      <c r="I24" s="15"/>
+      <c r="J24" s="15"/>
+      <c r="K24" s="16"/>
+      <c r="L24" s="14">
+        <v>0</v>
+      </c>
+      <c r="M24" s="15"/>
+      <c r="N24" s="15"/>
+      <c r="O24" s="16"/>
+      <c r="P24" s="14">
+        <v>0</v>
+      </c>
+      <c r="Q24" s="15"/>
+      <c r="R24" s="15"/>
+      <c r="S24" s="16"/>
+      <c r="T24" s="14">
+        <v>0</v>
+      </c>
+      <c r="U24" s="15"/>
+      <c r="V24" s="16"/>
+      <c r="W24" s="14">
+        <v>0</v>
+      </c>
+      <c r="X24" s="15"/>
+      <c r="Y24" s="16"/>
+      <c r="Z24" s="14"/>
+      <c r="AA24" s="16"/>
     </row>
     <row r="25" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="3">
@@ -1924,72 +1978,72 @@
       <c r="B25" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C25" s="15"/>
-      <c r="D25" s="16"/>
-      <c r="E25" s="16"/>
-      <c r="F25" s="16"/>
-      <c r="G25" s="17"/>
-      <c r="H25" s="15">
-        <v>0</v>
-      </c>
-      <c r="I25" s="16"/>
-      <c r="J25" s="16"/>
-      <c r="K25" s="17"/>
-      <c r="L25" s="15">
-        <v>0</v>
-      </c>
-      <c r="M25" s="16"/>
-      <c r="N25" s="16"/>
-      <c r="O25" s="17"/>
-      <c r="P25" s="15">
-        <v>0</v>
-      </c>
-      <c r="Q25" s="16"/>
-      <c r="R25" s="16"/>
-      <c r="S25" s="17"/>
-      <c r="T25" s="15">
-        <v>0</v>
-      </c>
-      <c r="U25" s="16"/>
-      <c r="V25" s="17"/>
-      <c r="W25" s="15">
-        <v>0</v>
-      </c>
-      <c r="X25" s="16"/>
-      <c r="Y25" s="17"/>
-      <c r="Z25" s="15"/>
-      <c r="AA25" s="17"/>
+      <c r="C25" s="14"/>
+      <c r="D25" s="15"/>
+      <c r="E25" s="15"/>
+      <c r="F25" s="15"/>
+      <c r="G25" s="16"/>
+      <c r="H25" s="14">
+        <v>0</v>
+      </c>
+      <c r="I25" s="15"/>
+      <c r="J25" s="15"/>
+      <c r="K25" s="16"/>
+      <c r="L25" s="14">
+        <v>0</v>
+      </c>
+      <c r="M25" s="15"/>
+      <c r="N25" s="15"/>
+      <c r="O25" s="16"/>
+      <c r="P25" s="14">
+        <v>0</v>
+      </c>
+      <c r="Q25" s="15"/>
+      <c r="R25" s="15"/>
+      <c r="S25" s="16"/>
+      <c r="T25" s="14">
+        <v>0</v>
+      </c>
+      <c r="U25" s="15"/>
+      <c r="V25" s="16"/>
+      <c r="W25" s="14">
+        <v>0</v>
+      </c>
+      <c r="X25" s="15"/>
+      <c r="Y25" s="16"/>
+      <c r="Z25" s="14"/>
+      <c r="AA25" s="16"/>
     </row>
     <row r="26" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="12" t="s">
+      <c r="A26" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="B26" s="14"/>
-      <c r="C26" s="14"/>
-      <c r="D26" s="14"/>
-      <c r="E26" s="14"/>
-      <c r="F26" s="14"/>
-      <c r="G26" s="14"/>
-      <c r="H26" s="14"/>
-      <c r="I26" s="14"/>
-      <c r="J26" s="14"/>
-      <c r="K26" s="14"/>
-      <c r="L26" s="14"/>
-      <c r="M26" s="14"/>
-      <c r="N26" s="14"/>
-      <c r="O26" s="14"/>
-      <c r="P26" s="14"/>
-      <c r="Q26" s="14"/>
-      <c r="R26" s="14"/>
-      <c r="S26" s="14"/>
-      <c r="T26" s="14"/>
-      <c r="U26" s="14"/>
-      <c r="V26" s="14"/>
-      <c r="W26" s="14"/>
-      <c r="X26" s="14"/>
-      <c r="Y26" s="14"/>
-      <c r="Z26" s="14"/>
-      <c r="AA26" s="14"/>
+      <c r="B26" s="13"/>
+      <c r="C26" s="13"/>
+      <c r="D26" s="13"/>
+      <c r="E26" s="13"/>
+      <c r="F26" s="13"/>
+      <c r="G26" s="13"/>
+      <c r="H26" s="13"/>
+      <c r="I26" s="13"/>
+      <c r="J26" s="13"/>
+      <c r="K26" s="13"/>
+      <c r="L26" s="13"/>
+      <c r="M26" s="13"/>
+      <c r="N26" s="13"/>
+      <c r="O26" s="13"/>
+      <c r="P26" s="13"/>
+      <c r="Q26" s="13"/>
+      <c r="R26" s="13"/>
+      <c r="S26" s="13"/>
+      <c r="T26" s="13"/>
+      <c r="U26" s="13"/>
+      <c r="V26" s="13"/>
+      <c r="W26" s="13"/>
+      <c r="X26" s="13"/>
+      <c r="Y26" s="13"/>
+      <c r="Z26" s="13"/>
+      <c r="AA26" s="13"/>
     </row>
     <row r="27" spans="1:27" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="6" t="s">
@@ -2694,15 +2748,15 @@
       <c r="G44" s="9"/>
     </row>
     <row r="45" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A45" s="19" t="s">
+      <c r="A45" s="23" t="s">
         <v>84</v>
       </c>
-      <c r="B45" s="19"/>
-      <c r="C45" s="19"/>
-      <c r="D45" s="19"/>
-      <c r="E45" s="19"/>
-      <c r="F45" s="19"/>
-      <c r="G45" s="19"/>
+      <c r="B45" s="23"/>
+      <c r="C45" s="23"/>
+      <c r="D45" s="23"/>
+      <c r="E45" s="23"/>
+      <c r="F45" s="23"/>
+      <c r="G45" s="23"/>
       <c r="H45" s="11"/>
       <c r="I45" s="10" t="s">
         <v>79</v>
@@ -2715,165 +2769,339 @@
       <c r="O45" s="10"/>
       <c r="P45" s="10"/>
       <c r="Q45" s="10"/>
-      <c r="S45" s="19" t="s">
+      <c r="S45" s="23" t="s">
         <v>80</v>
       </c>
-      <c r="T45" s="14"/>
-      <c r="U45" s="14"/>
-      <c r="V45" s="14"/>
-      <c r="W45" s="14"/>
-      <c r="X45" s="14"/>
-      <c r="Y45" s="14"/>
-      <c r="Z45" s="14"/>
-      <c r="AA45" s="14"/>
+      <c r="T45" s="13"/>
+      <c r="U45" s="13"/>
+      <c r="V45" s="13"/>
+      <c r="W45" s="13"/>
+      <c r="X45" s="13"/>
+      <c r="Y45" s="13"/>
+      <c r="Z45" s="13"/>
+      <c r="AA45" s="13"/>
     </row>
     <row r="46" spans="1:27" ht="54" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A46" s="12">
+      <c r="A46" s="20">
         <v>1</v>
       </c>
-      <c r="B46" s="12"/>
-      <c r="C46" s="12"/>
-      <c r="D46" s="12"/>
-      <c r="E46" s="12"/>
-      <c r="F46" s="12"/>
-      <c r="G46" s="12"/>
-      <c r="I46" s="18">
+      <c r="B46" s="20"/>
+      <c r="C46" s="20"/>
+      <c r="D46" s="20"/>
+      <c r="E46" s="20"/>
+      <c r="F46" s="20"/>
+      <c r="G46" s="20"/>
+      <c r="I46" s="12">
         <v>1</v>
       </c>
-      <c r="J46" s="18"/>
-      <c r="K46" s="18"/>
-      <c r="L46" s="18"/>
-      <c r="M46" s="18"/>
-      <c r="N46" s="18"/>
-      <c r="O46" s="18"/>
-      <c r="P46" s="18"/>
-      <c r="Q46" s="18"/>
-      <c r="S46" s="18">
+      <c r="J46" s="12"/>
+      <c r="K46" s="12"/>
+      <c r="L46" s="12"/>
+      <c r="M46" s="12"/>
+      <c r="N46" s="12"/>
+      <c r="O46" s="12"/>
+      <c r="P46" s="12"/>
+      <c r="Q46" s="12"/>
+      <c r="S46" s="12">
         <v>1</v>
       </c>
-      <c r="T46" s="14"/>
-      <c r="U46" s="14"/>
-      <c r="V46" s="14"/>
-      <c r="W46" s="14"/>
-      <c r="X46" s="14"/>
-      <c r="Y46" s="14"/>
-      <c r="Z46" s="14"/>
-      <c r="AA46" s="14"/>
+      <c r="T46" s="13"/>
+      <c r="U46" s="13"/>
+      <c r="V46" s="13"/>
+      <c r="W46" s="13"/>
+      <c r="X46" s="13"/>
+      <c r="Y46" s="13"/>
+      <c r="Z46" s="13"/>
+      <c r="AA46" s="13"/>
     </row>
     <row r="47" spans="1:27" ht="54" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A47" s="12">
+      <c r="A47" s="20">
         <v>2</v>
       </c>
-      <c r="B47" s="12"/>
-      <c r="C47" s="12"/>
-      <c r="D47" s="12"/>
-      <c r="E47" s="12"/>
-      <c r="F47" s="12"/>
-      <c r="G47" s="12"/>
-      <c r="I47" s="18" t="s">
+      <c r="B47" s="20"/>
+      <c r="C47" s="20"/>
+      <c r="D47" s="20"/>
+      <c r="E47" s="20"/>
+      <c r="F47" s="20"/>
+      <c r="G47" s="20"/>
+      <c r="I47" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="J47" s="18"/>
-      <c r="K47" s="18"/>
-      <c r="L47" s="18"/>
-      <c r="M47" s="18"/>
-      <c r="N47" s="18"/>
-      <c r="O47" s="18"/>
-      <c r="P47" s="18"/>
-      <c r="Q47" s="18"/>
-      <c r="S47" s="18" t="s">
+      <c r="J47" s="12"/>
+      <c r="K47" s="12"/>
+      <c r="L47" s="12"/>
+      <c r="M47" s="12"/>
+      <c r="N47" s="12"/>
+      <c r="O47" s="12"/>
+      <c r="P47" s="12"/>
+      <c r="Q47" s="12"/>
+      <c r="S47" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="T47" s="14"/>
-      <c r="U47" s="14"/>
-      <c r="V47" s="14"/>
-      <c r="W47" s="14"/>
-      <c r="X47" s="14"/>
-      <c r="Y47" s="14"/>
-      <c r="Z47" s="14"/>
-      <c r="AA47" s="14"/>
+      <c r="T47" s="13"/>
+      <c r="U47" s="13"/>
+      <c r="V47" s="13"/>
+      <c r="W47" s="13"/>
+      <c r="X47" s="13"/>
+      <c r="Y47" s="13"/>
+      <c r="Z47" s="13"/>
+      <c r="AA47" s="13"/>
     </row>
     <row r="48" spans="1:27" ht="54" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A48" s="12">
+      <c r="A48" s="20">
         <v>3</v>
       </c>
-      <c r="B48" s="12"/>
-      <c r="C48" s="12"/>
-      <c r="D48" s="12"/>
-      <c r="E48" s="12"/>
-      <c r="F48" s="12"/>
-      <c r="G48" s="12"/>
-      <c r="I48" s="18" t="s">
+      <c r="B48" s="20"/>
+      <c r="C48" s="20"/>
+      <c r="D48" s="20"/>
+      <c r="E48" s="20"/>
+      <c r="F48" s="20"/>
+      <c r="G48" s="20"/>
+      <c r="I48" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="J48" s="18"/>
-      <c r="K48" s="18"/>
-      <c r="L48" s="18"/>
-      <c r="M48" s="18"/>
-      <c r="N48" s="18"/>
-      <c r="O48" s="18"/>
-      <c r="P48" s="18"/>
-      <c r="Q48" s="18"/>
-      <c r="S48" s="18" t="s">
+      <c r="J48" s="12"/>
+      <c r="K48" s="12"/>
+      <c r="L48" s="12"/>
+      <c r="M48" s="12"/>
+      <c r="N48" s="12"/>
+      <c r="O48" s="12"/>
+      <c r="P48" s="12"/>
+      <c r="Q48" s="12"/>
+      <c r="S48" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="T48" s="14"/>
-      <c r="U48" s="14"/>
-      <c r="V48" s="14"/>
-      <c r="W48" s="14"/>
-      <c r="X48" s="14"/>
-      <c r="Y48" s="14"/>
-      <c r="Z48" s="14"/>
-      <c r="AA48" s="14"/>
+      <c r="T48" s="13"/>
+      <c r="U48" s="13"/>
+      <c r="V48" s="13"/>
+      <c r="W48" s="13"/>
+      <c r="X48" s="13"/>
+      <c r="Y48" s="13"/>
+      <c r="Z48" s="13"/>
+      <c r="AA48" s="13"/>
     </row>
     <row r="49" spans="1:27" ht="50" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A49" s="12">
+      <c r="A49" s="20">
         <v>4</v>
       </c>
-      <c r="B49" s="12"/>
-      <c r="C49" s="12"/>
-      <c r="D49" s="12"/>
-      <c r="E49" s="12"/>
-      <c r="F49" s="12"/>
-      <c r="G49" s="12"/>
-      <c r="I49" s="18" t="s">
+      <c r="B49" s="20"/>
+      <c r="C49" s="20"/>
+      <c r="D49" s="20"/>
+      <c r="E49" s="20"/>
+      <c r="F49" s="20"/>
+      <c r="G49" s="20"/>
+      <c r="I49" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="J49" s="18"/>
-      <c r="K49" s="18"/>
-      <c r="L49" s="18"/>
-      <c r="M49" s="18"/>
-      <c r="N49" s="18"/>
-      <c r="O49" s="18"/>
-      <c r="P49" s="18"/>
-      <c r="Q49" s="18"/>
-      <c r="S49" s="18" t="s">
+      <c r="J49" s="12"/>
+      <c r="K49" s="12"/>
+      <c r="L49" s="12"/>
+      <c r="M49" s="12"/>
+      <c r="N49" s="12"/>
+      <c r="O49" s="12"/>
+      <c r="P49" s="12"/>
+      <c r="Q49" s="12"/>
+      <c r="S49" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="T49" s="14"/>
-      <c r="U49" s="14"/>
-      <c r="V49" s="14"/>
-      <c r="W49" s="14"/>
-      <c r="X49" s="14"/>
-      <c r="Y49" s="14"/>
-      <c r="Z49" s="14"/>
-      <c r="AA49" s="14"/>
+      <c r="T49" s="13"/>
+      <c r="U49" s="13"/>
+      <c r="V49" s="13"/>
+      <c r="W49" s="13"/>
+      <c r="X49" s="13"/>
+      <c r="Y49" s="13"/>
+      <c r="Z49" s="13"/>
+      <c r="AA49" s="13"/>
     </row>
     <row r="50" spans="1:27" ht="25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="51" spans="1:27" ht="49.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A51" s="28" t="s">
+        <v>90</v>
+      </c>
+      <c r="B51" s="29"/>
+      <c r="C51" s="29"/>
+      <c r="D51" s="29"/>
+      <c r="E51" s="29"/>
+      <c r="F51" s="29"/>
+      <c r="G51" s="29"/>
+    </row>
+    <row r="52" spans="1:27" ht="62.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A52" s="30" t="s">
+        <v>91</v>
+      </c>
+      <c r="B52" s="20"/>
+      <c r="C52" s="20"/>
+      <c r="D52" s="20"/>
+      <c r="E52" s="20"/>
+      <c r="F52" s="20"/>
+      <c r="G52" s="20"/>
+    </row>
+    <row r="53" spans="1:27" ht="53.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A53" s="30" t="s">
+        <v>92</v>
+      </c>
+      <c r="B53" s="20"/>
+      <c r="C53" s="20"/>
+      <c r="D53" s="20"/>
+      <c r="E53" s="20"/>
+      <c r="F53" s="20"/>
+      <c r="G53" s="20"/>
+    </row>
+    <row r="54" spans="1:27" ht="53.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A54" s="30" t="s">
+        <v>93</v>
+      </c>
+      <c r="B54" s="20"/>
+      <c r="C54" s="20"/>
+      <c r="D54" s="20"/>
+      <c r="E54" s="20"/>
+      <c r="F54" s="20"/>
+      <c r="G54" s="20"/>
+    </row>
+    <row r="55" spans="1:27" ht="53.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A55" s="30" t="s">
+        <v>94</v>
+      </c>
+      <c r="B55" s="20"/>
+      <c r="C55" s="20"/>
+      <c r="D55" s="20"/>
+      <c r="E55" s="20"/>
+      <c r="F55" s="20"/>
+      <c r="G55" s="20"/>
+    </row>
   </sheetData>
-  <mergeCells count="162">
-    <mergeCell ref="S49:AA49"/>
-    <mergeCell ref="W16:Y16"/>
-    <mergeCell ref="I46:Q46"/>
-    <mergeCell ref="S46:AA46"/>
-    <mergeCell ref="Z15:AA15"/>
-    <mergeCell ref="Z24:AA24"/>
-    <mergeCell ref="P10:S10"/>
-    <mergeCell ref="H10:K10"/>
-    <mergeCell ref="P25:S25"/>
-    <mergeCell ref="Z12:AA12"/>
-    <mergeCell ref="T19:V19"/>
-    <mergeCell ref="H25:K25"/>
+  <mergeCells count="167">
+    <mergeCell ref="A51:G51"/>
+    <mergeCell ref="A52:G52"/>
+    <mergeCell ref="A53:G53"/>
+    <mergeCell ref="A54:G54"/>
+    <mergeCell ref="A55:G55"/>
+    <mergeCell ref="A3:AA3"/>
+    <mergeCell ref="P14:S14"/>
+    <mergeCell ref="H20:K20"/>
+    <mergeCell ref="I48:Q48"/>
+    <mergeCell ref="S45:AA45"/>
+    <mergeCell ref="W17:Y17"/>
+    <mergeCell ref="A5:AA5"/>
+    <mergeCell ref="W11:Y11"/>
+    <mergeCell ref="L13:O13"/>
+    <mergeCell ref="W19:Y19"/>
+    <mergeCell ref="H6:K6"/>
+    <mergeCell ref="P21:S21"/>
+    <mergeCell ref="H21:K21"/>
+    <mergeCell ref="P8:S8"/>
+    <mergeCell ref="C8:G8"/>
+    <mergeCell ref="L15:O15"/>
+    <mergeCell ref="T15:V15"/>
+    <mergeCell ref="C17:G17"/>
+    <mergeCell ref="T24:V24"/>
+    <mergeCell ref="W25:Y25"/>
+    <mergeCell ref="L23:O23"/>
+    <mergeCell ref="P23:S23"/>
+    <mergeCell ref="Z10:AA10"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="W6:Y6"/>
+    <mergeCell ref="L8:O8"/>
+    <mergeCell ref="Z20:AA20"/>
+    <mergeCell ref="W15:Y15"/>
+    <mergeCell ref="I49:Q49"/>
+    <mergeCell ref="P17:S17"/>
+    <mergeCell ref="H16:K16"/>
+    <mergeCell ref="L10:O10"/>
+    <mergeCell ref="C13:G13"/>
+    <mergeCell ref="L25:O25"/>
+    <mergeCell ref="T25:V25"/>
+    <mergeCell ref="H22:K22"/>
+    <mergeCell ref="P19:S19"/>
+    <mergeCell ref="Z6:AA6"/>
+    <mergeCell ref="L9:O9"/>
+    <mergeCell ref="C6:G6"/>
+    <mergeCell ref="T9:V9"/>
+    <mergeCell ref="C15:G15"/>
+    <mergeCell ref="P12:S12"/>
+    <mergeCell ref="C16:G16"/>
+    <mergeCell ref="T23:V23"/>
+    <mergeCell ref="C25:G25"/>
+    <mergeCell ref="A49:G49"/>
+    <mergeCell ref="L7:O7"/>
+    <mergeCell ref="T7:V7"/>
+    <mergeCell ref="C9:G9"/>
+    <mergeCell ref="T16:V16"/>
+    <mergeCell ref="C11:G11"/>
+    <mergeCell ref="T18:V18"/>
+    <mergeCell ref="L24:O24"/>
+    <mergeCell ref="L18:O18"/>
+    <mergeCell ref="L11:O11"/>
+    <mergeCell ref="T11:V11"/>
+    <mergeCell ref="C19:G19"/>
+    <mergeCell ref="P7:S7"/>
+    <mergeCell ref="H7:K7"/>
+    <mergeCell ref="P16:S16"/>
+    <mergeCell ref="T10:V10"/>
+    <mergeCell ref="W4:AA4"/>
+    <mergeCell ref="H19:K19"/>
+    <mergeCell ref="I47:Q47"/>
+    <mergeCell ref="L22:O22"/>
+    <mergeCell ref="P13:S13"/>
+    <mergeCell ref="C24:G24"/>
+    <mergeCell ref="H12:K12"/>
+    <mergeCell ref="L6:O6"/>
+    <mergeCell ref="T12:V12"/>
+    <mergeCell ref="T21:V21"/>
+    <mergeCell ref="P15:S15"/>
+    <mergeCell ref="H14:K14"/>
+    <mergeCell ref="Z7:AA7"/>
+    <mergeCell ref="Z16:AA16"/>
+    <mergeCell ref="C10:G10"/>
+    <mergeCell ref="Z18:AA18"/>
+    <mergeCell ref="Z8:AA8"/>
+    <mergeCell ref="W14:Y14"/>
+    <mergeCell ref="Z17:AA17"/>
+    <mergeCell ref="W23:Y23"/>
+    <mergeCell ref="W13:Y13"/>
+    <mergeCell ref="Z9:AA9"/>
+    <mergeCell ref="A46:G46"/>
+    <mergeCell ref="T13:V13"/>
+    <mergeCell ref="A47:G47"/>
+    <mergeCell ref="Z14:AA14"/>
+    <mergeCell ref="P11:S11"/>
+    <mergeCell ref="W10:Y10"/>
+    <mergeCell ref="W24:Y24"/>
+    <mergeCell ref="H17:K17"/>
+    <mergeCell ref="H11:K11"/>
+    <mergeCell ref="L20:O20"/>
+    <mergeCell ref="A48:G48"/>
+    <mergeCell ref="L17:O17"/>
+    <mergeCell ref="Z23:AA23"/>
+    <mergeCell ref="C23:G23"/>
+    <mergeCell ref="S47:AA47"/>
+    <mergeCell ref="H24:K24"/>
+    <mergeCell ref="A45:G45"/>
+    <mergeCell ref="Z19:AA19"/>
+    <mergeCell ref="H4:V4"/>
+    <mergeCell ref="C18:G18"/>
+    <mergeCell ref="S48:AA48"/>
+    <mergeCell ref="W20:Y20"/>
+    <mergeCell ref="H13:K13"/>
+    <mergeCell ref="L21:O21"/>
+    <mergeCell ref="W22:Y22"/>
+    <mergeCell ref="H15:K15"/>
+    <mergeCell ref="P24:S24"/>
+    <mergeCell ref="H23:K23"/>
+    <mergeCell ref="H18:K18"/>
+    <mergeCell ref="W12:Y12"/>
+    <mergeCell ref="W21:Y21"/>
+    <mergeCell ref="A26:AA26"/>
+    <mergeCell ref="Z25:AA25"/>
+    <mergeCell ref="C20:G20"/>
+    <mergeCell ref="H8:K8"/>
+    <mergeCell ref="W9:Y9"/>
+    <mergeCell ref="T8:V8"/>
+    <mergeCell ref="T17:V17"/>
+    <mergeCell ref="L16:O16"/>
+    <mergeCell ref="Z22:AA22"/>
+    <mergeCell ref="C22:G22"/>
+    <mergeCell ref="C4:G4"/>
     <mergeCell ref="A2:AA2"/>
     <mergeCell ref="T22:V22"/>
     <mergeCell ref="W18:Y18"/>
@@ -2898,135 +3126,22 @@
     <mergeCell ref="W7:Y7"/>
     <mergeCell ref="C12:G12"/>
     <mergeCell ref="P9:S9"/>
-    <mergeCell ref="H4:V4"/>
-    <mergeCell ref="C18:G18"/>
-    <mergeCell ref="S48:AA48"/>
-    <mergeCell ref="W20:Y20"/>
-    <mergeCell ref="H13:K13"/>
-    <mergeCell ref="L21:O21"/>
-    <mergeCell ref="W22:Y22"/>
-    <mergeCell ref="H15:K15"/>
-    <mergeCell ref="P24:S24"/>
-    <mergeCell ref="H23:K23"/>
-    <mergeCell ref="H18:K18"/>
-    <mergeCell ref="W12:Y12"/>
-    <mergeCell ref="W21:Y21"/>
-    <mergeCell ref="A26:AA26"/>
-    <mergeCell ref="Z25:AA25"/>
-    <mergeCell ref="C20:G20"/>
-    <mergeCell ref="H8:K8"/>
-    <mergeCell ref="W9:Y9"/>
-    <mergeCell ref="T8:V8"/>
-    <mergeCell ref="T17:V17"/>
-    <mergeCell ref="L16:O16"/>
-    <mergeCell ref="Z22:AA22"/>
-    <mergeCell ref="C22:G22"/>
-    <mergeCell ref="C4:G4"/>
-    <mergeCell ref="A47:G47"/>
-    <mergeCell ref="Z14:AA14"/>
-    <mergeCell ref="P11:S11"/>
-    <mergeCell ref="W10:Y10"/>
-    <mergeCell ref="W24:Y24"/>
-    <mergeCell ref="H17:K17"/>
-    <mergeCell ref="H11:K11"/>
-    <mergeCell ref="L20:O20"/>
-    <mergeCell ref="A48:G48"/>
-    <mergeCell ref="L17:O17"/>
-    <mergeCell ref="Z23:AA23"/>
-    <mergeCell ref="C23:G23"/>
-    <mergeCell ref="S47:AA47"/>
-    <mergeCell ref="H24:K24"/>
-    <mergeCell ref="A45:G45"/>
-    <mergeCell ref="W4:AA4"/>
-    <mergeCell ref="H19:K19"/>
-    <mergeCell ref="I47:Q47"/>
-    <mergeCell ref="L22:O22"/>
-    <mergeCell ref="P13:S13"/>
-    <mergeCell ref="C24:G24"/>
-    <mergeCell ref="H12:K12"/>
-    <mergeCell ref="L6:O6"/>
-    <mergeCell ref="T12:V12"/>
-    <mergeCell ref="T21:V21"/>
-    <mergeCell ref="P15:S15"/>
-    <mergeCell ref="H14:K14"/>
-    <mergeCell ref="Z7:AA7"/>
-    <mergeCell ref="Z16:AA16"/>
-    <mergeCell ref="C10:G10"/>
-    <mergeCell ref="Z18:AA18"/>
-    <mergeCell ref="Z8:AA8"/>
-    <mergeCell ref="W14:Y14"/>
-    <mergeCell ref="Z17:AA17"/>
-    <mergeCell ref="W23:Y23"/>
-    <mergeCell ref="W13:Y13"/>
-    <mergeCell ref="Z9:AA9"/>
-    <mergeCell ref="A46:G46"/>
-    <mergeCell ref="T13:V13"/>
-    <mergeCell ref="L7:O7"/>
-    <mergeCell ref="T7:V7"/>
-    <mergeCell ref="C9:G9"/>
-    <mergeCell ref="T16:V16"/>
-    <mergeCell ref="C11:G11"/>
-    <mergeCell ref="T18:V18"/>
-    <mergeCell ref="L24:O24"/>
-    <mergeCell ref="L18:O18"/>
-    <mergeCell ref="L11:O11"/>
-    <mergeCell ref="T11:V11"/>
-    <mergeCell ref="C19:G19"/>
-    <mergeCell ref="P7:S7"/>
-    <mergeCell ref="H7:K7"/>
-    <mergeCell ref="P16:S16"/>
-    <mergeCell ref="T10:V10"/>
-    <mergeCell ref="Z19:AA19"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="W6:Y6"/>
-    <mergeCell ref="L8:O8"/>
-    <mergeCell ref="Z20:AA20"/>
-    <mergeCell ref="W15:Y15"/>
-    <mergeCell ref="I49:Q49"/>
-    <mergeCell ref="P17:S17"/>
-    <mergeCell ref="H16:K16"/>
-    <mergeCell ref="L10:O10"/>
-    <mergeCell ref="C13:G13"/>
-    <mergeCell ref="L25:O25"/>
-    <mergeCell ref="T25:V25"/>
-    <mergeCell ref="H22:K22"/>
-    <mergeCell ref="P19:S19"/>
-    <mergeCell ref="Z6:AA6"/>
-    <mergeCell ref="L9:O9"/>
-    <mergeCell ref="C6:G6"/>
-    <mergeCell ref="T9:V9"/>
-    <mergeCell ref="C15:G15"/>
-    <mergeCell ref="P12:S12"/>
-    <mergeCell ref="C16:G16"/>
-    <mergeCell ref="T23:V23"/>
-    <mergeCell ref="C25:G25"/>
-    <mergeCell ref="A49:G49"/>
-    <mergeCell ref="A3:AA3"/>
-    <mergeCell ref="P14:S14"/>
-    <mergeCell ref="H20:K20"/>
-    <mergeCell ref="I48:Q48"/>
-    <mergeCell ref="S45:AA45"/>
-    <mergeCell ref="W17:Y17"/>
-    <mergeCell ref="A5:AA5"/>
-    <mergeCell ref="W11:Y11"/>
-    <mergeCell ref="L13:O13"/>
-    <mergeCell ref="W19:Y19"/>
-    <mergeCell ref="H6:K6"/>
-    <mergeCell ref="P21:S21"/>
-    <mergeCell ref="H21:K21"/>
-    <mergeCell ref="P8:S8"/>
-    <mergeCell ref="C8:G8"/>
-    <mergeCell ref="L15:O15"/>
-    <mergeCell ref="T15:V15"/>
-    <mergeCell ref="C17:G17"/>
-    <mergeCell ref="T24:V24"/>
-    <mergeCell ref="W25:Y25"/>
-    <mergeCell ref="L23:O23"/>
-    <mergeCell ref="P23:S23"/>
-    <mergeCell ref="Z10:AA10"/>
+    <mergeCell ref="S49:AA49"/>
+    <mergeCell ref="W16:Y16"/>
+    <mergeCell ref="I46:Q46"/>
+    <mergeCell ref="S46:AA46"/>
+    <mergeCell ref="Z15:AA15"/>
+    <mergeCell ref="Z24:AA24"/>
+    <mergeCell ref="P10:S10"/>
+    <mergeCell ref="H10:K10"/>
+    <mergeCell ref="P25:S25"/>
+    <mergeCell ref="Z12:AA12"/>
+    <mergeCell ref="T19:V19"/>
+    <mergeCell ref="H25:K25"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" r:id="rId1"/>
   <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Support flexible final summaries and automatic No Compromise
</commit_message>
<xml_diff>
--- a/templates/template_general.xlsx
+++ b/templates/template_general.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Bot\Market_Survey\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1B045FC-0648-4A64-95F5-ECCA58BAA02B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17DE714E-5136-4BC6-BB1D-8C740B8F473A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="94">
   <si>
     <t>Market Improvement Report</t>
   </si>
@@ -274,12 +274,6 @@
     <t>Hitech 1500mL</t>
   </si>
   <si>
-    <t>Key Issues</t>
-  </si>
-  <si>
-    <t>INITIATIVE IDEA / SUGGESTION</t>
-  </si>
-  <si>
     <t>2.</t>
   </si>
   <si>
@@ -289,9 +283,6 @@
     <t>4.</t>
   </si>
   <si>
-    <t>ចំណុចដួល</t>
-  </si>
-  <si>
     <t>Location of Visit:</t>
   </si>
   <si>
@@ -310,25 +301,29 @@
     <t>No Compromise</t>
   </si>
   <si>
-    <t>1.Mass Products មិនត្រូវឲ្យខ្វះស្លកក្នុងផ្ទះមួយ
-(CBL/Wurkz/Exprez/Dazz/Water/Sport PET 500ml/Ize PET 500ml)</t>
-  </si>
-  <si>
-    <t>2.ផលិតផលហួសដឺឡេ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3. ការបញ្ចូលរបាយការណ៍លក់មិនត្រឹមត្រូវ
-</t>
-  </si>
-  <si>
     <t>4. របាយការណ៍លក់ជូនអតិថិជនមិនពិត (ទាំងចំនួនលក់ និងតម្លៃ)។</t>
+  </si>
+  <si>
+    <t>បញ្ហាទីផ្សារ</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> បញ្ហាត្រូវដោះស្រាយ</t>
+  </si>
+  <si>
+    <t>1.Mass Products មិនត្រូវឲ្យខ្វះស្លកក្នុងផ្ទះមួយ(CBL/Wurkz/Exprez/Dazz/Water/Sport PET 500ml/Ize PET 500ml)</t>
+  </si>
+  <si>
+    <t>2.ផលិតផលហួសការកំណត់</t>
+  </si>
+  <si>
+    <t>3. ការបញ្ចូលរបាយការណ៍លក់មិនត្រឹមត្រូវ</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -403,7 +398,14 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="20"/>
+      <sz val="18"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -548,14 +550,17 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -563,41 +568,40 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -731,6 +735,189 @@
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{95199885-0DDC-586F-4B36-11B1346C57DC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="1047750" cy="1047750"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>6350</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Image 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F4978D84-8A64-D7B4-F157-6A10E3767AF3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="1047750" cy="1047750"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>6350</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 2" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1F87ED97-C3A1-E2C8-2CA7-4111409C6EC9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="1047750" cy="1047750"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>6350</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1027" name="Picture 3" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6C034566-D112-44CE-AE72-A84C420E2B15}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -991,11 +1178,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AA55"/>
+  <dimension ref="A1:AA50"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -1021,134 +1208,134 @@
       <c r="D1" s="5"/>
     </row>
     <row r="2" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="17" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
-      <c r="G2" s="13"/>
-      <c r="H2" s="13"/>
-      <c r="I2" s="13"/>
-      <c r="J2" s="13"/>
-      <c r="K2" s="13"/>
-      <c r="L2" s="13"/>
-      <c r="M2" s="13"/>
-      <c r="N2" s="13"/>
-      <c r="O2" s="13"/>
-      <c r="P2" s="13"/>
-      <c r="Q2" s="13"/>
-      <c r="R2" s="13"/>
-      <c r="S2" s="13"/>
-      <c r="T2" s="13"/>
-      <c r="U2" s="13"/>
-      <c r="V2" s="13"/>
-      <c r="W2" s="13"/>
-      <c r="X2" s="13"/>
-      <c r="Y2" s="13"/>
-      <c r="Z2" s="13"/>
-      <c r="AA2" s="13"/>
+      <c r="A2" s="27" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
+      <c r="I2" s="14"/>
+      <c r="J2" s="14"/>
+      <c r="K2" s="14"/>
+      <c r="L2" s="14"/>
+      <c r="M2" s="14"/>
+      <c r="N2" s="14"/>
+      <c r="O2" s="14"/>
+      <c r="P2" s="14"/>
+      <c r="Q2" s="14"/>
+      <c r="R2" s="14"/>
+      <c r="S2" s="14"/>
+      <c r="T2" s="14"/>
+      <c r="U2" s="14"/>
+      <c r="V2" s="14"/>
+      <c r="W2" s="14"/>
+      <c r="X2" s="14"/>
+      <c r="Y2" s="14"/>
+      <c r="Z2" s="14"/>
+      <c r="AA2" s="14"/>
     </row>
     <row r="3" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="26" t="s">
-        <v>89</v>
-      </c>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="13"/>
-      <c r="G3" s="13"/>
-      <c r="H3" s="13"/>
-      <c r="I3" s="13"/>
-      <c r="J3" s="13"/>
-      <c r="K3" s="13"/>
-      <c r="L3" s="13"/>
-      <c r="M3" s="13"/>
-      <c r="N3" s="13"/>
-      <c r="O3" s="13"/>
-      <c r="P3" s="13"/>
-      <c r="Q3" s="13"/>
-      <c r="R3" s="13"/>
-      <c r="S3" s="13"/>
-      <c r="T3" s="13"/>
-      <c r="U3" s="13"/>
-      <c r="V3" s="13"/>
-      <c r="W3" s="13"/>
-      <c r="X3" s="13"/>
-      <c r="Y3" s="13"/>
-      <c r="Z3" s="13"/>
-      <c r="AA3" s="13"/>
+      <c r="A3" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
+      <c r="H3" s="14"/>
+      <c r="I3" s="14"/>
+      <c r="J3" s="14"/>
+      <c r="K3" s="14"/>
+      <c r="L3" s="14"/>
+      <c r="M3" s="14"/>
+      <c r="N3" s="14"/>
+      <c r="O3" s="14"/>
+      <c r="P3" s="14"/>
+      <c r="Q3" s="14"/>
+      <c r="R3" s="14"/>
+      <c r="S3" s="14"/>
+      <c r="T3" s="14"/>
+      <c r="U3" s="14"/>
+      <c r="V3" s="14"/>
+      <c r="W3" s="14"/>
+      <c r="X3" s="14"/>
+      <c r="Y3" s="14"/>
+      <c r="Z3" s="14"/>
+      <c r="AA3" s="14"/>
     </row>
     <row r="4" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A4" s="22" t="s">
-        <v>86</v>
-      </c>
-      <c r="B4" s="16"/>
+        <v>83</v>
+      </c>
+      <c r="B4" s="17"/>
       <c r="C4" s="22" t="s">
-        <v>87</v>
-      </c>
-      <c r="D4" s="15"/>
-      <c r="E4" s="15"/>
-      <c r="F4" s="15"/>
-      <c r="G4" s="16"/>
-      <c r="H4" s="19" t="s">
+        <v>84</v>
+      </c>
+      <c r="D4" s="16"/>
+      <c r="E4" s="16"/>
+      <c r="F4" s="16"/>
+      <c r="G4" s="17"/>
+      <c r="H4" s="25" t="s">
+        <v>82</v>
+      </c>
+      <c r="I4" s="16"/>
+      <c r="J4" s="16"/>
+      <c r="K4" s="16"/>
+      <c r="L4" s="16"/>
+      <c r="M4" s="16"/>
+      <c r="N4" s="16"/>
+      <c r="O4" s="16"/>
+      <c r="P4" s="16"/>
+      <c r="Q4" s="16"/>
+      <c r="R4" s="16"/>
+      <c r="S4" s="16"/>
+      <c r="T4" s="16"/>
+      <c r="U4" s="16"/>
+      <c r="V4" s="17"/>
+      <c r="W4" s="22" t="s">
         <v>85</v>
       </c>
-      <c r="I4" s="15"/>
-      <c r="J4" s="15"/>
-      <c r="K4" s="15"/>
-      <c r="L4" s="15"/>
-      <c r="M4" s="15"/>
-      <c r="N4" s="15"/>
-      <c r="O4" s="15"/>
-      <c r="P4" s="15"/>
-      <c r="Q4" s="15"/>
-      <c r="R4" s="15"/>
-      <c r="S4" s="15"/>
-      <c r="T4" s="15"/>
-      <c r="U4" s="15"/>
-      <c r="V4" s="16"/>
-      <c r="W4" s="22" t="s">
-        <v>88</v>
-      </c>
-      <c r="X4" s="15"/>
-      <c r="Y4" s="15"/>
-      <c r="Z4" s="15"/>
-      <c r="AA4" s="16"/>
+      <c r="X4" s="16"/>
+      <c r="Y4" s="16"/>
+      <c r="Z4" s="16"/>
+      <c r="AA4" s="17"/>
     </row>
     <row r="5" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="27" t="s">
+      <c r="A5" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="15"/>
-      <c r="C5" s="15"/>
-      <c r="D5" s="15"/>
-      <c r="E5" s="15"/>
-      <c r="F5" s="15"/>
-      <c r="G5" s="15"/>
-      <c r="H5" s="15"/>
-      <c r="I5" s="15"/>
-      <c r="J5" s="15"/>
-      <c r="K5" s="15"/>
-      <c r="L5" s="15"/>
-      <c r="M5" s="15"/>
-      <c r="N5" s="15"/>
-      <c r="O5" s="15"/>
-      <c r="P5" s="15"/>
-      <c r="Q5" s="15"/>
-      <c r="R5" s="15"/>
-      <c r="S5" s="15"/>
-      <c r="T5" s="15"/>
-      <c r="U5" s="15"/>
-      <c r="V5" s="15"/>
-      <c r="W5" s="15"/>
-      <c r="X5" s="15"/>
-      <c r="Y5" s="15"/>
-      <c r="Z5" s="15"/>
-      <c r="AA5" s="16"/>
+      <c r="B5" s="16"/>
+      <c r="C5" s="16"/>
+      <c r="D5" s="16"/>
+      <c r="E5" s="16"/>
+      <c r="F5" s="16"/>
+      <c r="G5" s="16"/>
+      <c r="H5" s="16"/>
+      <c r="I5" s="16"/>
+      <c r="J5" s="16"/>
+      <c r="K5" s="16"/>
+      <c r="L5" s="16"/>
+      <c r="M5" s="16"/>
+      <c r="N5" s="16"/>
+      <c r="O5" s="16"/>
+      <c r="P5" s="16"/>
+      <c r="Q5" s="16"/>
+      <c r="R5" s="16"/>
+      <c r="S5" s="16"/>
+      <c r="T5" s="16"/>
+      <c r="U5" s="16"/>
+      <c r="V5" s="16"/>
+      <c r="W5" s="16"/>
+      <c r="X5" s="16"/>
+      <c r="Y5" s="16"/>
+      <c r="Z5" s="16"/>
+      <c r="AA5" s="17"/>
     </row>
     <row r="6" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
@@ -1157,45 +1344,45 @@
       <c r="B6" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="25" t="s">
+      <c r="C6" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="D6" s="15"/>
-      <c r="E6" s="15"/>
-      <c r="F6" s="15"/>
-      <c r="G6" s="16"/>
-      <c r="H6" s="18" t="s">
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="16"/>
+      <c r="G6" s="17"/>
+      <c r="H6" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="I6" s="15"/>
-      <c r="J6" s="15"/>
-      <c r="K6" s="16"/>
-      <c r="L6" s="18" t="s">
+      <c r="I6" s="16"/>
+      <c r="J6" s="16"/>
+      <c r="K6" s="17"/>
+      <c r="L6" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="M6" s="15"/>
-      <c r="N6" s="15"/>
-      <c r="O6" s="16"/>
-      <c r="P6" s="18" t="s">
+      <c r="M6" s="16"/>
+      <c r="N6" s="16"/>
+      <c r="O6" s="17"/>
+      <c r="P6" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="Q6" s="15"/>
-      <c r="R6" s="15"/>
-      <c r="S6" s="16"/>
-      <c r="T6" s="18" t="s">
+      <c r="Q6" s="16"/>
+      <c r="R6" s="16"/>
+      <c r="S6" s="17"/>
+      <c r="T6" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="U6" s="15"/>
-      <c r="V6" s="16"/>
-      <c r="W6" s="24" t="s">
+      <c r="U6" s="16"/>
+      <c r="V6" s="17"/>
+      <c r="W6" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="X6" s="15"/>
-      <c r="Y6" s="16"/>
-      <c r="Z6" s="24" t="s">
+      <c r="X6" s="16"/>
+      <c r="Y6" s="17"/>
+      <c r="Z6" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="AA6" s="16"/>
+      <c r="AA6" s="17"/>
     </row>
     <row r="7" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="3">
@@ -1204,41 +1391,41 @@
       <c r="B7" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="14"/>
-      <c r="D7" s="15"/>
-      <c r="E7" s="15"/>
-      <c r="F7" s="15"/>
-      <c r="G7" s="16"/>
-      <c r="H7" s="14">
-        <v>0</v>
-      </c>
-      <c r="I7" s="15"/>
-      <c r="J7" s="15"/>
-      <c r="K7" s="16"/>
-      <c r="L7" s="14">
-        <v>0</v>
-      </c>
-      <c r="M7" s="15"/>
-      <c r="N7" s="15"/>
-      <c r="O7" s="16"/>
-      <c r="P7" s="14">
-        <v>0</v>
-      </c>
-      <c r="Q7" s="15"/>
-      <c r="R7" s="15"/>
-      <c r="S7" s="16"/>
-      <c r="T7" s="14">
-        <v>0</v>
-      </c>
-      <c r="U7" s="15"/>
-      <c r="V7" s="16"/>
-      <c r="W7" s="14">
-        <v>0</v>
-      </c>
-      <c r="X7" s="15"/>
-      <c r="Y7" s="16"/>
-      <c r="Z7" s="14"/>
-      <c r="AA7" s="16"/>
+      <c r="C7" s="15"/>
+      <c r="D7" s="16"/>
+      <c r="E7" s="16"/>
+      <c r="F7" s="16"/>
+      <c r="G7" s="17"/>
+      <c r="H7" s="15">
+        <v>0</v>
+      </c>
+      <c r="I7" s="16"/>
+      <c r="J7" s="16"/>
+      <c r="K7" s="17"/>
+      <c r="L7" s="15">
+        <v>0</v>
+      </c>
+      <c r="M7" s="16"/>
+      <c r="N7" s="16"/>
+      <c r="O7" s="17"/>
+      <c r="P7" s="15">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="16"/>
+      <c r="R7" s="16"/>
+      <c r="S7" s="17"/>
+      <c r="T7" s="15">
+        <v>0</v>
+      </c>
+      <c r="U7" s="16"/>
+      <c r="V7" s="17"/>
+      <c r="W7" s="15">
+        <v>0</v>
+      </c>
+      <c r="X7" s="16"/>
+      <c r="Y7" s="17"/>
+      <c r="Z7" s="15"/>
+      <c r="AA7" s="17"/>
     </row>
     <row r="8" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="3">
@@ -1247,41 +1434,41 @@
       <c r="B8" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="14"/>
-      <c r="D8" s="15"/>
-      <c r="E8" s="15"/>
-      <c r="F8" s="15"/>
-      <c r="G8" s="16"/>
-      <c r="H8" s="14">
-        <v>0</v>
-      </c>
-      <c r="I8" s="15"/>
-      <c r="J8" s="15"/>
-      <c r="K8" s="16"/>
-      <c r="L8" s="14">
-        <v>0</v>
-      </c>
-      <c r="M8" s="15"/>
-      <c r="N8" s="15"/>
-      <c r="O8" s="16"/>
-      <c r="P8" s="14">
-        <v>0</v>
-      </c>
-      <c r="Q8" s="15"/>
-      <c r="R8" s="15"/>
-      <c r="S8" s="16"/>
-      <c r="T8" s="21">
-        <v>0</v>
-      </c>
-      <c r="U8" s="15"/>
-      <c r="V8" s="16"/>
-      <c r="W8" s="14">
-        <v>0</v>
-      </c>
-      <c r="X8" s="15"/>
-      <c r="Y8" s="16"/>
-      <c r="Z8" s="14"/>
-      <c r="AA8" s="16"/>
+      <c r="C8" s="15"/>
+      <c r="D8" s="16"/>
+      <c r="E8" s="16"/>
+      <c r="F8" s="16"/>
+      <c r="G8" s="17"/>
+      <c r="H8" s="15">
+        <v>0</v>
+      </c>
+      <c r="I8" s="16"/>
+      <c r="J8" s="16"/>
+      <c r="K8" s="17"/>
+      <c r="L8" s="15">
+        <v>0</v>
+      </c>
+      <c r="M8" s="16"/>
+      <c r="N8" s="16"/>
+      <c r="O8" s="17"/>
+      <c r="P8" s="15">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="16"/>
+      <c r="R8" s="16"/>
+      <c r="S8" s="17"/>
+      <c r="T8" s="26">
+        <v>0</v>
+      </c>
+      <c r="U8" s="16"/>
+      <c r="V8" s="17"/>
+      <c r="W8" s="15">
+        <v>0</v>
+      </c>
+      <c r="X8" s="16"/>
+      <c r="Y8" s="17"/>
+      <c r="Z8" s="15"/>
+      <c r="AA8" s="17"/>
     </row>
     <row r="9" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="3">
@@ -1290,41 +1477,41 @@
       <c r="B9" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="14"/>
-      <c r="D9" s="15"/>
-      <c r="E9" s="15"/>
-      <c r="F9" s="15"/>
-      <c r="G9" s="16"/>
-      <c r="H9" s="14">
-        <v>0</v>
-      </c>
-      <c r="I9" s="15"/>
-      <c r="J9" s="15"/>
-      <c r="K9" s="16"/>
-      <c r="L9" s="14">
-        <v>0</v>
-      </c>
-      <c r="M9" s="15"/>
-      <c r="N9" s="15"/>
-      <c r="O9" s="16"/>
-      <c r="P9" s="14">
-        <v>0</v>
-      </c>
-      <c r="Q9" s="15"/>
-      <c r="R9" s="15"/>
-      <c r="S9" s="16"/>
-      <c r="T9" s="14">
-        <v>0</v>
-      </c>
-      <c r="U9" s="15"/>
-      <c r="V9" s="16"/>
-      <c r="W9" s="14">
-        <v>0</v>
-      </c>
-      <c r="X9" s="15"/>
-      <c r="Y9" s="16"/>
-      <c r="Z9" s="14"/>
-      <c r="AA9" s="16"/>
+      <c r="C9" s="15"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="16"/>
+      <c r="F9" s="16"/>
+      <c r="G9" s="17"/>
+      <c r="H9" s="15">
+        <v>0</v>
+      </c>
+      <c r="I9" s="16"/>
+      <c r="J9" s="16"/>
+      <c r="K9" s="17"/>
+      <c r="L9" s="15">
+        <v>0</v>
+      </c>
+      <c r="M9" s="16"/>
+      <c r="N9" s="16"/>
+      <c r="O9" s="17"/>
+      <c r="P9" s="15">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="16"/>
+      <c r="R9" s="16"/>
+      <c r="S9" s="17"/>
+      <c r="T9" s="15">
+        <v>0</v>
+      </c>
+      <c r="U9" s="16"/>
+      <c r="V9" s="17"/>
+      <c r="W9" s="15">
+        <v>0</v>
+      </c>
+      <c r="X9" s="16"/>
+      <c r="Y9" s="17"/>
+      <c r="Z9" s="15"/>
+      <c r="AA9" s="17"/>
     </row>
     <row r="10" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="3">
@@ -1333,41 +1520,41 @@
       <c r="B10" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="14"/>
-      <c r="D10" s="15"/>
-      <c r="E10" s="15"/>
-      <c r="F10" s="15"/>
-      <c r="G10" s="16"/>
-      <c r="H10" s="14">
-        <v>0</v>
-      </c>
-      <c r="I10" s="15"/>
-      <c r="J10" s="15"/>
-      <c r="K10" s="16"/>
-      <c r="L10" s="14">
-        <v>0</v>
-      </c>
-      <c r="M10" s="15"/>
-      <c r="N10" s="15"/>
-      <c r="O10" s="16"/>
-      <c r="P10" s="14">
-        <v>0</v>
-      </c>
-      <c r="Q10" s="15"/>
-      <c r="R10" s="15"/>
-      <c r="S10" s="16"/>
-      <c r="T10" s="14">
-        <v>0</v>
-      </c>
-      <c r="U10" s="15"/>
-      <c r="V10" s="16"/>
-      <c r="W10" s="14">
-        <v>0</v>
-      </c>
-      <c r="X10" s="15"/>
-      <c r="Y10" s="16"/>
-      <c r="Z10" s="14"/>
-      <c r="AA10" s="16"/>
+      <c r="C10" s="15"/>
+      <c r="D10" s="16"/>
+      <c r="E10" s="16"/>
+      <c r="F10" s="16"/>
+      <c r="G10" s="17"/>
+      <c r="H10" s="15">
+        <v>0</v>
+      </c>
+      <c r="I10" s="16"/>
+      <c r="J10" s="16"/>
+      <c r="K10" s="17"/>
+      <c r="L10" s="15">
+        <v>0</v>
+      </c>
+      <c r="M10" s="16"/>
+      <c r="N10" s="16"/>
+      <c r="O10" s="17"/>
+      <c r="P10" s="15">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="16"/>
+      <c r="R10" s="16"/>
+      <c r="S10" s="17"/>
+      <c r="T10" s="15">
+        <v>0</v>
+      </c>
+      <c r="U10" s="16"/>
+      <c r="V10" s="17"/>
+      <c r="W10" s="15">
+        <v>0</v>
+      </c>
+      <c r="X10" s="16"/>
+      <c r="Y10" s="17"/>
+      <c r="Z10" s="15"/>
+      <c r="AA10" s="17"/>
     </row>
     <row r="11" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="3">
@@ -1376,41 +1563,41 @@
       <c r="B11" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="14"/>
-      <c r="D11" s="15"/>
-      <c r="E11" s="15"/>
-      <c r="F11" s="15"/>
-      <c r="G11" s="16"/>
-      <c r="H11" s="14">
-        <v>0</v>
-      </c>
-      <c r="I11" s="15"/>
-      <c r="J11" s="15"/>
-      <c r="K11" s="16"/>
-      <c r="L11" s="14">
-        <v>0</v>
-      </c>
-      <c r="M11" s="15"/>
-      <c r="N11" s="15"/>
-      <c r="O11" s="16"/>
-      <c r="P11" s="14">
-        <v>0</v>
-      </c>
-      <c r="Q11" s="15"/>
-      <c r="R11" s="15"/>
-      <c r="S11" s="16"/>
-      <c r="T11" s="14">
-        <v>0</v>
-      </c>
-      <c r="U11" s="15"/>
-      <c r="V11" s="16"/>
-      <c r="W11" s="14">
-        <v>0</v>
-      </c>
-      <c r="X11" s="15"/>
-      <c r="Y11" s="16"/>
-      <c r="Z11" s="14"/>
-      <c r="AA11" s="16"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="16"/>
+      <c r="E11" s="16"/>
+      <c r="F11" s="16"/>
+      <c r="G11" s="17"/>
+      <c r="H11" s="15">
+        <v>0</v>
+      </c>
+      <c r="I11" s="16"/>
+      <c r="J11" s="16"/>
+      <c r="K11" s="17"/>
+      <c r="L11" s="15">
+        <v>0</v>
+      </c>
+      <c r="M11" s="16"/>
+      <c r="N11" s="16"/>
+      <c r="O11" s="17"/>
+      <c r="P11" s="15">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="16"/>
+      <c r="R11" s="16"/>
+      <c r="S11" s="17"/>
+      <c r="T11" s="15">
+        <v>0</v>
+      </c>
+      <c r="U11" s="16"/>
+      <c r="V11" s="17"/>
+      <c r="W11" s="15">
+        <v>0</v>
+      </c>
+      <c r="X11" s="16"/>
+      <c r="Y11" s="17"/>
+      <c r="Z11" s="15"/>
+      <c r="AA11" s="17"/>
     </row>
     <row r="12" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="3">
@@ -1419,41 +1606,41 @@
       <c r="B12" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="14"/>
-      <c r="D12" s="15"/>
-      <c r="E12" s="15"/>
-      <c r="F12" s="15"/>
-      <c r="G12" s="16"/>
-      <c r="H12" s="14">
-        <v>0</v>
-      </c>
-      <c r="I12" s="15"/>
-      <c r="J12" s="15"/>
-      <c r="K12" s="16"/>
-      <c r="L12" s="14">
-        <v>0</v>
-      </c>
-      <c r="M12" s="15"/>
-      <c r="N12" s="15"/>
-      <c r="O12" s="16"/>
-      <c r="P12" s="14">
-        <v>0</v>
-      </c>
-      <c r="Q12" s="15"/>
-      <c r="R12" s="15"/>
-      <c r="S12" s="16"/>
-      <c r="T12" s="14">
-        <v>0</v>
-      </c>
-      <c r="U12" s="15"/>
-      <c r="V12" s="16"/>
-      <c r="W12" s="14">
-        <v>0</v>
-      </c>
-      <c r="X12" s="15"/>
-      <c r="Y12" s="16"/>
-      <c r="Z12" s="14"/>
-      <c r="AA12" s="16"/>
+      <c r="C12" s="15"/>
+      <c r="D12" s="16"/>
+      <c r="E12" s="16"/>
+      <c r="F12" s="16"/>
+      <c r="G12" s="17"/>
+      <c r="H12" s="15">
+        <v>0</v>
+      </c>
+      <c r="I12" s="16"/>
+      <c r="J12" s="16"/>
+      <c r="K12" s="17"/>
+      <c r="L12" s="15">
+        <v>0</v>
+      </c>
+      <c r="M12" s="16"/>
+      <c r="N12" s="16"/>
+      <c r="O12" s="17"/>
+      <c r="P12" s="15">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="16"/>
+      <c r="R12" s="16"/>
+      <c r="S12" s="17"/>
+      <c r="T12" s="15">
+        <v>0</v>
+      </c>
+      <c r="U12" s="16"/>
+      <c r="V12" s="17"/>
+      <c r="W12" s="15">
+        <v>0</v>
+      </c>
+      <c r="X12" s="16"/>
+      <c r="Y12" s="17"/>
+      <c r="Z12" s="15"/>
+      <c r="AA12" s="17"/>
     </row>
     <row r="13" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="3">
@@ -1462,41 +1649,41 @@
       <c r="B13" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C13" s="14"/>
-      <c r="D13" s="15"/>
-      <c r="E13" s="15"/>
-      <c r="F13" s="15"/>
-      <c r="G13" s="16"/>
-      <c r="H13" s="14">
-        <v>0</v>
-      </c>
-      <c r="I13" s="15"/>
-      <c r="J13" s="15"/>
-      <c r="K13" s="16"/>
-      <c r="L13" s="14">
-        <v>0</v>
-      </c>
-      <c r="M13" s="15"/>
-      <c r="N13" s="15"/>
-      <c r="O13" s="16"/>
-      <c r="P13" s="14">
-        <v>0</v>
-      </c>
-      <c r="Q13" s="15"/>
-      <c r="R13" s="15"/>
-      <c r="S13" s="16"/>
-      <c r="T13" s="14">
-        <v>0</v>
-      </c>
-      <c r="U13" s="15"/>
-      <c r="V13" s="16"/>
-      <c r="W13" s="14">
-        <v>0</v>
-      </c>
-      <c r="X13" s="15"/>
-      <c r="Y13" s="16"/>
-      <c r="Z13" s="14"/>
-      <c r="AA13" s="16"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="16"/>
+      <c r="E13" s="16"/>
+      <c r="F13" s="16"/>
+      <c r="G13" s="17"/>
+      <c r="H13" s="15">
+        <v>0</v>
+      </c>
+      <c r="I13" s="16"/>
+      <c r="J13" s="16"/>
+      <c r="K13" s="17"/>
+      <c r="L13" s="15">
+        <v>0</v>
+      </c>
+      <c r="M13" s="16"/>
+      <c r="N13" s="16"/>
+      <c r="O13" s="17"/>
+      <c r="P13" s="15">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="16"/>
+      <c r="R13" s="16"/>
+      <c r="S13" s="17"/>
+      <c r="T13" s="15">
+        <v>0</v>
+      </c>
+      <c r="U13" s="16"/>
+      <c r="V13" s="17"/>
+      <c r="W13" s="15">
+        <v>0</v>
+      </c>
+      <c r="X13" s="16"/>
+      <c r="Y13" s="17"/>
+      <c r="Z13" s="15"/>
+      <c r="AA13" s="17"/>
     </row>
     <row r="14" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="3">
@@ -1505,41 +1692,41 @@
       <c r="B14" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="14"/>
-      <c r="D14" s="15"/>
-      <c r="E14" s="15"/>
-      <c r="F14" s="15"/>
-      <c r="G14" s="16"/>
-      <c r="H14" s="14">
-        <v>0</v>
-      </c>
-      <c r="I14" s="15"/>
-      <c r="J14" s="15"/>
-      <c r="K14" s="16"/>
-      <c r="L14" s="14">
-        <v>0</v>
-      </c>
-      <c r="M14" s="15"/>
-      <c r="N14" s="15"/>
-      <c r="O14" s="16"/>
-      <c r="P14" s="14">
-        <v>0</v>
-      </c>
-      <c r="Q14" s="15"/>
-      <c r="R14" s="15"/>
-      <c r="S14" s="16"/>
-      <c r="T14" s="14">
-        <v>0</v>
-      </c>
-      <c r="U14" s="15"/>
-      <c r="V14" s="16"/>
-      <c r="W14" s="14">
-        <v>0</v>
-      </c>
-      <c r="X14" s="15"/>
-      <c r="Y14" s="16"/>
-      <c r="Z14" s="14"/>
-      <c r="AA14" s="16"/>
+      <c r="C14" s="15"/>
+      <c r="D14" s="16"/>
+      <c r="E14" s="16"/>
+      <c r="F14" s="16"/>
+      <c r="G14" s="17"/>
+      <c r="H14" s="15">
+        <v>0</v>
+      </c>
+      <c r="I14" s="16"/>
+      <c r="J14" s="16"/>
+      <c r="K14" s="17"/>
+      <c r="L14" s="15">
+        <v>0</v>
+      </c>
+      <c r="M14" s="16"/>
+      <c r="N14" s="16"/>
+      <c r="O14" s="17"/>
+      <c r="P14" s="15">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="16"/>
+      <c r="R14" s="16"/>
+      <c r="S14" s="17"/>
+      <c r="T14" s="15">
+        <v>0</v>
+      </c>
+      <c r="U14" s="16"/>
+      <c r="V14" s="17"/>
+      <c r="W14" s="15">
+        <v>0</v>
+      </c>
+      <c r="X14" s="16"/>
+      <c r="Y14" s="17"/>
+      <c r="Z14" s="15"/>
+      <c r="AA14" s="17"/>
     </row>
     <row r="15" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="3">
@@ -1548,41 +1735,41 @@
       <c r="B15" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C15" s="14"/>
-      <c r="D15" s="15"/>
-      <c r="E15" s="15"/>
-      <c r="F15" s="15"/>
-      <c r="G15" s="16"/>
-      <c r="H15" s="14">
-        <v>0</v>
-      </c>
-      <c r="I15" s="15"/>
-      <c r="J15" s="15"/>
-      <c r="K15" s="16"/>
-      <c r="L15" s="14">
-        <v>0</v>
-      </c>
-      <c r="M15" s="15"/>
-      <c r="N15" s="15"/>
-      <c r="O15" s="16"/>
-      <c r="P15" s="14">
-        <v>0</v>
-      </c>
-      <c r="Q15" s="15"/>
-      <c r="R15" s="15"/>
-      <c r="S15" s="16"/>
-      <c r="T15" s="14">
-        <v>0</v>
-      </c>
-      <c r="U15" s="15"/>
-      <c r="V15" s="16"/>
-      <c r="W15" s="14">
-        <v>0</v>
-      </c>
-      <c r="X15" s="15"/>
-      <c r="Y15" s="16"/>
-      <c r="Z15" s="14"/>
-      <c r="AA15" s="16"/>
+      <c r="C15" s="15"/>
+      <c r="D15" s="16"/>
+      <c r="E15" s="16"/>
+      <c r="F15" s="16"/>
+      <c r="G15" s="17"/>
+      <c r="H15" s="15">
+        <v>0</v>
+      </c>
+      <c r="I15" s="16"/>
+      <c r="J15" s="16"/>
+      <c r="K15" s="17"/>
+      <c r="L15" s="15">
+        <v>0</v>
+      </c>
+      <c r="M15" s="16"/>
+      <c r="N15" s="16"/>
+      <c r="O15" s="17"/>
+      <c r="P15" s="15">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="16"/>
+      <c r="R15" s="16"/>
+      <c r="S15" s="17"/>
+      <c r="T15" s="15">
+        <v>0</v>
+      </c>
+      <c r="U15" s="16"/>
+      <c r="V15" s="17"/>
+      <c r="W15" s="15">
+        <v>0</v>
+      </c>
+      <c r="X15" s="16"/>
+      <c r="Y15" s="17"/>
+      <c r="Z15" s="15"/>
+      <c r="AA15" s="17"/>
     </row>
     <row r="16" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="3">
@@ -1591,41 +1778,41 @@
       <c r="B16" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C16" s="14"/>
-      <c r="D16" s="15"/>
-      <c r="E16" s="15"/>
-      <c r="F16" s="15"/>
-      <c r="G16" s="16"/>
-      <c r="H16" s="14">
-        <v>0</v>
-      </c>
-      <c r="I16" s="15"/>
-      <c r="J16" s="15"/>
-      <c r="K16" s="16"/>
-      <c r="L16" s="14">
-        <v>0</v>
-      </c>
-      <c r="M16" s="15"/>
-      <c r="N16" s="15"/>
-      <c r="O16" s="16"/>
-      <c r="P16" s="14">
-        <v>0</v>
-      </c>
-      <c r="Q16" s="15"/>
-      <c r="R16" s="15"/>
-      <c r="S16" s="16"/>
-      <c r="T16" s="14">
-        <v>0</v>
-      </c>
-      <c r="U16" s="15"/>
-      <c r="V16" s="16"/>
-      <c r="W16" s="14">
-        <v>0</v>
-      </c>
-      <c r="X16" s="15"/>
-      <c r="Y16" s="16"/>
-      <c r="Z16" s="14"/>
-      <c r="AA16" s="16"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="16"/>
+      <c r="E16" s="16"/>
+      <c r="F16" s="16"/>
+      <c r="G16" s="17"/>
+      <c r="H16" s="15">
+        <v>0</v>
+      </c>
+      <c r="I16" s="16"/>
+      <c r="J16" s="16"/>
+      <c r="K16" s="17"/>
+      <c r="L16" s="15">
+        <v>0</v>
+      </c>
+      <c r="M16" s="16"/>
+      <c r="N16" s="16"/>
+      <c r="O16" s="17"/>
+      <c r="P16" s="15">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="16"/>
+      <c r="R16" s="16"/>
+      <c r="S16" s="17"/>
+      <c r="T16" s="15">
+        <v>0</v>
+      </c>
+      <c r="U16" s="16"/>
+      <c r="V16" s="17"/>
+      <c r="W16" s="15">
+        <v>0</v>
+      </c>
+      <c r="X16" s="16"/>
+      <c r="Y16" s="17"/>
+      <c r="Z16" s="15"/>
+      <c r="AA16" s="17"/>
     </row>
     <row r="17" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="3">
@@ -1634,41 +1821,41 @@
       <c r="B17" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="14"/>
-      <c r="D17" s="15"/>
-      <c r="E17" s="15"/>
-      <c r="F17" s="15"/>
-      <c r="G17" s="16"/>
-      <c r="H17" s="14">
-        <v>0</v>
-      </c>
-      <c r="I17" s="15"/>
-      <c r="J17" s="15"/>
-      <c r="K17" s="16"/>
-      <c r="L17" s="14">
-        <v>0</v>
-      </c>
-      <c r="M17" s="15"/>
-      <c r="N17" s="15"/>
-      <c r="O17" s="16"/>
-      <c r="P17" s="14">
-        <v>0</v>
-      </c>
-      <c r="Q17" s="15"/>
-      <c r="R17" s="15"/>
-      <c r="S17" s="16"/>
-      <c r="T17" s="14">
-        <v>0</v>
-      </c>
-      <c r="U17" s="15"/>
-      <c r="V17" s="16"/>
-      <c r="W17" s="14">
-        <v>0</v>
-      </c>
-      <c r="X17" s="15"/>
-      <c r="Y17" s="16"/>
-      <c r="Z17" s="14"/>
-      <c r="AA17" s="16"/>
+      <c r="C17" s="15"/>
+      <c r="D17" s="16"/>
+      <c r="E17" s="16"/>
+      <c r="F17" s="16"/>
+      <c r="G17" s="17"/>
+      <c r="H17" s="15">
+        <v>0</v>
+      </c>
+      <c r="I17" s="16"/>
+      <c r="J17" s="16"/>
+      <c r="K17" s="17"/>
+      <c r="L17" s="15">
+        <v>0</v>
+      </c>
+      <c r="M17" s="16"/>
+      <c r="N17" s="16"/>
+      <c r="O17" s="17"/>
+      <c r="P17" s="15">
+        <v>0</v>
+      </c>
+      <c r="Q17" s="16"/>
+      <c r="R17" s="16"/>
+      <c r="S17" s="17"/>
+      <c r="T17" s="15">
+        <v>0</v>
+      </c>
+      <c r="U17" s="16"/>
+      <c r="V17" s="17"/>
+      <c r="W17" s="15">
+        <v>0</v>
+      </c>
+      <c r="X17" s="16"/>
+      <c r="Y17" s="17"/>
+      <c r="Z17" s="15"/>
+      <c r="AA17" s="17"/>
     </row>
     <row r="18" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="3">
@@ -1677,41 +1864,41 @@
       <c r="B18" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C18" s="14"/>
-      <c r="D18" s="15"/>
-      <c r="E18" s="15"/>
-      <c r="F18" s="15"/>
-      <c r="G18" s="16"/>
-      <c r="H18" s="14">
-        <v>0</v>
-      </c>
-      <c r="I18" s="15"/>
-      <c r="J18" s="15"/>
-      <c r="K18" s="16"/>
-      <c r="L18" s="14">
-        <v>0</v>
-      </c>
-      <c r="M18" s="15"/>
-      <c r="N18" s="15"/>
-      <c r="O18" s="16"/>
-      <c r="P18" s="14">
-        <v>0</v>
-      </c>
-      <c r="Q18" s="15"/>
-      <c r="R18" s="15"/>
-      <c r="S18" s="16"/>
-      <c r="T18" s="14">
-        <v>0</v>
-      </c>
-      <c r="U18" s="15"/>
-      <c r="V18" s="16"/>
-      <c r="W18" s="14">
-        <v>0</v>
-      </c>
-      <c r="X18" s="15"/>
-      <c r="Y18" s="16"/>
-      <c r="Z18" s="14"/>
-      <c r="AA18" s="16"/>
+      <c r="C18" s="15"/>
+      <c r="D18" s="16"/>
+      <c r="E18" s="16"/>
+      <c r="F18" s="16"/>
+      <c r="G18" s="17"/>
+      <c r="H18" s="15">
+        <v>0</v>
+      </c>
+      <c r="I18" s="16"/>
+      <c r="J18" s="16"/>
+      <c r="K18" s="17"/>
+      <c r="L18" s="15">
+        <v>0</v>
+      </c>
+      <c r="M18" s="16"/>
+      <c r="N18" s="16"/>
+      <c r="O18" s="17"/>
+      <c r="P18" s="15">
+        <v>0</v>
+      </c>
+      <c r="Q18" s="16"/>
+      <c r="R18" s="16"/>
+      <c r="S18" s="17"/>
+      <c r="T18" s="15">
+        <v>0</v>
+      </c>
+      <c r="U18" s="16"/>
+      <c r="V18" s="17"/>
+      <c r="W18" s="15">
+        <v>0</v>
+      </c>
+      <c r="X18" s="16"/>
+      <c r="Y18" s="17"/>
+      <c r="Z18" s="15"/>
+      <c r="AA18" s="17"/>
     </row>
     <row r="19" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="3">
@@ -1720,41 +1907,41 @@
       <c r="B19" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C19" s="14"/>
-      <c r="D19" s="15"/>
-      <c r="E19" s="15"/>
-      <c r="F19" s="15"/>
-      <c r="G19" s="16"/>
-      <c r="H19" s="14">
-        <v>0</v>
-      </c>
-      <c r="I19" s="15"/>
-      <c r="J19" s="15"/>
-      <c r="K19" s="16"/>
-      <c r="L19" s="14">
-        <v>0</v>
-      </c>
-      <c r="M19" s="15"/>
-      <c r="N19" s="15"/>
-      <c r="O19" s="16"/>
-      <c r="P19" s="14">
-        <v>0</v>
-      </c>
-      <c r="Q19" s="15"/>
-      <c r="R19" s="15"/>
-      <c r="S19" s="16"/>
-      <c r="T19" s="14">
-        <v>0</v>
-      </c>
-      <c r="U19" s="15"/>
-      <c r="V19" s="16"/>
-      <c r="W19" s="14">
-        <v>0</v>
-      </c>
-      <c r="X19" s="15"/>
-      <c r="Y19" s="16"/>
-      <c r="Z19" s="14"/>
-      <c r="AA19" s="16"/>
+      <c r="C19" s="15"/>
+      <c r="D19" s="16"/>
+      <c r="E19" s="16"/>
+      <c r="F19" s="16"/>
+      <c r="G19" s="17"/>
+      <c r="H19" s="15">
+        <v>0</v>
+      </c>
+      <c r="I19" s="16"/>
+      <c r="J19" s="16"/>
+      <c r="K19" s="17"/>
+      <c r="L19" s="15">
+        <v>0</v>
+      </c>
+      <c r="M19" s="16"/>
+      <c r="N19" s="16"/>
+      <c r="O19" s="17"/>
+      <c r="P19" s="15">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="16"/>
+      <c r="R19" s="16"/>
+      <c r="S19" s="17"/>
+      <c r="T19" s="15">
+        <v>0</v>
+      </c>
+      <c r="U19" s="16"/>
+      <c r="V19" s="17"/>
+      <c r="W19" s="15">
+        <v>0</v>
+      </c>
+      <c r="X19" s="16"/>
+      <c r="Y19" s="17"/>
+      <c r="Z19" s="15"/>
+      <c r="AA19" s="17"/>
     </row>
     <row r="20" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="3">
@@ -1763,41 +1950,41 @@
       <c r="B20" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C20" s="14"/>
-      <c r="D20" s="15"/>
-      <c r="E20" s="15"/>
-      <c r="F20" s="15"/>
-      <c r="G20" s="16"/>
-      <c r="H20" s="14">
-        <v>0</v>
-      </c>
-      <c r="I20" s="15"/>
-      <c r="J20" s="15"/>
-      <c r="K20" s="16"/>
-      <c r="L20" s="14">
-        <v>0</v>
-      </c>
-      <c r="M20" s="15"/>
-      <c r="N20" s="15"/>
-      <c r="O20" s="16"/>
-      <c r="P20" s="14">
-        <v>0</v>
-      </c>
-      <c r="Q20" s="15"/>
-      <c r="R20" s="15"/>
-      <c r="S20" s="16"/>
-      <c r="T20" s="14">
-        <v>0</v>
-      </c>
-      <c r="U20" s="15"/>
-      <c r="V20" s="16"/>
-      <c r="W20" s="14">
-        <v>0</v>
-      </c>
-      <c r="X20" s="15"/>
-      <c r="Y20" s="16"/>
-      <c r="Z20" s="14"/>
-      <c r="AA20" s="16"/>
+      <c r="C20" s="15"/>
+      <c r="D20" s="16"/>
+      <c r="E20" s="16"/>
+      <c r="F20" s="16"/>
+      <c r="G20" s="17"/>
+      <c r="H20" s="15">
+        <v>0</v>
+      </c>
+      <c r="I20" s="16"/>
+      <c r="J20" s="16"/>
+      <c r="K20" s="17"/>
+      <c r="L20" s="15">
+        <v>0</v>
+      </c>
+      <c r="M20" s="16"/>
+      <c r="N20" s="16"/>
+      <c r="O20" s="17"/>
+      <c r="P20" s="15">
+        <v>0</v>
+      </c>
+      <c r="Q20" s="16"/>
+      <c r="R20" s="16"/>
+      <c r="S20" s="17"/>
+      <c r="T20" s="15">
+        <v>0</v>
+      </c>
+      <c r="U20" s="16"/>
+      <c r="V20" s="17"/>
+      <c r="W20" s="15">
+        <v>0</v>
+      </c>
+      <c r="X20" s="16"/>
+      <c r="Y20" s="17"/>
+      <c r="Z20" s="15"/>
+      <c r="AA20" s="17"/>
     </row>
     <row r="21" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="3">
@@ -1806,41 +1993,41 @@
       <c r="B21" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C21" s="14"/>
-      <c r="D21" s="15"/>
-      <c r="E21" s="15"/>
-      <c r="F21" s="15"/>
-      <c r="G21" s="16"/>
-      <c r="H21" s="14">
-        <v>0</v>
-      </c>
-      <c r="I21" s="15"/>
-      <c r="J21" s="15"/>
-      <c r="K21" s="16"/>
-      <c r="L21" s="14">
-        <v>0</v>
-      </c>
-      <c r="M21" s="15"/>
-      <c r="N21" s="15"/>
-      <c r="O21" s="16"/>
-      <c r="P21" s="14">
-        <v>0</v>
-      </c>
-      <c r="Q21" s="15"/>
-      <c r="R21" s="15"/>
-      <c r="S21" s="16"/>
-      <c r="T21" s="14">
-        <v>0</v>
-      </c>
-      <c r="U21" s="15"/>
-      <c r="V21" s="16"/>
-      <c r="W21" s="14">
-        <v>0</v>
-      </c>
-      <c r="X21" s="15"/>
-      <c r="Y21" s="16"/>
-      <c r="Z21" s="14"/>
-      <c r="AA21" s="16"/>
+      <c r="C21" s="15"/>
+      <c r="D21" s="16"/>
+      <c r="E21" s="16"/>
+      <c r="F21" s="16"/>
+      <c r="G21" s="17"/>
+      <c r="H21" s="15">
+        <v>0</v>
+      </c>
+      <c r="I21" s="16"/>
+      <c r="J21" s="16"/>
+      <c r="K21" s="17"/>
+      <c r="L21" s="15">
+        <v>0</v>
+      </c>
+      <c r="M21" s="16"/>
+      <c r="N21" s="16"/>
+      <c r="O21" s="17"/>
+      <c r="P21" s="15">
+        <v>0</v>
+      </c>
+      <c r="Q21" s="16"/>
+      <c r="R21" s="16"/>
+      <c r="S21" s="17"/>
+      <c r="T21" s="15">
+        <v>0</v>
+      </c>
+      <c r="U21" s="16"/>
+      <c r="V21" s="17"/>
+      <c r="W21" s="15">
+        <v>0</v>
+      </c>
+      <c r="X21" s="16"/>
+      <c r="Y21" s="17"/>
+      <c r="Z21" s="15"/>
+      <c r="AA21" s="17"/>
     </row>
     <row r="22" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="3">
@@ -1849,41 +2036,41 @@
       <c r="B22" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C22" s="14"/>
-      <c r="D22" s="15"/>
-      <c r="E22" s="15"/>
-      <c r="F22" s="15"/>
-      <c r="G22" s="16"/>
-      <c r="H22" s="14">
-        <v>0</v>
-      </c>
-      <c r="I22" s="15"/>
-      <c r="J22" s="15"/>
-      <c r="K22" s="16"/>
-      <c r="L22" s="14">
-        <v>0</v>
-      </c>
-      <c r="M22" s="15"/>
-      <c r="N22" s="15"/>
-      <c r="O22" s="16"/>
-      <c r="P22" s="14">
-        <v>0</v>
-      </c>
-      <c r="Q22" s="15"/>
-      <c r="R22" s="15"/>
-      <c r="S22" s="16"/>
-      <c r="T22" s="14">
-        <v>0</v>
-      </c>
-      <c r="U22" s="15"/>
-      <c r="V22" s="16"/>
-      <c r="W22" s="14">
-        <v>0</v>
-      </c>
-      <c r="X22" s="15"/>
-      <c r="Y22" s="16"/>
-      <c r="Z22" s="14"/>
-      <c r="AA22" s="16"/>
+      <c r="C22" s="15"/>
+      <c r="D22" s="16"/>
+      <c r="E22" s="16"/>
+      <c r="F22" s="16"/>
+      <c r="G22" s="17"/>
+      <c r="H22" s="15">
+        <v>0</v>
+      </c>
+      <c r="I22" s="16"/>
+      <c r="J22" s="16"/>
+      <c r="K22" s="17"/>
+      <c r="L22" s="15">
+        <v>0</v>
+      </c>
+      <c r="M22" s="16"/>
+      <c r="N22" s="16"/>
+      <c r="O22" s="17"/>
+      <c r="P22" s="15">
+        <v>0</v>
+      </c>
+      <c r="Q22" s="16"/>
+      <c r="R22" s="16"/>
+      <c r="S22" s="17"/>
+      <c r="T22" s="15">
+        <v>0</v>
+      </c>
+      <c r="U22" s="16"/>
+      <c r="V22" s="17"/>
+      <c r="W22" s="15">
+        <v>0</v>
+      </c>
+      <c r="X22" s="16"/>
+      <c r="Y22" s="17"/>
+      <c r="Z22" s="15"/>
+      <c r="AA22" s="17"/>
     </row>
     <row r="23" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="3">
@@ -1892,41 +2079,41 @@
       <c r="B23" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C23" s="14"/>
-      <c r="D23" s="15"/>
-      <c r="E23" s="15"/>
-      <c r="F23" s="15"/>
-      <c r="G23" s="16"/>
-      <c r="H23" s="14">
-        <v>0</v>
-      </c>
-      <c r="I23" s="15"/>
-      <c r="J23" s="15"/>
-      <c r="K23" s="16"/>
-      <c r="L23" s="14">
-        <v>0</v>
-      </c>
-      <c r="M23" s="15"/>
-      <c r="N23" s="15"/>
-      <c r="O23" s="16"/>
-      <c r="P23" s="14">
-        <v>0</v>
-      </c>
-      <c r="Q23" s="15"/>
-      <c r="R23" s="15"/>
-      <c r="S23" s="16"/>
-      <c r="T23" s="14">
-        <v>0</v>
-      </c>
-      <c r="U23" s="15"/>
-      <c r="V23" s="16"/>
-      <c r="W23" s="14">
-        <v>0</v>
-      </c>
-      <c r="X23" s="15"/>
-      <c r="Y23" s="16"/>
-      <c r="Z23" s="14"/>
-      <c r="AA23" s="16"/>
+      <c r="C23" s="15"/>
+      <c r="D23" s="16"/>
+      <c r="E23" s="16"/>
+      <c r="F23" s="16"/>
+      <c r="G23" s="17"/>
+      <c r="H23" s="15">
+        <v>0</v>
+      </c>
+      <c r="I23" s="16"/>
+      <c r="J23" s="16"/>
+      <c r="K23" s="17"/>
+      <c r="L23" s="15">
+        <v>0</v>
+      </c>
+      <c r="M23" s="16"/>
+      <c r="N23" s="16"/>
+      <c r="O23" s="17"/>
+      <c r="P23" s="15">
+        <v>0</v>
+      </c>
+      <c r="Q23" s="16"/>
+      <c r="R23" s="16"/>
+      <c r="S23" s="17"/>
+      <c r="T23" s="15">
+        <v>0</v>
+      </c>
+      <c r="U23" s="16"/>
+      <c r="V23" s="17"/>
+      <c r="W23" s="15">
+        <v>0</v>
+      </c>
+      <c r="X23" s="16"/>
+      <c r="Y23" s="17"/>
+      <c r="Z23" s="15"/>
+      <c r="AA23" s="17"/>
     </row>
     <row r="24" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="3">
@@ -1935,41 +2122,41 @@
       <c r="B24" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C24" s="14"/>
-      <c r="D24" s="15"/>
-      <c r="E24" s="15"/>
-      <c r="F24" s="15"/>
-      <c r="G24" s="16"/>
-      <c r="H24" s="14">
-        <v>0</v>
-      </c>
-      <c r="I24" s="15"/>
-      <c r="J24" s="15"/>
-      <c r="K24" s="16"/>
-      <c r="L24" s="14">
-        <v>0</v>
-      </c>
-      <c r="M24" s="15"/>
-      <c r="N24" s="15"/>
-      <c r="O24" s="16"/>
-      <c r="P24" s="14">
-        <v>0</v>
-      </c>
-      <c r="Q24" s="15"/>
-      <c r="R24" s="15"/>
-      <c r="S24" s="16"/>
-      <c r="T24" s="14">
-        <v>0</v>
-      </c>
-      <c r="U24" s="15"/>
-      <c r="V24" s="16"/>
-      <c r="W24" s="14">
-        <v>0</v>
-      </c>
-      <c r="X24" s="15"/>
-      <c r="Y24" s="16"/>
-      <c r="Z24" s="14"/>
-      <c r="AA24" s="16"/>
+      <c r="C24" s="15"/>
+      <c r="D24" s="16"/>
+      <c r="E24" s="16"/>
+      <c r="F24" s="16"/>
+      <c r="G24" s="17"/>
+      <c r="H24" s="15">
+        <v>0</v>
+      </c>
+      <c r="I24" s="16"/>
+      <c r="J24" s="16"/>
+      <c r="K24" s="17"/>
+      <c r="L24" s="15">
+        <v>0</v>
+      </c>
+      <c r="M24" s="16"/>
+      <c r="N24" s="16"/>
+      <c r="O24" s="17"/>
+      <c r="P24" s="15">
+        <v>0</v>
+      </c>
+      <c r="Q24" s="16"/>
+      <c r="R24" s="16"/>
+      <c r="S24" s="17"/>
+      <c r="T24" s="15">
+        <v>0</v>
+      </c>
+      <c r="U24" s="16"/>
+      <c r="V24" s="17"/>
+      <c r="W24" s="15">
+        <v>0</v>
+      </c>
+      <c r="X24" s="16"/>
+      <c r="Y24" s="17"/>
+      <c r="Z24" s="15"/>
+      <c r="AA24" s="17"/>
     </row>
     <row r="25" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="3">
@@ -1978,72 +2165,72 @@
       <c r="B25" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C25" s="14"/>
-      <c r="D25" s="15"/>
-      <c r="E25" s="15"/>
-      <c r="F25" s="15"/>
-      <c r="G25" s="16"/>
-      <c r="H25" s="14">
-        <v>0</v>
-      </c>
-      <c r="I25" s="15"/>
-      <c r="J25" s="15"/>
-      <c r="K25" s="16"/>
-      <c r="L25" s="14">
-        <v>0</v>
-      </c>
-      <c r="M25" s="15"/>
-      <c r="N25" s="15"/>
-      <c r="O25" s="16"/>
-      <c r="P25" s="14">
-        <v>0</v>
-      </c>
-      <c r="Q25" s="15"/>
-      <c r="R25" s="15"/>
-      <c r="S25" s="16"/>
-      <c r="T25" s="14">
-        <v>0</v>
-      </c>
-      <c r="U25" s="15"/>
-      <c r="V25" s="16"/>
-      <c r="W25" s="14">
-        <v>0</v>
-      </c>
-      <c r="X25" s="15"/>
-      <c r="Y25" s="16"/>
-      <c r="Z25" s="14"/>
-      <c r="AA25" s="16"/>
+      <c r="C25" s="15"/>
+      <c r="D25" s="16"/>
+      <c r="E25" s="16"/>
+      <c r="F25" s="16"/>
+      <c r="G25" s="17"/>
+      <c r="H25" s="15">
+        <v>0</v>
+      </c>
+      <c r="I25" s="16"/>
+      <c r="J25" s="16"/>
+      <c r="K25" s="17"/>
+      <c r="L25" s="15">
+        <v>0</v>
+      </c>
+      <c r="M25" s="16"/>
+      <c r="N25" s="16"/>
+      <c r="O25" s="17"/>
+      <c r="P25" s="15">
+        <v>0</v>
+      </c>
+      <c r="Q25" s="16"/>
+      <c r="R25" s="16"/>
+      <c r="S25" s="17"/>
+      <c r="T25" s="15">
+        <v>0</v>
+      </c>
+      <c r="U25" s="16"/>
+      <c r="V25" s="17"/>
+      <c r="W25" s="15">
+        <v>0</v>
+      </c>
+      <c r="X25" s="16"/>
+      <c r="Y25" s="17"/>
+      <c r="Z25" s="15"/>
+      <c r="AA25" s="17"/>
     </row>
     <row r="26" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="20" t="s">
+      <c r="A26" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="B26" s="13"/>
-      <c r="C26" s="13"/>
-      <c r="D26" s="13"/>
-      <c r="E26" s="13"/>
-      <c r="F26" s="13"/>
-      <c r="G26" s="13"/>
-      <c r="H26" s="13"/>
-      <c r="I26" s="13"/>
-      <c r="J26" s="13"/>
-      <c r="K26" s="13"/>
-      <c r="L26" s="13"/>
-      <c r="M26" s="13"/>
-      <c r="N26" s="13"/>
-      <c r="O26" s="13"/>
-      <c r="P26" s="13"/>
-      <c r="Q26" s="13"/>
-      <c r="R26" s="13"/>
-      <c r="S26" s="13"/>
-      <c r="T26" s="13"/>
-      <c r="U26" s="13"/>
-      <c r="V26" s="13"/>
-      <c r="W26" s="13"/>
-      <c r="X26" s="13"/>
-      <c r="Y26" s="13"/>
-      <c r="Z26" s="13"/>
-      <c r="AA26" s="13"/>
+      <c r="B26" s="14"/>
+      <c r="C26" s="14"/>
+      <c r="D26" s="14"/>
+      <c r="E26" s="14"/>
+      <c r="F26" s="14"/>
+      <c r="G26" s="14"/>
+      <c r="H26" s="14"/>
+      <c r="I26" s="14"/>
+      <c r="J26" s="14"/>
+      <c r="K26" s="14"/>
+      <c r="L26" s="14"/>
+      <c r="M26" s="14"/>
+      <c r="N26" s="14"/>
+      <c r="O26" s="14"/>
+      <c r="P26" s="14"/>
+      <c r="Q26" s="14"/>
+      <c r="R26" s="14"/>
+      <c r="S26" s="14"/>
+      <c r="T26" s="14"/>
+      <c r="U26" s="14"/>
+      <c r="V26" s="14"/>
+      <c r="W26" s="14"/>
+      <c r="X26" s="14"/>
+      <c r="Y26" s="14"/>
+      <c r="Z26" s="14"/>
+      <c r="AA26" s="14"/>
     </row>
     <row r="27" spans="1:27" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="6" t="s">
@@ -2747,329 +2934,212 @@
       <c r="F44" s="9"/>
       <c r="G44" s="9"/>
     </row>
-    <row r="45" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A45" s="23" t="s">
-        <v>84</v>
-      </c>
-      <c r="B45" s="23"/>
-      <c r="C45" s="23"/>
-      <c r="D45" s="23"/>
-      <c r="E45" s="23"/>
-      <c r="F45" s="23"/>
-      <c r="G45" s="23"/>
-      <c r="H45" s="11"/>
-      <c r="I45" s="10" t="s">
+    <row r="45" spans="1:27" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A45" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="B45" s="11"/>
+      <c r="C45" s="11"/>
+      <c r="D45" s="11"/>
+      <c r="E45" s="11"/>
+      <c r="F45" s="11"/>
+      <c r="G45" s="11"/>
+      <c r="H45" s="10"/>
+      <c r="I45" s="30" t="s">
+        <v>89</v>
+      </c>
+      <c r="J45" s="19"/>
+      <c r="K45" s="19"/>
+      <c r="L45" s="19"/>
+      <c r="M45" s="19"/>
+      <c r="N45" s="19"/>
+      <c r="O45" s="19"/>
+      <c r="P45" s="19"/>
+      <c r="Q45" s="19"/>
+      <c r="S45" s="30" t="s">
+        <v>90</v>
+      </c>
+      <c r="T45" s="14"/>
+      <c r="U45" s="14"/>
+      <c r="V45" s="14"/>
+      <c r="W45" s="14"/>
+      <c r="X45" s="14"/>
+      <c r="Y45" s="14"/>
+      <c r="Z45" s="14"/>
+      <c r="AA45" s="14"/>
+    </row>
+    <row r="46" spans="1:27" ht="54" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A46" s="28" t="s">
+        <v>91</v>
+      </c>
+      <c r="B46" s="29"/>
+      <c r="C46" s="29"/>
+      <c r="D46" s="29"/>
+      <c r="E46" s="29"/>
+      <c r="F46" s="29"/>
+      <c r="G46" s="29"/>
+      <c r="I46" s="18">
+        <v>1</v>
+      </c>
+      <c r="J46" s="18"/>
+      <c r="K46" s="18"/>
+      <c r="L46" s="18"/>
+      <c r="M46" s="18"/>
+      <c r="N46" s="18"/>
+      <c r="O46" s="18"/>
+      <c r="P46" s="18"/>
+      <c r="Q46" s="18"/>
+      <c r="S46" s="18">
+        <v>1</v>
+      </c>
+      <c r="T46" s="14"/>
+      <c r="U46" s="14"/>
+      <c r="V46" s="14"/>
+      <c r="W46" s="14"/>
+      <c r="X46" s="14"/>
+      <c r="Y46" s="14"/>
+      <c r="Z46" s="14"/>
+      <c r="AA46" s="14"/>
+    </row>
+    <row r="47" spans="1:27" ht="54" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A47" s="29" t="s">
+        <v>92</v>
+      </c>
+      <c r="B47" s="29"/>
+      <c r="C47" s="29"/>
+      <c r="D47" s="29"/>
+      <c r="E47" s="29"/>
+      <c r="F47" s="29"/>
+      <c r="G47" s="29"/>
+      <c r="I47" s="18" t="s">
         <v>79</v>
       </c>
-      <c r="J45" s="10"/>
-      <c r="K45" s="10"/>
-      <c r="L45" s="10"/>
-      <c r="M45" s="10"/>
-      <c r="N45" s="10"/>
-      <c r="O45" s="10"/>
-      <c r="P45" s="10"/>
-      <c r="Q45" s="10"/>
-      <c r="S45" s="23" t="s">
+      <c r="J47" s="18"/>
+      <c r="K47" s="18"/>
+      <c r="L47" s="18"/>
+      <c r="M47" s="18"/>
+      <c r="N47" s="18"/>
+      <c r="O47" s="18"/>
+      <c r="P47" s="18"/>
+      <c r="Q47" s="18"/>
+      <c r="S47" s="18" t="s">
+        <v>79</v>
+      </c>
+      <c r="T47" s="14"/>
+      <c r="U47" s="14"/>
+      <c r="V47" s="14"/>
+      <c r="W47" s="14"/>
+      <c r="X47" s="14"/>
+      <c r="Y47" s="14"/>
+      <c r="Z47" s="14"/>
+      <c r="AA47" s="14"/>
+    </row>
+    <row r="48" spans="1:27" ht="54" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A48" s="29" t="s">
+        <v>93</v>
+      </c>
+      <c r="B48" s="12"/>
+      <c r="C48" s="12"/>
+      <c r="D48" s="12"/>
+      <c r="E48" s="12"/>
+      <c r="F48" s="12"/>
+      <c r="G48" s="12"/>
+      <c r="I48" s="18" t="s">
         <v>80</v>
       </c>
-      <c r="T45" s="13"/>
-      <c r="U45" s="13"/>
-      <c r="V45" s="13"/>
-      <c r="W45" s="13"/>
-      <c r="X45" s="13"/>
-      <c r="Y45" s="13"/>
-      <c r="Z45" s="13"/>
-      <c r="AA45" s="13"/>
-    </row>
-    <row r="46" spans="1:27" ht="54" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A46" s="20">
-        <v>1</v>
-      </c>
-      <c r="B46" s="20"/>
-      <c r="C46" s="20"/>
-      <c r="D46" s="20"/>
-      <c r="E46" s="20"/>
-      <c r="F46" s="20"/>
-      <c r="G46" s="20"/>
-      <c r="I46" s="12">
-        <v>1</v>
-      </c>
-      <c r="J46" s="12"/>
-      <c r="K46" s="12"/>
-      <c r="L46" s="12"/>
-      <c r="M46" s="12"/>
-      <c r="N46" s="12"/>
-      <c r="O46" s="12"/>
-      <c r="P46" s="12"/>
-      <c r="Q46" s="12"/>
-      <c r="S46" s="12">
-        <v>1</v>
-      </c>
-      <c r="T46" s="13"/>
-      <c r="U46" s="13"/>
-      <c r="V46" s="13"/>
-      <c r="W46" s="13"/>
-      <c r="X46" s="13"/>
-      <c r="Y46" s="13"/>
-      <c r="Z46" s="13"/>
-      <c r="AA46" s="13"/>
-    </row>
-    <row r="47" spans="1:27" ht="54" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A47" s="20">
-        <v>2</v>
-      </c>
-      <c r="B47" s="20"/>
-      <c r="C47" s="20"/>
-      <c r="D47" s="20"/>
-      <c r="E47" s="20"/>
-      <c r="F47" s="20"/>
-      <c r="G47" s="20"/>
-      <c r="I47" s="12" t="s">
+      <c r="J48" s="18"/>
+      <c r="K48" s="18"/>
+      <c r="L48" s="18"/>
+      <c r="M48" s="18"/>
+      <c r="N48" s="18"/>
+      <c r="O48" s="18"/>
+      <c r="P48" s="18"/>
+      <c r="Q48" s="18"/>
+      <c r="S48" s="18" t="s">
+        <v>80</v>
+      </c>
+      <c r="T48" s="14"/>
+      <c r="U48" s="14"/>
+      <c r="V48" s="14"/>
+      <c r="W48" s="14"/>
+      <c r="X48" s="14"/>
+      <c r="Y48" s="14"/>
+      <c r="Z48" s="14"/>
+      <c r="AA48" s="14"/>
+    </row>
+    <row r="49" spans="1:27" ht="50" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A49" s="29" t="s">
+        <v>88</v>
+      </c>
+      <c r="B49" s="12"/>
+      <c r="C49" s="12"/>
+      <c r="D49" s="12"/>
+      <c r="E49" s="12"/>
+      <c r="F49" s="12"/>
+      <c r="G49" s="12"/>
+      <c r="I49" s="18" t="s">
         <v>81</v>
       </c>
-      <c r="J47" s="12"/>
-      <c r="K47" s="12"/>
-      <c r="L47" s="12"/>
-      <c r="M47" s="12"/>
-      <c r="N47" s="12"/>
-      <c r="O47" s="12"/>
-      <c r="P47" s="12"/>
-      <c r="Q47" s="12"/>
-      <c r="S47" s="12" t="s">
+      <c r="J49" s="18"/>
+      <c r="K49" s="18"/>
+      <c r="L49" s="18"/>
+      <c r="M49" s="18"/>
+      <c r="N49" s="18"/>
+      <c r="O49" s="18"/>
+      <c r="P49" s="18"/>
+      <c r="Q49" s="18"/>
+      <c r="S49" s="18" t="s">
         <v>81</v>
       </c>
-      <c r="T47" s="13"/>
-      <c r="U47" s="13"/>
-      <c r="V47" s="13"/>
-      <c r="W47" s="13"/>
-      <c r="X47" s="13"/>
-      <c r="Y47" s="13"/>
-      <c r="Z47" s="13"/>
-      <c r="AA47" s="13"/>
-    </row>
-    <row r="48" spans="1:27" ht="54" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A48" s="20">
-        <v>3</v>
-      </c>
-      <c r="B48" s="20"/>
-      <c r="C48" s="20"/>
-      <c r="D48" s="20"/>
-      <c r="E48" s="20"/>
-      <c r="F48" s="20"/>
-      <c r="G48" s="20"/>
-      <c r="I48" s="12" t="s">
-        <v>82</v>
-      </c>
-      <c r="J48" s="12"/>
-      <c r="K48" s="12"/>
-      <c r="L48" s="12"/>
-      <c r="M48" s="12"/>
-      <c r="N48" s="12"/>
-      <c r="O48" s="12"/>
-      <c r="P48" s="12"/>
-      <c r="Q48" s="12"/>
-      <c r="S48" s="12" t="s">
-        <v>82</v>
-      </c>
-      <c r="T48" s="13"/>
-      <c r="U48" s="13"/>
-      <c r="V48" s="13"/>
-      <c r="W48" s="13"/>
-      <c r="X48" s="13"/>
-      <c r="Y48" s="13"/>
-      <c r="Z48" s="13"/>
-      <c r="AA48" s="13"/>
-    </row>
-    <row r="49" spans="1:27" ht="50" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A49" s="20">
-        <v>4</v>
-      </c>
-      <c r="B49" s="20"/>
-      <c r="C49" s="20"/>
-      <c r="D49" s="20"/>
-      <c r="E49" s="20"/>
-      <c r="F49" s="20"/>
-      <c r="G49" s="20"/>
-      <c r="I49" s="12" t="s">
-        <v>83</v>
-      </c>
-      <c r="J49" s="12"/>
-      <c r="K49" s="12"/>
-      <c r="L49" s="12"/>
-      <c r="M49" s="12"/>
-      <c r="N49" s="12"/>
-      <c r="O49" s="12"/>
-      <c r="P49" s="12"/>
-      <c r="Q49" s="12"/>
-      <c r="S49" s="12" t="s">
-        <v>83</v>
-      </c>
-      <c r="T49" s="13"/>
-      <c r="U49" s="13"/>
-      <c r="V49" s="13"/>
-      <c r="W49" s="13"/>
-      <c r="X49" s="13"/>
-      <c r="Y49" s="13"/>
-      <c r="Z49" s="13"/>
-      <c r="AA49" s="13"/>
+      <c r="T49" s="14"/>
+      <c r="U49" s="14"/>
+      <c r="V49" s="14"/>
+      <c r="W49" s="14"/>
+      <c r="X49" s="14"/>
+      <c r="Y49" s="14"/>
+      <c r="Z49" s="14"/>
+      <c r="AA49" s="14"/>
     </row>
     <row r="50" spans="1:27" ht="25" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="51" spans="1:27" ht="49.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A51" s="28" t="s">
-        <v>90</v>
-      </c>
-      <c r="B51" s="29"/>
-      <c r="C51" s="29"/>
-      <c r="D51" s="29"/>
-      <c r="E51" s="29"/>
-      <c r="F51" s="29"/>
-      <c r="G51" s="29"/>
-    </row>
-    <row r="52" spans="1:27" ht="62.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A52" s="30" t="s">
-        <v>91</v>
-      </c>
-      <c r="B52" s="20"/>
-      <c r="C52" s="20"/>
-      <c r="D52" s="20"/>
-      <c r="E52" s="20"/>
-      <c r="F52" s="20"/>
-      <c r="G52" s="20"/>
-    </row>
-    <row r="53" spans="1:27" ht="53.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A53" s="30" t="s">
-        <v>92</v>
-      </c>
-      <c r="B53" s="20"/>
-      <c r="C53" s="20"/>
-      <c r="D53" s="20"/>
-      <c r="E53" s="20"/>
-      <c r="F53" s="20"/>
-      <c r="G53" s="20"/>
-    </row>
-    <row r="54" spans="1:27" ht="53.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A54" s="30" t="s">
-        <v>93</v>
-      </c>
-      <c r="B54" s="20"/>
-      <c r="C54" s="20"/>
-      <c r="D54" s="20"/>
-      <c r="E54" s="20"/>
-      <c r="F54" s="20"/>
-      <c r="G54" s="20"/>
-    </row>
-    <row r="55" spans="1:27" ht="53.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A55" s="30" t="s">
-        <v>94</v>
-      </c>
-      <c r="B55" s="20"/>
-      <c r="C55" s="20"/>
-      <c r="D55" s="20"/>
-      <c r="E55" s="20"/>
-      <c r="F55" s="20"/>
-      <c r="G55" s="20"/>
-    </row>
   </sheetData>
-  <mergeCells count="167">
-    <mergeCell ref="A51:G51"/>
-    <mergeCell ref="A52:G52"/>
-    <mergeCell ref="A53:G53"/>
-    <mergeCell ref="A54:G54"/>
-    <mergeCell ref="A55:G55"/>
-    <mergeCell ref="A3:AA3"/>
-    <mergeCell ref="P14:S14"/>
-    <mergeCell ref="H20:K20"/>
-    <mergeCell ref="I48:Q48"/>
-    <mergeCell ref="S45:AA45"/>
-    <mergeCell ref="W17:Y17"/>
-    <mergeCell ref="A5:AA5"/>
-    <mergeCell ref="W11:Y11"/>
-    <mergeCell ref="L13:O13"/>
-    <mergeCell ref="W19:Y19"/>
-    <mergeCell ref="H6:K6"/>
-    <mergeCell ref="P21:S21"/>
-    <mergeCell ref="H21:K21"/>
-    <mergeCell ref="P8:S8"/>
-    <mergeCell ref="C8:G8"/>
-    <mergeCell ref="L15:O15"/>
-    <mergeCell ref="T15:V15"/>
-    <mergeCell ref="C17:G17"/>
-    <mergeCell ref="T24:V24"/>
-    <mergeCell ref="W25:Y25"/>
-    <mergeCell ref="L23:O23"/>
-    <mergeCell ref="P23:S23"/>
-    <mergeCell ref="Z10:AA10"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="W6:Y6"/>
-    <mergeCell ref="L8:O8"/>
-    <mergeCell ref="Z20:AA20"/>
-    <mergeCell ref="W15:Y15"/>
-    <mergeCell ref="I49:Q49"/>
-    <mergeCell ref="P17:S17"/>
-    <mergeCell ref="H16:K16"/>
-    <mergeCell ref="L10:O10"/>
-    <mergeCell ref="C13:G13"/>
-    <mergeCell ref="L25:O25"/>
-    <mergeCell ref="T25:V25"/>
-    <mergeCell ref="H22:K22"/>
-    <mergeCell ref="P19:S19"/>
-    <mergeCell ref="Z6:AA6"/>
-    <mergeCell ref="L9:O9"/>
-    <mergeCell ref="C6:G6"/>
-    <mergeCell ref="T9:V9"/>
-    <mergeCell ref="C15:G15"/>
-    <mergeCell ref="P12:S12"/>
-    <mergeCell ref="C16:G16"/>
-    <mergeCell ref="T23:V23"/>
-    <mergeCell ref="C25:G25"/>
-    <mergeCell ref="A49:G49"/>
-    <mergeCell ref="L7:O7"/>
-    <mergeCell ref="T7:V7"/>
-    <mergeCell ref="C9:G9"/>
-    <mergeCell ref="T16:V16"/>
-    <mergeCell ref="C11:G11"/>
-    <mergeCell ref="T18:V18"/>
-    <mergeCell ref="L24:O24"/>
-    <mergeCell ref="L18:O18"/>
-    <mergeCell ref="L11:O11"/>
-    <mergeCell ref="T11:V11"/>
-    <mergeCell ref="C19:G19"/>
-    <mergeCell ref="P7:S7"/>
-    <mergeCell ref="H7:K7"/>
-    <mergeCell ref="P16:S16"/>
-    <mergeCell ref="T10:V10"/>
-    <mergeCell ref="W4:AA4"/>
-    <mergeCell ref="H19:K19"/>
-    <mergeCell ref="I47:Q47"/>
-    <mergeCell ref="L22:O22"/>
-    <mergeCell ref="P13:S13"/>
-    <mergeCell ref="C24:G24"/>
-    <mergeCell ref="H12:K12"/>
-    <mergeCell ref="L6:O6"/>
-    <mergeCell ref="T12:V12"/>
-    <mergeCell ref="T21:V21"/>
-    <mergeCell ref="P15:S15"/>
-    <mergeCell ref="H14:K14"/>
-    <mergeCell ref="Z7:AA7"/>
-    <mergeCell ref="Z16:AA16"/>
-    <mergeCell ref="C10:G10"/>
-    <mergeCell ref="Z18:AA18"/>
-    <mergeCell ref="Z8:AA8"/>
-    <mergeCell ref="W14:Y14"/>
-    <mergeCell ref="Z17:AA17"/>
-    <mergeCell ref="W23:Y23"/>
-    <mergeCell ref="W13:Y13"/>
-    <mergeCell ref="Z9:AA9"/>
-    <mergeCell ref="A46:G46"/>
-    <mergeCell ref="T13:V13"/>
-    <mergeCell ref="A47:G47"/>
-    <mergeCell ref="Z14:AA14"/>
-    <mergeCell ref="P11:S11"/>
-    <mergeCell ref="W10:Y10"/>
-    <mergeCell ref="W24:Y24"/>
-    <mergeCell ref="H17:K17"/>
-    <mergeCell ref="H11:K11"/>
-    <mergeCell ref="L20:O20"/>
+  <mergeCells count="163">
+    <mergeCell ref="S49:AA49"/>
+    <mergeCell ref="W16:Y16"/>
+    <mergeCell ref="I46:Q46"/>
+    <mergeCell ref="S46:AA46"/>
+    <mergeCell ref="Z15:AA15"/>
+    <mergeCell ref="Z24:AA24"/>
+    <mergeCell ref="P10:S10"/>
+    <mergeCell ref="H10:K10"/>
+    <mergeCell ref="P25:S25"/>
+    <mergeCell ref="Z12:AA12"/>
+    <mergeCell ref="T19:V19"/>
+    <mergeCell ref="H25:K25"/>
+    <mergeCell ref="I45:Q45"/>
+    <mergeCell ref="C4:G4"/>
+    <mergeCell ref="A2:AA2"/>
+    <mergeCell ref="T22:V22"/>
+    <mergeCell ref="W18:Y18"/>
+    <mergeCell ref="P20:S20"/>
+    <mergeCell ref="W8:Y8"/>
+    <mergeCell ref="T6:V6"/>
+    <mergeCell ref="Z21:AA21"/>
+    <mergeCell ref="L19:O19"/>
+    <mergeCell ref="C21:G21"/>
+    <mergeCell ref="H9:K9"/>
+    <mergeCell ref="P22:S22"/>
+    <mergeCell ref="L12:O12"/>
+    <mergeCell ref="P6:S6"/>
+    <mergeCell ref="Z13:AA13"/>
+    <mergeCell ref="T20:V20"/>
+    <mergeCell ref="C7:G7"/>
+    <mergeCell ref="L14:O14"/>
+    <mergeCell ref="T14:V14"/>
+    <mergeCell ref="P18:S18"/>
+    <mergeCell ref="Z11:AA11"/>
+    <mergeCell ref="C14:G14"/>
+    <mergeCell ref="W7:Y7"/>
+    <mergeCell ref="C12:G12"/>
     <mergeCell ref="A48:G48"/>
     <mergeCell ref="L17:O17"/>
     <mergeCell ref="Z23:AA23"/>
@@ -3094,6 +3164,22 @@
     <mergeCell ref="A26:AA26"/>
     <mergeCell ref="Z25:AA25"/>
     <mergeCell ref="C20:G20"/>
+    <mergeCell ref="Z8:AA8"/>
+    <mergeCell ref="W14:Y14"/>
+    <mergeCell ref="Z17:AA17"/>
+    <mergeCell ref="W23:Y23"/>
+    <mergeCell ref="W13:Y13"/>
+    <mergeCell ref="Z9:AA9"/>
+    <mergeCell ref="A46:G46"/>
+    <mergeCell ref="T13:V13"/>
+    <mergeCell ref="A47:G47"/>
+    <mergeCell ref="Z14:AA14"/>
+    <mergeCell ref="P11:S11"/>
+    <mergeCell ref="W10:Y10"/>
+    <mergeCell ref="W24:Y24"/>
+    <mergeCell ref="H17:K17"/>
+    <mergeCell ref="H11:K11"/>
+    <mergeCell ref="L20:O20"/>
     <mergeCell ref="H8:K8"/>
     <mergeCell ref="W9:Y9"/>
     <mergeCell ref="T8:V8"/>
@@ -3101,47 +3187,88 @@
     <mergeCell ref="L16:O16"/>
     <mergeCell ref="Z22:AA22"/>
     <mergeCell ref="C22:G22"/>
-    <mergeCell ref="C4:G4"/>
-    <mergeCell ref="A2:AA2"/>
-    <mergeCell ref="T22:V22"/>
-    <mergeCell ref="W18:Y18"/>
-    <mergeCell ref="P20:S20"/>
-    <mergeCell ref="W8:Y8"/>
-    <mergeCell ref="T6:V6"/>
-    <mergeCell ref="Z21:AA21"/>
-    <mergeCell ref="L19:O19"/>
-    <mergeCell ref="C21:G21"/>
-    <mergeCell ref="H9:K9"/>
-    <mergeCell ref="P22:S22"/>
-    <mergeCell ref="L12:O12"/>
-    <mergeCell ref="P6:S6"/>
-    <mergeCell ref="Z13:AA13"/>
-    <mergeCell ref="T20:V20"/>
-    <mergeCell ref="C7:G7"/>
-    <mergeCell ref="L14:O14"/>
-    <mergeCell ref="T14:V14"/>
-    <mergeCell ref="P18:S18"/>
-    <mergeCell ref="Z11:AA11"/>
-    <mergeCell ref="C14:G14"/>
-    <mergeCell ref="W7:Y7"/>
-    <mergeCell ref="C12:G12"/>
     <mergeCell ref="P9:S9"/>
-    <mergeCell ref="S49:AA49"/>
-    <mergeCell ref="W16:Y16"/>
-    <mergeCell ref="I46:Q46"/>
-    <mergeCell ref="S46:AA46"/>
-    <mergeCell ref="Z15:AA15"/>
-    <mergeCell ref="Z24:AA24"/>
-    <mergeCell ref="P10:S10"/>
-    <mergeCell ref="H10:K10"/>
-    <mergeCell ref="P25:S25"/>
-    <mergeCell ref="Z12:AA12"/>
-    <mergeCell ref="T19:V19"/>
-    <mergeCell ref="H25:K25"/>
+    <mergeCell ref="I47:Q47"/>
+    <mergeCell ref="L22:O22"/>
+    <mergeCell ref="P13:S13"/>
+    <mergeCell ref="C24:G24"/>
+    <mergeCell ref="H12:K12"/>
+    <mergeCell ref="L6:O6"/>
+    <mergeCell ref="T12:V12"/>
+    <mergeCell ref="T21:V21"/>
+    <mergeCell ref="P15:S15"/>
+    <mergeCell ref="H14:K14"/>
+    <mergeCell ref="C10:G10"/>
+    <mergeCell ref="I49:Q49"/>
+    <mergeCell ref="P17:S17"/>
+    <mergeCell ref="H16:K16"/>
+    <mergeCell ref="L10:O10"/>
+    <mergeCell ref="C13:G13"/>
+    <mergeCell ref="L25:O25"/>
+    <mergeCell ref="T25:V25"/>
+    <mergeCell ref="H22:K22"/>
+    <mergeCell ref="P19:S19"/>
+    <mergeCell ref="C15:G15"/>
+    <mergeCell ref="P12:S12"/>
+    <mergeCell ref="C16:G16"/>
+    <mergeCell ref="T23:V23"/>
+    <mergeCell ref="C25:G25"/>
+    <mergeCell ref="A49:G49"/>
+    <mergeCell ref="T16:V16"/>
+    <mergeCell ref="C11:G11"/>
+    <mergeCell ref="T18:V18"/>
+    <mergeCell ref="L24:O24"/>
+    <mergeCell ref="L18:O18"/>
+    <mergeCell ref="L11:O11"/>
+    <mergeCell ref="T11:V11"/>
+    <mergeCell ref="C19:G19"/>
+    <mergeCell ref="P16:S16"/>
+    <mergeCell ref="W25:Y25"/>
+    <mergeCell ref="L23:O23"/>
+    <mergeCell ref="P23:S23"/>
+    <mergeCell ref="Z10:AA10"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="W6:Y6"/>
+    <mergeCell ref="L8:O8"/>
+    <mergeCell ref="Z20:AA20"/>
+    <mergeCell ref="W15:Y15"/>
+    <mergeCell ref="Z6:AA6"/>
+    <mergeCell ref="L9:O9"/>
+    <mergeCell ref="C6:G6"/>
+    <mergeCell ref="T9:V9"/>
+    <mergeCell ref="L7:O7"/>
+    <mergeCell ref="T7:V7"/>
+    <mergeCell ref="C9:G9"/>
+    <mergeCell ref="P7:S7"/>
+    <mergeCell ref="H7:K7"/>
+    <mergeCell ref="T10:V10"/>
+    <mergeCell ref="W4:AA4"/>
+    <mergeCell ref="H19:K19"/>
+    <mergeCell ref="Z7:AA7"/>
+    <mergeCell ref="Z16:AA16"/>
+    <mergeCell ref="Z18:AA18"/>
+    <mergeCell ref="A3:AA3"/>
+    <mergeCell ref="P14:S14"/>
+    <mergeCell ref="H20:K20"/>
+    <mergeCell ref="I48:Q48"/>
+    <mergeCell ref="S45:AA45"/>
+    <mergeCell ref="W17:Y17"/>
+    <mergeCell ref="A5:AA5"/>
+    <mergeCell ref="W11:Y11"/>
+    <mergeCell ref="L13:O13"/>
+    <mergeCell ref="W19:Y19"/>
+    <mergeCell ref="H6:K6"/>
+    <mergeCell ref="P21:S21"/>
+    <mergeCell ref="H21:K21"/>
+    <mergeCell ref="P8:S8"/>
+    <mergeCell ref="C8:G8"/>
+    <mergeCell ref="L15:O15"/>
+    <mergeCell ref="T15:V15"/>
+    <mergeCell ref="C17:G17"/>
+    <mergeCell ref="T24:V24"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" r:id="rId1"/>
   <drawing r:id="rId2"/>
-  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>